<commit_message>
add Entrenamientos en Inicio
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,9 +16,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
-    <t>fecha</t>
+    <t>date</t>
   </si>
   <si>
     <t>video</t>
@@ -30,27 +30,46 @@
     <t>https://youtu.be/ivunOFSM1ME</t>
   </si>
   <si>
-    <t>Trabajo principal 11 vs 11. Ataque, Defensa y Transiciones</t>
+    <t>Trabajo principal</t>
   </si>
   <si>
     <t>https://youtu.be/n5sBx_cosTY</t>
   </si>
   <si>
-    <t>Parte1: 8 vs 8 con 4 porterías &amp; Reducido con 4 comodines por fuera</t>
+    <t>Parte 1 Trabajo previo</t>
   </si>
   <si>
     <t>https://youtu.be/X55mwKhQgTI</t>
   </si>
   <si>
-    <t>Parte2; 8 vs 8 con 4 porterías &amp; Reducido con 4 comodines por fuera</t>
+    <t>Parte 2 Trabajo previo</t>
+  </si>
+  <si>
+    <t>https://youtu.be/_kizq4KY_jk</t>
+  </si>
+  <si>
+    <t>Juego de posesión</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xmtyeaOQRJY</t>
+  </si>
+  <si>
+    <t>Juego de posesión con variante</t>
+  </si>
+  <si>
+    <t>https://youtu.be/G6DleZgwdZc</t>
+  </si>
+  <si>
+    <t>Trabajo principal 11vs11</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
+    <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -104,14 +123,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -125,6 +144,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -342,7 +364,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="10.71"/>
     <col customWidth="1" min="2" max="2" width="29.71"/>
-    <col customWidth="1" min="3" max="3" width="59.29"/>
+    <col customWidth="1" min="3" max="3" width="29.29"/>
     <col customWidth="1" min="4" max="14" width="9.14"/>
   </cols>
   <sheetData>
@@ -350,10 +372,10 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -388,6 +410,39 @@
       </c>
       <c r="C4" s="7" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8">
+        <v>46093.0</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8">
+        <v>46093.0</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8">
+        <v>46093.0</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1"/>
@@ -1375,10 +1430,13 @@
     <hyperlink r:id="rId1" ref="B2"/>
     <hyperlink r:id="rId2" ref="B3"/>
     <hyperlink r:id="rId3" ref="B4"/>
+    <hyperlink r:id="rId4" ref="B5"/>
+    <hyperlink r:id="rId5" ref="B6"/>
+    <hyperlink r:id="rId6" ref="B7"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add 1 entrenamiento faltante 12/03
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="bddpj7SCcX/rHN2Iof3YYfLNZUWQHW6ectyxn+51mGg="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="lbdTynPsi5GwOpD1EUfWOz1DWvJKGY5AnoxFKV7uzic="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>date</t>
   </si>
@@ -45,6 +45,24 @@
     <t>Parte 2 Activación</t>
   </si>
   <si>
+    <t>https://youtu.be/KkCJE1znlL4</t>
+  </si>
+  <si>
+    <t>Transición defensa-ataque</t>
+  </si>
+  <si>
+    <t>https://youtu.be/pN42QiGJiAQ</t>
+  </si>
+  <si>
+    <t>Secuencia de pases</t>
+  </si>
+  <si>
+    <t>https://youtu.be/WWsgIcZPxpg</t>
+  </si>
+  <si>
+    <t>Reducido</t>
+  </si>
+  <si>
     <t>https://youtu.be/_kizq4KY_jk</t>
   </si>
   <si>
@@ -61,18 +79,6 @@
   </si>
   <si>
     <t>Trabajo principal 11vs11</t>
-  </si>
-  <si>
-    <t>https://youtu.be/KkCJE1znlL4</t>
-  </si>
-  <si>
-    <t>Transición defensa-ataque</t>
-  </si>
-  <si>
-    <t>https://youtu.be/pN42QiGJiAQ</t>
-  </si>
-  <si>
-    <t>Secuencia de pases</t>
   </si>
   <si>
     <t>https://youtu.be/sZKL7Xz15aM</t>
@@ -438,7 +444,7 @@
     </row>
     <row r="5">
       <c r="A5" s="8">
-        <v>46093.0</v>
+        <v>46092.0</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>9</v>
@@ -449,7 +455,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8">
-        <v>46093.0</v>
+        <v>46092.0</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>11</v>
@@ -465,13 +471,13 @@
       <c r="B7" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="7" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8">
-        <v>46092.0</v>
+        <v>46093.0</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>15</v>
@@ -482,7 +488,7 @@
     </row>
     <row r="9">
       <c r="A9" s="8">
-        <v>46092.0</v>
+        <v>46093.0</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>17</v>
@@ -493,12 +499,12 @@
     </row>
     <row r="10">
       <c r="A10" s="8">
-        <v>46094.0</v>
+        <v>46093.0</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="5" t="s">
         <v>20</v>
       </c>
     </row>
@@ -513,7 +519,17 @@
         <v>22</v>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1"/>
+    <row r="12">
+      <c r="A12" s="8">
+        <v>46094.0</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>24</v>
+      </c>
+    </row>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
     <row r="20" ht="15.75" customHeight="1"/>
@@ -1493,6 +1509,7 @@
     <row r="994" ht="15.75" customHeight="1"/>
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="B2"/>
@@ -1505,10 +1522,11 @@
     <hyperlink r:id="rId8" ref="B9"/>
     <hyperlink r:id="rId9" ref="B10"/>
     <hyperlink r:id="rId10" ref="B11"/>
+    <hyperlink r:id="rId11" ref="B12"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId11"/>
+  <drawing r:id="rId12"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
comentarioa entrenamientos  - update excel
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,42 +9,54 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="lbdTynPsi5GwOpD1EUfWOz1DWvJKGY5AnoxFKV7uzic="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Zd2bzr3F57PIdj0Z1LFheCHbwMhROcEBkIiM90EgRzo="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>date</t>
   </si>
   <si>
+    <t>parte_entreno</t>
+  </si>
+  <si>
     <t>video</t>
   </si>
   <si>
     <t>Nombre</t>
   </si>
   <si>
+    <t>comentarios</t>
+  </si>
+  <si>
+    <t>activación</t>
+  </si>
+  <si>
+    <t>https://youtu.be/n5sBx_cosTY</t>
+  </si>
+  <si>
+    <t>Parte 1 Activación</t>
+  </si>
+  <si>
+    <t>https://youtu.be/X55mwKhQgTI</t>
+  </si>
+  <si>
+    <t>Parte 2 Activación</t>
+  </si>
+  <si>
+    <t>principal</t>
+  </si>
+  <si>
     <t>https://youtu.be/ivunOFSM1ME</t>
   </si>
   <si>
     <t>Trabajo principal</t>
   </si>
   <si>
-    <t>https://youtu.be/n5sBx_cosTY</t>
-  </si>
-  <si>
-    <t>Parte 1 Activación</t>
-  </si>
-  <si>
-    <t>https://youtu.be/X55mwKhQgTI</t>
-  </si>
-  <si>
-    <t>Parte 2 Activación</t>
-  </si>
-  <si>
     <t>https://youtu.be/KkCJE1znlL4</t>
   </si>
   <si>
@@ -66,13 +78,19 @@
     <t>https://youtu.be/_kizq4KY_jk</t>
   </si>
   <si>
-    <t>Juego de posesión</t>
+    <t>Juego de posesión libre</t>
+  </si>
+  <si>
+    <t>En el juego de posesión libre (14 vs 13) se observa que algunos jugadores quedan aislados del balón, disminuyendo su participación. Además, por momentos se evidencia una ocupación inadecuada de los espacios, con varios jugadores concentrándose en una misma zona del campo</t>
   </si>
   <si>
     <t>https://youtu.be/xmtyeaOQRJY</t>
   </si>
   <si>
-    <t>Juego de posesión con variante</t>
+    <t>Juego de posesión + 4 arcos</t>
+  </si>
+  <si>
+    <t>En el juego de posesión con cuatro arcos, el objetivo de sumar puntos al realizar una pared entre los arcos permitió que los jugadores se distribuyan mejor en el campo. No obstante, se observaron dificultades en la ocupación racional de los espacios y en la ejecución de la presión tras pérdida.</t>
   </si>
   <si>
     <t>https://youtu.be/G6DleZgwdZc</t>
@@ -101,7 +119,7 @@
     <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -115,9 +133,24 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -128,15 +161,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
-    </font>
-    <font>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -153,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -161,10 +185,10 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -173,10 +197,16 @@
     <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -393,141 +423,187 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="10.71"/>
-    <col customWidth="1" min="2" max="2" width="29.71"/>
-    <col customWidth="1" min="3" max="3" width="29.29"/>
-    <col customWidth="1" min="4" max="14" width="9.14"/>
+    <col customWidth="1" min="2" max="3" width="29.71"/>
+    <col customWidth="1" min="4" max="4" width="36.57"/>
+    <col customWidth="1" min="5" max="5" width="12.0"/>
+    <col customWidth="1" min="6" max="15" width="9.14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3">
+      <c r="A2" s="4">
         <v>46087.0</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>4</v>
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3">
+      <c r="A3" s="4">
         <v>46087.0</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="7" t="s">
-        <v>6</v>
+      <c r="C3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3">
+      <c r="A4" s="4">
         <v>46087.0</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>8</v>
+      <c r="B4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8">
+      <c r="A5" s="10">
         <v>46092.0</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>10</v>
+      <c r="B5" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8">
+      <c r="A6" s="10">
         <v>46092.0</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>12</v>
+      <c r="B6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8">
+      <c r="A7" s="10">
         <v>46093.0</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>14</v>
+      <c r="B7" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8">
+      <c r="A8" s="10">
         <v>46093.0</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>16</v>
+      <c r="B8" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="8">
+      <c r="A9" s="10">
         <v>46093.0</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>18</v>
+      <c r="B9" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8">
+      <c r="A10" s="10">
         <v>46093.0</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>20</v>
+      <c r="B10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8">
+      <c r="A11" s="10">
         <v>46094.0</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>22</v>
+      <c r="B11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8">
+      <c r="A12" s="10">
         <v>46094.0</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>24</v>
+      <c r="B12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1"/>
@@ -1512,17 +1588,17 @@
     <row r="997" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B2"/>
-    <hyperlink r:id="rId2" ref="B3"/>
-    <hyperlink r:id="rId3" ref="B4"/>
-    <hyperlink r:id="rId4" ref="B5"/>
-    <hyperlink r:id="rId5" ref="B6"/>
-    <hyperlink r:id="rId6" ref="B7"/>
-    <hyperlink r:id="rId7" ref="B8"/>
-    <hyperlink r:id="rId8" ref="B9"/>
-    <hyperlink r:id="rId9" ref="B10"/>
-    <hyperlink r:id="rId10" ref="B11"/>
-    <hyperlink r:id="rId11" ref="B12"/>
+    <hyperlink r:id="rId1" ref="C2"/>
+    <hyperlink r:id="rId2" ref="C3"/>
+    <hyperlink r:id="rId3" ref="C4"/>
+    <hyperlink r:id="rId4" ref="C5"/>
+    <hyperlink r:id="rId5" ref="C6"/>
+    <hyperlink r:id="rId6" ref="C7"/>
+    <hyperlink r:id="rId7" ref="C8"/>
+    <hyperlink r:id="rId8" ref="C9"/>
+    <hyperlink r:id="rId9" ref="C10"/>
+    <hyperlink r:id="rId10" ref="C11"/>
+    <hyperlink r:id="rId11" ref="C12"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
comentarios entrenamientos- cualquier tutpo
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="31">
   <si>
     <t>date</t>
   </si>
@@ -99,13 +99,13 @@
     <t>Trabajo principal 11vs11</t>
   </si>
   <si>
+    <t>https://youtu.be/aUB0ivrBZ5Y</t>
+  </si>
+  <si>
     <t>https://youtu.be/sZKL7Xz15aM</t>
   </si>
   <si>
     <t>Orientación corporal - Secuencia de pases</t>
-  </si>
-  <si>
-    <t>https://youtu.be/aUB0ivrBZ5Y</t>
   </si>
   <si>
     <t>Defensa: altura bloque defensivo</t>
@@ -577,6 +577,9 @@
       <c r="D10" s="9" t="s">
         <v>26</v>
       </c>
+      <c r="E10" s="6" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10">
@@ -586,10 +589,10 @@
         <v>5</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12">
@@ -600,7 +603,7 @@
         <v>10</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>30</v>
@@ -1597,12 +1600,13 @@
     <hyperlink r:id="rId7" ref="C8"/>
     <hyperlink r:id="rId8" ref="C9"/>
     <hyperlink r:id="rId9" ref="C10"/>
-    <hyperlink r:id="rId10" ref="C11"/>
-    <hyperlink r:id="rId11" ref="C12"/>
+    <hyperlink r:id="rId10" ref="E10"/>
+    <hyperlink r:id="rId11" ref="C11"/>
+    <hyperlink r:id="rId12" ref="C12"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId12"/>
+  <drawing r:id="rId13"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
INFORME 13-3 VERDE SOLO
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="35">
   <si>
     <t>date</t>
   </si>
@@ -114,7 +114,13 @@
     <t>Defensa: altura bloque defensivo</t>
   </si>
   <si>
-    <t>https://youtu.be/y-FhcawgroY</t>
+    <t>https://youtu.be/34bsA2CBhR8</t>
+  </si>
+  <si>
+    <t>https://youtu.be/49fjSv1kONA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partido de práctica </t>
   </si>
 </sst>
 </file>
@@ -634,6 +640,18 @@
       </c>
     </row>
     <row r="13">
+      <c r="A13" s="10">
+        <v>46095.0</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>34</v>
+      </c>
       <c r="E13" s="12"/>
     </row>
     <row r="18" ht="15.75" customHeight="1"/>
@@ -1630,10 +1648,11 @@
     <hyperlink r:id="rId10" ref="C11"/>
     <hyperlink r:id="rId11" ref="C12"/>
     <hyperlink r:id="rId12" ref="E12"/>
+    <hyperlink r:id="rId13" ref="C13"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId13"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add video entrenamientos 17-03
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="Zd2bzr3F57PIdj0Z1LFheCHbwMhROcEBkIiM90EgRzo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="XfP2vcvOrOF1Zrq4pTgU79YJpAZonK0/hQHcdwQx+JU="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="46">
   <si>
     <t>date</t>
   </si>
@@ -124,15 +124,46 @@
   </si>
   <si>
     <t xml:space="preserve">Partido de práctica </t>
+  </si>
+  <si>
+    <t>pruebas</t>
+  </si>
+  <si>
+    <t>https://youtu.be/GUwuiwzLQOo</t>
+  </si>
+  <si>
+    <t>Yo-yo test</t>
+  </si>
+  <si>
+    <t>Pre activación</t>
+  </si>
+  <si>
+    <t>https://youtu.be/3EX6bh7VSE4</t>
+  </si>
+  <si>
+    <t>Activación: parte1</t>
+  </si>
+  <si>
+    <t>https://youtu.be/7y4N7vAIObI</t>
+  </si>
+  <si>
+    <t>Activación: rondos</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-dOzqM2vlgk</t>
+  </si>
+  <si>
+    <t>Cambios de orientación</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="D/M/YYYY"/>
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -201,7 +232,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -237,6 +268,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -660,7 +694,62 @@
       </c>
       <c r="E13" s="12"/>
     </row>
-    <row r="18" ht="15.75" customHeight="1"/>
+    <row r="14">
+      <c r="A14" s="13">
+        <v>46097.0</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13">
+        <v>46098.0</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13">
+        <v>46098.0</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <v>46098.0</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="19" ht="15.75" customHeight="1"/>
     <row r="20" ht="15.75" customHeight="1"/>
     <row r="21" ht="15.75" customHeight="1"/>
@@ -1640,6 +1729,7 @@
     <row r="995" ht="15.75" customHeight="1"/>
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -1656,10 +1746,14 @@
     <hyperlink r:id="rId12" ref="C12"/>
     <hyperlink r:id="rId13" ref="E12"/>
     <hyperlink r:id="rId14" ref="C13"/>
+    <hyperlink r:id="rId15" ref="C14"/>
+    <hyperlink r:id="rId16" ref="C15"/>
+    <hyperlink r:id="rId17" ref="C16"/>
+    <hyperlink r:id="rId18" ref="C17"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId15"/>
+  <drawing r:id="rId19"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add video entrenamiento 18-03
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="XfP2vcvOrOF1Zrq4pTgU79YJpAZonK0/hQHcdwQx+JU="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="FRKDRpntz1Z9Sb+vqAo05clanKXWihQJsJaeT5Mbh00="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
   <si>
     <t>date</t>
   </si>
@@ -154,6 +154,18 @@
   </si>
   <si>
     <t>Cambios de orientación</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xG2IbfbCNP4</t>
+  </si>
+  <si>
+    <t>Activación sin balón</t>
+  </si>
+  <si>
+    <t>https://youtu.be/nhWVeRTy_Gc</t>
+  </si>
+  <si>
+    <t>Se inició con el equipo blanco en una estructura 3-5-2 y el equipo naranja en un sistema 4-4-2, incidiendo principalmente en el inicio de juego estático(saque de meta). En el siguiente bloque se invirtieron las estructuras iniciales entre ambos equipos. Durante el desarrollo de la tarea, se buscó generar una superioridad numérica de 3 vs 1 en el carril exterior para progresar. Posteriormente se realizaba el cambio de orientación hacia el carril opuesto y la finalización de la jugada mediante un centro al área.</t>
   </si>
 </sst>
 </file>
@@ -232,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -273,6 +285,7 @@
     <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -750,11 +763,50 @@
         <v>45</v>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1"/>
-    <row r="20" ht="15.75" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
+    <row r="18">
+      <c r="A18" s="13">
+        <v>46099.0</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="E18" s="12"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13">
+        <v>46099.0</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="12" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="E20" s="14"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="E21" s="12"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="E22" s="14"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="E23" s="12"/>
+    </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
     <row r="26" ht="15.75" customHeight="1"/>
@@ -1730,6 +1782,7 @@
     <row r="996" ht="15.75" customHeight="1"/>
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -1750,10 +1803,12 @@
     <hyperlink r:id="rId16" ref="C15"/>
     <hyperlink r:id="rId17" ref="C16"/>
     <hyperlink r:id="rId18" ref="C17"/>
+    <hyperlink r:id="rId19" ref="C18"/>
+    <hyperlink r:id="rId20" ref="C19"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId19"/>
+  <drawing r:id="rId21"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add videos: parido vs Nazca
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="54">
   <si>
     <t>date</t>
   </si>
@@ -126,6 +126,9 @@
     <t xml:space="preserve">Partido de práctica </t>
   </si>
   <si>
+    <t>https://youtu.be/Ub1KGSTFWaY</t>
+  </si>
+  <si>
     <t>pruebas</t>
   </si>
   <si>
@@ -166,6 +169,15 @@
   </si>
   <si>
     <t>Se inició con el equipo blanco en una estructura 3-5-2 y el equipo naranja en un sistema 4-4-2, incidiendo principalmente en el inicio de juego estático(saque de meta). En el siguiente bloque se invirtieron las estructuras iniciales entre ambos equipos. Durante el desarrollo de la tarea, se buscó generar una superioridad numérica de 3 vs 1 en el carril exterior para progresar. Posteriormente se realizaba el cambio de orientación hacia el carril opuesto y la finalización de la jugada mediante un centro al área.</t>
+  </si>
+  <si>
+    <t>amistoso</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Xk6znucIHM8</t>
+  </si>
+  <si>
+    <t>Partido vs Santos FC</t>
   </si>
 </sst>
 </file>
@@ -279,10 +291,10 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
@@ -705,107 +717,121 @@
       <c r="D13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="12"/>
+      <c r="E13" s="11" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="13">
+      <c r="A14" s="12">
         <v>46097.0</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13">
+      <c r="A15" s="12">
         <v>46098.0</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13">
+      <c r="A16" s="12">
         <v>46098.0</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13">
+      <c r="A17" s="12">
         <v>46098.0</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13">
+      <c r="A18" s="12">
         <v>46099.0</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>5</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E18" s="12"/>
+        <v>48</v>
+      </c>
+      <c r="E18" s="13"/>
     </row>
     <row r="19">
-      <c r="A19" s="13">
+      <c r="A19" s="12">
         <v>46099.0</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="12" t="s">
-        <v>49</v>
+      <c r="E19" s="13" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="12">
+        <v>46102.0</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>53</v>
+      </c>
       <c r="E20" s="14"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="E21" s="12"/>
+      <c r="E21" s="13"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="E22" s="14"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="E23" s="12"/>
+      <c r="E23" s="13"/>
     </row>
     <row r="24" ht="15.75" customHeight="1"/>
     <row r="25" ht="15.75" customHeight="1"/>
@@ -1799,16 +1825,18 @@
     <hyperlink r:id="rId12" ref="C12"/>
     <hyperlink r:id="rId13" ref="E12"/>
     <hyperlink r:id="rId14" ref="C13"/>
-    <hyperlink r:id="rId15" ref="C14"/>
-    <hyperlink r:id="rId16" ref="C15"/>
-    <hyperlink r:id="rId17" ref="C16"/>
-    <hyperlink r:id="rId18" ref="C17"/>
-    <hyperlink r:id="rId19" ref="C18"/>
-    <hyperlink r:id="rId20" ref="C19"/>
+    <hyperlink r:id="rId15" ref="E13"/>
+    <hyperlink r:id="rId16" ref="C14"/>
+    <hyperlink r:id="rId17" ref="C15"/>
+    <hyperlink r:id="rId18" ref="C16"/>
+    <hyperlink r:id="rId19" ref="C17"/>
+    <hyperlink r:id="rId20" ref="C18"/>
+    <hyperlink r:id="rId21" ref="C19"/>
+    <hyperlink r:id="rId22" ref="C20"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId21"/>
+  <drawing r:id="rId23"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add video amistos U 28-03
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="101">
   <si>
     <t>date</t>
   </si>
@@ -250,6 +250,12 @@
   </si>
   <si>
     <t xml:space="preserve">10 vs 10 | 5 toques </t>
+  </si>
+  <si>
+    <t>https://youtu.be/0_4O_T7QRPg</t>
+  </si>
+  <si>
+    <t>Amistoso vs Universitario</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -1089,7 +1095,17 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="12">
+        <v>46109.0</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
     <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
@@ -2093,11 +2109,12 @@
     <hyperlink r:id="rId28" ref="C25"/>
     <hyperlink r:id="rId29" ref="C26"/>
     <hyperlink r:id="rId30" ref="C27"/>
+    <hyperlink r:id="rId31" ref="C28"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId31"/>
+  <drawing r:id="rId32"/>
 </worksheet>
 </file>
 
@@ -2113,18 +2130,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2132,13 +2149,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2146,13 +2163,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2160,21 +2177,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>79</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2182,13 +2199,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2196,13 +2213,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2210,42 +2227,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2253,13 +2270,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2267,21 +2284,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2289,13 +2306,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2303,26 +2320,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update entrenamientos hasta 0304
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="104">
   <si>
     <t>date</t>
   </si>
@@ -256,6 +256,15 @@
   </si>
   <si>
     <t>Amistoso vs Universitario</t>
+  </si>
+  <si>
+    <t>Amistoso vs Municipal</t>
+  </si>
+  <si>
+    <t>https://youtu.be/8Xf9SK91JKc</t>
+  </si>
+  <si>
+    <t>Amistoso vs S. Cristal</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -1106,8 +1115,25 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1"/>
-    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="12">
+        <v>46114.0</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="12">
+        <v>46115.0</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
@@ -2110,11 +2136,12 @@
     <hyperlink r:id="rId29" ref="C26"/>
     <hyperlink r:id="rId30" ref="C27"/>
     <hyperlink r:id="rId31" ref="C28"/>
+    <hyperlink r:id="rId32" ref="C30"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId32"/>
+  <drawing r:id="rId33"/>
 </worksheet>
 </file>
 
@@ -2130,18 +2157,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2149,13 +2176,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2163,13 +2190,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2177,21 +2204,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B6" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2199,13 +2226,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2213,13 +2240,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2227,42 +2254,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2270,13 +2297,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2284,21 +2311,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2306,13 +2333,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2320,26 +2347,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento 04 y 07 de abril
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="109">
   <si>
     <t>date</t>
   </si>
@@ -258,6 +258,9 @@
     <t>Amistoso vs Universitario</t>
   </si>
   <si>
+    <t>https://youtu.be/3bDA_rtL_Vs</t>
+  </si>
+  <si>
     <t>Amistoso vs Municipal</t>
   </si>
   <si>
@@ -265,6 +268,18 @@
   </si>
   <si>
     <t>Amistoso vs S. Cristal</t>
+  </si>
+  <si>
+    <t>https://youtu.be/X1vXECYNzh0</t>
+  </si>
+  <si>
+    <t>Reducido + definición</t>
+  </si>
+  <si>
+    <t>https://youtu.be/PHP58KYb47I</t>
+  </si>
+  <si>
+    <t>Pelota parada y reducido</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -1117,25 +1132,48 @@
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="12">
-        <v>46114.0</v>
+        <v>46113.0</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>70</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="12">
-        <v>46115.0</v>
+        <v>46114.0</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1"/>
-    <row r="32" ht="15.75" customHeight="1"/>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="12">
+        <v>46116.0</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="12">
+        <v>46119.0</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
@@ -2136,12 +2174,15 @@
     <hyperlink r:id="rId29" ref="C26"/>
     <hyperlink r:id="rId30" ref="C27"/>
     <hyperlink r:id="rId31" ref="C28"/>
-    <hyperlink r:id="rId32" ref="C30"/>
+    <hyperlink r:id="rId32" ref="C29"/>
+    <hyperlink r:id="rId33" ref="C30"/>
+    <hyperlink r:id="rId34" ref="C31"/>
+    <hyperlink r:id="rId35" ref="C32"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId33"/>
+  <drawing r:id="rId36"/>
 </worksheet>
 </file>
 
@@ -2157,18 +2198,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2176,13 +2217,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2190,13 +2231,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2204,21 +2245,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2226,13 +2267,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2240,13 +2281,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>83</v>
-      </c>
       <c r="I8" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2254,42 +2295,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2297,13 +2338,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2311,21 +2352,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2333,13 +2374,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I18" s="5" t="s">
         <v>84</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="I18" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2347,26 +2388,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add video amistoso vs PAcifico
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="111">
   <si>
     <t>date</t>
   </si>
@@ -280,6 +280,12 @@
   </si>
   <si>
     <t>Pelota parada y reducido</t>
+  </si>
+  <si>
+    <t>https://youtu.be/odrktL-0Hnk</t>
+  </si>
+  <si>
+    <t>Amistoso vs Pacífico FC</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -1174,7 +1180,17 @@
         <v>77</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="12">
+        <v>46120.0</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>
@@ -2178,11 +2194,12 @@
     <hyperlink r:id="rId33" ref="C30"/>
     <hyperlink r:id="rId34" ref="C31"/>
     <hyperlink r:id="rId35" ref="C32"/>
+    <hyperlink r:id="rId36" ref="C33"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId36"/>
+  <drawing r:id="rId37"/>
 </worksheet>
 </file>
 
@@ -2198,18 +2215,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2217,13 +2234,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2231,13 +2248,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2245,21 +2262,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>87</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2267,13 +2284,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2281,13 +2298,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2295,42 +2312,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2338,13 +2355,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2352,21 +2369,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2374,13 +2391,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2388,26 +2405,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento regreso de Lima
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -10,14 +10,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="NRU55Wbw9z11eqq6+GGX68DODvVv2WBcNfwsQoKThig="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="hei4pOW1qlb/hUfW6D3P3iKZbMqCsgEoQXCCdosrhzU="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="124">
   <si>
     <t>date</t>
   </si>
@@ -288,6 +288,45 @@
     <t>Amistoso vs Pacífico FC</t>
   </si>
   <si>
+    <t>https://www.youtube.com/watch?v=LtiJAa6vzso</t>
+  </si>
+  <si>
+    <t>1er turno - 8:00am</t>
+  </si>
+  <si>
+    <t>2do turno - 3:00pm</t>
+  </si>
+  <si>
+    <t>Turno único - 9:00am</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ZTZxFwlGCNk</t>
+  </si>
+  <si>
+    <t>2do Turno 3:00pm</t>
+  </si>
+  <si>
+    <t>1) Arqueros. 2) Secuencia de pases 2 toques solo derecha, 2 toques solo izquierda, dos toque ambos pies obligatorio, 1 toque derecha, 1 toque izquierda. 3) Rondos. 4) Reducido</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-E6BGD98zegIL</t>
+  </si>
+  <si>
+    <t>3er turno - 3:00pm</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=K4N1JCZkOFo</t>
+  </si>
+  <si>
+    <t>https://youtu.be/VdQyflL3y8I</t>
+  </si>
+  <si>
+    <t>Turno único - 1:00pm</t>
+  </si>
+  <si>
+    <t>Rondos 4 vs 1 - Futbol 11 vs 11, Dando algunas condiciones al equipo defensor, Bloque Alto, Medio, bajo</t>
+  </si>
+  <si>
     <t>VERDE</t>
   </si>
   <si>
@@ -390,7 +429,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -446,13 +485,23 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -461,7 +510,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -502,8 +551,21 @@
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -724,7 +786,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="10.71"/>
-    <col customWidth="1" min="2" max="3" width="29.71"/>
+    <col customWidth="1" min="2" max="2" width="14.71"/>
+    <col customWidth="1" min="3" max="3" width="44.29"/>
     <col customWidth="1" min="4" max="4" width="36.57"/>
     <col customWidth="1" min="5" max="5" width="12.0"/>
     <col customWidth="1" min="6" max="15" width="9.14"/>
@@ -1022,19 +1085,19 @@
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="12">
+      <c r="A20" s="14">
         <v>46102.0</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="14"/>
+      <c r="E20" s="17"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="12">
@@ -1058,7 +1121,7 @@
       <c r="D22" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="14"/>
+      <c r="E22" s="17"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="12">
@@ -1079,7 +1142,7 @@
       <c r="B24" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="15" t="s">
+      <c r="C24" s="18" t="s">
         <v>58</v>
       </c>
       <c r="D24" s="5" t="s">
@@ -1126,35 +1189,38 @@
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="12">
+      <c r="A28" s="14">
         <v>46109.0</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="B28" s="19"/>
+      <c r="C28" s="16" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="15" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="12">
+      <c r="A29" s="14">
         <v>46113.0</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="B29" s="19"/>
+      <c r="C29" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="15" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="12">
+      <c r="A30" s="14">
         <v>46114.0</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="B30" s="19"/>
+      <c r="C30" s="16" t="s">
         <v>72</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="15" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1162,7 +1228,7 @@
       <c r="A31" s="12">
         <v>46116.0</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="18" t="s">
         <v>74</v>
       </c>
       <c r="D31" s="5" t="s">
@@ -1181,24 +1247,105 @@
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="12">
+      <c r="A33" s="14">
         <v>46120.0</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="B33" s="19"/>
+      <c r="C33" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="15" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1"/>
-    <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
-    <row r="37" ht="15.75" customHeight="1"/>
-    <row r="38" ht="15.75" customHeight="1"/>
-    <row r="39" ht="15.75" customHeight="1"/>
-    <row r="40" ht="15.75" customHeight="1"/>
-    <row r="41" ht="15.75" customHeight="1"/>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="12">
+        <v>46127.0</v>
+      </c>
+      <c r="C34" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="12">
+        <v>46127.0</v>
+      </c>
+      <c r="C35" s="20"/>
+      <c r="D35" s="5" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="12">
+        <v>46128.0</v>
+      </c>
+      <c r="C36" s="20"/>
+      <c r="D36" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="12">
+        <v>46129.0</v>
+      </c>
+      <c r="C37" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="D37" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="E37" s="5" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="12">
+        <v>46130.0</v>
+      </c>
+      <c r="C38" s="18" t="s">
+        <v>87</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="12">
+        <v>46131.0</v>
+      </c>
+      <c r="C39" s="20"/>
+      <c r="D39" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="12">
+        <v>46131.0</v>
+      </c>
+      <c r="C40" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="12">
+        <v>46132.0</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>92</v>
+      </c>
+    </row>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1"/>
     <row r="44" ht="15.75" customHeight="1"/>
@@ -2157,6 +2304,12 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
+    <row r="1005" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -2195,11 +2348,16 @@
     <hyperlink r:id="rId34" ref="C31"/>
     <hyperlink r:id="rId35" ref="C32"/>
     <hyperlink r:id="rId36" ref="C33"/>
+    <hyperlink r:id="rId37" ref="C34"/>
+    <hyperlink r:id="rId38" ref="C37"/>
+    <hyperlink r:id="rId39" ref="C38"/>
+    <hyperlink r:id="rId40" ref="C40"/>
+    <hyperlink r:id="rId41" ref="C41"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId37"/>
+  <drawing r:id="rId42"/>
 </worksheet>
 </file>
 
@@ -2215,18 +2373,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>80</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2234,13 +2392,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>85</v>
+        <v>98</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2248,13 +2406,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2262,21 +2420,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2284,13 +2442,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2298,13 +2456,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2312,42 +2470,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2355,13 +2513,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2369,21 +2527,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2391,13 +2549,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2405,26 +2563,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento 19/04 turno2
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="128">
   <si>
     <t>date</t>
   </si>
@@ -294,9 +294,15 @@
     <t>1er turno - 8:00am</t>
   </si>
   <si>
+    <t>https://youtu.be/3rSESA4TROM</t>
+  </si>
+  <si>
     <t>2do turno - 3:00pm</t>
   </si>
   <si>
+    <t>https://www.youtube.com/watch?v=9e1xepsJYq0</t>
+  </si>
+  <si>
     <t>Turno único - 9:00am</t>
   </si>
   <si>
@@ -312,10 +318,16 @@
     <t>https://www.youtube.com/watch?v=-E6BGD98zegIL</t>
   </si>
   <si>
+    <t>https://youtu.be/gmf6pZ7NCOQ</t>
+  </si>
+  <si>
+    <t>2do turno - 10:00am</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=K4N1JCZkOFo</t>
+  </si>
+  <si>
     <t>3er turno - 3:00pm</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=K4N1JCZkOFo</t>
   </si>
   <si>
     <t>https://youtu.be/VdQyflL3y8I</t>
@@ -510,7 +522,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -565,9 +577,6 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -787,7 +796,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="10.71"/>
     <col customWidth="1" min="2" max="2" width="14.71"/>
-    <col customWidth="1" min="3" max="3" width="44.29"/>
+    <col customWidth="1" min="3" max="3" width="45.43"/>
     <col customWidth="1" min="4" max="4" width="36.57"/>
     <col customWidth="1" min="5" max="5" width="12.0"/>
     <col customWidth="1" min="6" max="15" width="9.14"/>
@@ -1273,18 +1282,22 @@
       <c r="A35" s="12">
         <v>46127.0</v>
       </c>
-      <c r="C35" s="20"/>
+      <c r="C35" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="D35" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="12">
         <v>46128.0</v>
       </c>
-      <c r="C36" s="20"/>
+      <c r="C36" s="18" t="s">
+        <v>84</v>
+      </c>
       <c r="D36" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
@@ -1292,13 +1305,13 @@
         <v>46129.0</v>
       </c>
       <c r="C37" s="18" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
@@ -1306,19 +1319,21 @@
         <v>46130.0</v>
       </c>
       <c r="C38" s="18" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="12">
         <v>46131.0</v>
       </c>
-      <c r="C39" s="20"/>
+      <c r="C39" s="18" t="s">
+        <v>90</v>
+      </c>
       <c r="D39" s="5" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -1326,10 +1341,10 @@
         <v>46131.0</v>
       </c>
       <c r="C40" s="18" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
@@ -1337,13 +1352,13 @@
         <v>46132.0</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1"/>
@@ -2349,15 +2364,18 @@
     <hyperlink r:id="rId35" ref="C32"/>
     <hyperlink r:id="rId36" ref="C33"/>
     <hyperlink r:id="rId37" ref="C34"/>
-    <hyperlink r:id="rId38" ref="C37"/>
-    <hyperlink r:id="rId39" ref="C38"/>
-    <hyperlink r:id="rId40" ref="C40"/>
-    <hyperlink r:id="rId41" ref="C41"/>
+    <hyperlink r:id="rId38" ref="C35"/>
+    <hyperlink r:id="rId39" ref="C36"/>
+    <hyperlink r:id="rId40" ref="C37"/>
+    <hyperlink r:id="rId41" ref="C38"/>
+    <hyperlink r:id="rId42" ref="C39"/>
+    <hyperlink r:id="rId43" ref="C40"/>
+    <hyperlink r:id="rId44" ref="C41"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId42"/>
+  <drawing r:id="rId45"/>
 </worksheet>
 </file>
 
@@ -2373,18 +2391,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2392,13 +2410,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2406,13 +2424,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2420,21 +2438,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2442,13 +2460,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2456,13 +2474,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2470,42 +2488,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2513,13 +2531,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2527,21 +2545,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2549,13 +2567,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2563,26 +2581,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 24-04
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="148">
   <si>
     <t>date</t>
   </si>
@@ -360,6 +360,71 @@
     <t>3er turno - 4pm</t>
   </si>
   <si>
+    <t>https://www.youtube.com/watch?v=9_M1nZB-ZKI</t>
+  </si>
+  <si>
+    <t>1ER TURNO - 9am</t>
+  </si>
+  <si>
+    <t>Entrenamiento del 23 de abril 
+Fase de Activación: 20 minutos de carrera continua - trabajo de resistencia, arte principal:
+Juego reducido 11VS11
+Equipo blanco:
+1. taylor /Bebote 
+2. ⁠cueva
+3. ⁠acasiete
+4. ⁠casas 
+5. ⁠Chávez
+6. ⁠Ortiz
+7. ⁠Romaric
+8. ⁠Ferreira
+9. ⁠centurión 
+10. ⁠Jair
+11. ⁠Joaquín 
+Equipo verde
+1. Escalante/Eden
+2. ⁠Perea
+3. ⁠Joaquín 
+4. ⁠Fernández
+5. ⁠Macines 
+6. ⁠Jerjes
+7. ⁠chinga
+8. ⁠Jeremy
+9. ⁠Pedro
+10. ⁠Zúñiga 
+11. ⁠castro</t>
+  </si>
+  <si>
+    <t>https://youtu.be/2A5FJYTC-Q0</t>
+  </si>
+  <si>
+    <t>2DO TURNO - 4:30P.M</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bXof8DRI8G0</t>
+  </si>
+  <si>
+    <t>1ER TURNO - 7:00am</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secuencia de pases , Centros y Definición. </t>
+  </si>
+  <si>
+    <t>https://youtu.be/5iB_95FahgA</t>
+  </si>
+  <si>
+    <t>2DO TURNO - 11:00am</t>
+  </si>
+  <si>
+    <t>Cambios de orientacion - Centros y Definicion</t>
+  </si>
+  <si>
+    <t>3ER TURNO- 3:00 P.M</t>
+  </si>
+  <si>
+    <t>Juego 11 VS 11</t>
+  </si>
+  <si>
     <t>VERDE</t>
   </si>
   <si>
@@ -462,7 +527,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -522,6 +587,11 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font>
+      <b/>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -543,7 +613,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -598,6 +668,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1413,11 +1486,68 @@
         <v>103</v>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="12">
+        <v>46135.0</v>
+      </c>
+      <c r="C44" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="E44" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="H44" s="5"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="12">
+        <v>46135.0</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="12">
+        <v>46136.0</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="12">
+        <v>46136.0</v>
+      </c>
+      <c r="C47" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="E47" s="5" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="D48" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>116</v>
+      </c>
+    </row>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
@@ -2424,11 +2554,15 @@
     <hyperlink r:id="rId44" ref="C41"/>
     <hyperlink r:id="rId45" ref="C42"/>
     <hyperlink r:id="rId46" ref="C43"/>
+    <hyperlink r:id="rId47" ref="C44"/>
+    <hyperlink r:id="rId48" ref="C45"/>
+    <hyperlink r:id="rId49" ref="C46"/>
+    <hyperlink r:id="rId50" ref="C47"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId47"/>
+  <drawing r:id="rId51"/>
 </worksheet>
 </file>
 
@@ -2444,18 +2578,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>104</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="J2" s="5">
         <v>6.0</v>
@@ -2463,13 +2597,13 @@
     </row>
     <row r="3">
       <c r="A3" s="5" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="J3" s="5">
         <v>1.0</v>
@@ -2477,13 +2611,13 @@
     </row>
     <row r="4">
       <c r="A4" s="5" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="J4" s="5">
         <v>1.0</v>
@@ -2491,21 +2625,21 @@
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="J6" s="5">
         <v>2.0</v>
@@ -2513,13 +2647,13 @@
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>117</v>
+        <v>130</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="J7" s="5">
         <v>1.0</v>
@@ -2527,13 +2661,13 @@
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>114</v>
+        <v>127</v>
       </c>
       <c r="I8" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="J8" s="5">
         <v>1.0</v>
@@ -2541,42 +2675,42 @@
     </row>
     <row r="9">
       <c r="A9" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>121</v>
+        <v>134</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>125</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="J14" s="5">
         <v>2.0</v>
@@ -2584,13 +2718,13 @@
     </row>
     <row r="15">
       <c r="A15" s="5" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="J15" s="5">
         <v>2.0</v>
@@ -2598,21 +2732,21 @@
     </row>
     <row r="16">
       <c r="A16" s="5" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>107</v>
+        <v>120</v>
       </c>
       <c r="J17" s="5">
         <v>3.0</v>
@@ -2620,13 +2754,13 @@
     </row>
     <row r="18">
       <c r="A18" s="5" t="s">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>120</v>
+        <v>133</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="J18" s="5">
         <v>2.0</v>
@@ -2634,26 +2768,26 @@
     </row>
     <row r="19">
       <c r="A19" s="5" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="s">
-        <v>133</v>
+        <v>146</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>134</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 24-04 3 turno
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,9 +17,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="148">
-  <si>
-    <t>date</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="148">
+  <si>
+    <t>https://youtu.be/_8Jx9h36Sp8</t>
   </si>
   <si>
     <t>parte_entreno</t>
@@ -527,12 +527,19 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -613,62 +620,65 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="5" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="2" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -900,651 +910,657 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4">
+      <c r="A2" s="5">
         <v>46087.0</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3" s="5">
         <v>46087.0</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4">
+      <c r="A4" s="5">
         <v>46087.0</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10">
+      <c r="A5" s="11">
         <v>46092.0</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10">
+      <c r="A6" s="11">
         <v>46092.0</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="10">
+      <c r="A7" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="10">
+      <c r="A8" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="10">
+      <c r="A9" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="10">
+      <c r="A10" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="10">
+      <c r="A11" s="11">
         <v>46094.0</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="10">
+      <c r="A12" s="11">
         <v>46094.0</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="12" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="10">
+      <c r="A13" s="11">
         <v>46095.0</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="12" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12">
+      <c r="A14" s="13">
         <v>46097.0</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12">
+      <c r="A15" s="13">
         <v>46098.0</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12">
+      <c r="A16" s="13">
         <v>46098.0</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12">
+      <c r="A17" s="13">
         <v>46098.0</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12">
+      <c r="A18" s="13">
         <v>46099.0</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E18" s="13"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19">
-      <c r="A19" s="12">
+      <c r="A19" s="13">
         <v>46099.0</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="14" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="14">
+      <c r="A20" s="15">
         <v>46102.0</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="16" t="s">
+      <c r="C20" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="E20" s="17"/>
+      <c r="E20" s="18"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="12">
+      <c r="A21" s="13">
         <v>46103.0</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E21" s="13"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="12">
+      <c r="A22" s="13">
         <v>46104.0</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E22" s="17"/>
+      <c r="E22" s="18"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="12">
+      <c r="A23" s="13">
         <v>46105.0</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="13"/>
+      <c r="E23" s="14"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="12">
+      <c r="A24" s="13">
         <v>46106.0</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" s="7" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="12">
+      <c r="A25" s="13">
         <v>46108.0</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="12">
+      <c r="A26" s="13">
         <v>46108.0</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="12">
+      <c r="A27" s="13">
         <v>46108.0</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="6" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="14">
+      <c r="A28" s="15">
         <v>46109.0</v>
       </c>
-      <c r="B28" s="19"/>
-      <c r="C28" s="16" t="s">
+      <c r="B28" s="20"/>
+      <c r="C28" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="16" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="14">
+      <c r="A29" s="15">
         <v>46113.0</v>
       </c>
-      <c r="B29" s="19"/>
-      <c r="C29" s="16" t="s">
+      <c r="B29" s="20"/>
+      <c r="C29" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="16" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="14">
+      <c r="A30" s="15">
         <v>46114.0</v>
       </c>
-      <c r="B30" s="19"/>
-      <c r="C30" s="16" t="s">
+      <c r="B30" s="20"/>
+      <c r="C30" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="16" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="12">
+      <c r="A31" s="13">
         <v>46116.0</v>
       </c>
-      <c r="C31" s="18" t="s">
+      <c r="C31" s="19" t="s">
         <v>74</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="12">
+      <c r="A32" s="13">
         <v>46119.0</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="6" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="14">
+      <c r="A33" s="15">
         <v>46120.0</v>
       </c>
-      <c r="B33" s="19"/>
-      <c r="C33" s="16" t="s">
+      <c r="B33" s="20"/>
+      <c r="C33" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="D33" s="15" t="s">
+      <c r="D33" s="16" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="12">
+      <c r="A34" s="13">
         <v>46127.0</v>
       </c>
-      <c r="C34" s="18" t="s">
+      <c r="C34" s="19" t="s">
         <v>80</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="6" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="12">
+      <c r="A35" s="13">
         <v>46127.0</v>
       </c>
-      <c r="C35" s="18" t="s">
+      <c r="C35" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E35" s="6" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="12">
+      <c r="A36" s="13">
         <v>46128.0</v>
       </c>
-      <c r="C36" s="18" t="s">
+      <c r="C36" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="6" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="12">
+      <c r="A37" s="13">
         <v>46129.0</v>
       </c>
-      <c r="C37" s="18" t="s">
+      <c r="C37" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="12">
+      <c r="A38" s="13">
         <v>46130.0</v>
       </c>
-      <c r="C38" s="18" t="s">
+      <c r="C38" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="6" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="12">
+      <c r="A39" s="13">
         <v>46131.0</v>
       </c>
-      <c r="C39" s="18" t="s">
+      <c r="C39" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" s="6" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="12">
+      <c r="A40" s="13">
         <v>46131.0</v>
       </c>
-      <c r="C40" s="18" t="s">
+      <c r="C40" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="6" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="12">
+      <c r="A41" s="13">
         <v>46132.0</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D41" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E41" s="6" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="12">
+      <c r="A42" s="13">
         <v>46133.0</v>
       </c>
-      <c r="C42" s="18" t="s">
+      <c r="C42" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="D42" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" s="6" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="12">
+      <c r="A43" s="13">
         <v>46133.0</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D43" s="5" t="s">
+      <c r="D43" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="12">
+      <c r="A44" s="13">
         <v>46135.0</v>
       </c>
-      <c r="C44" s="18" t="s">
+      <c r="C44" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="D44" s="5" t="s">
+      <c r="D44" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E44" s="5" t="s">
+      <c r="E44" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="H44" s="5"/>
+      <c r="H44" s="6"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="12">
+      <c r="A45" s="13">
         <v>46135.0</v>
       </c>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D45" s="5" t="s">
+      <c r="D45" s="6" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="12">
+      <c r="A46" s="13">
         <v>46136.0</v>
       </c>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D46" s="5" t="s">
+      <c r="D46" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="E46" s="5" t="s">
+      <c r="E46" s="6" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="12">
+      <c r="A47" s="13">
         <v>46136.0</v>
       </c>
-      <c r="C47" s="20" t="s">
+      <c r="C47" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="D47" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="E47" s="5" t="s">
+      <c r="E47" s="6" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="D48" s="5" t="s">
+      <c r="A48" s="13">
+        <v>46136.0</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D48" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E48" s="5" t="s">
+      <c r="E48" s="6" t="s">
         <v>116</v>
       </c>
     </row>
@@ -2508,61 +2524,63 @@
     <row r="1006" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="C2"/>
-    <hyperlink r:id="rId2" ref="C3"/>
-    <hyperlink r:id="rId3" ref="C4"/>
-    <hyperlink r:id="rId4" ref="C5"/>
-    <hyperlink r:id="rId5" ref="C6"/>
-    <hyperlink r:id="rId6" ref="C7"/>
-    <hyperlink r:id="rId7" ref="C8"/>
-    <hyperlink r:id="rId8" ref="C9"/>
-    <hyperlink r:id="rId9" ref="C10"/>
-    <hyperlink r:id="rId10" ref="E10"/>
-    <hyperlink r:id="rId11" ref="C11"/>
-    <hyperlink r:id="rId12" ref="C12"/>
-    <hyperlink r:id="rId13" ref="E12"/>
-    <hyperlink r:id="rId14" ref="C13"/>
-    <hyperlink r:id="rId15" ref="E13"/>
-    <hyperlink r:id="rId16" ref="C14"/>
-    <hyperlink r:id="rId17" ref="C15"/>
-    <hyperlink r:id="rId18" ref="C16"/>
-    <hyperlink r:id="rId19" ref="C17"/>
-    <hyperlink r:id="rId20" ref="C18"/>
-    <hyperlink r:id="rId21" ref="C19"/>
-    <hyperlink r:id="rId22" ref="C20"/>
-    <hyperlink r:id="rId23" ref="C21"/>
-    <hyperlink r:id="rId24" ref="C22"/>
-    <hyperlink r:id="rId25" ref="C23"/>
-    <hyperlink r:id="rId26" ref="C24"/>
-    <hyperlink r:id="rId27" ref="E24"/>
-    <hyperlink r:id="rId28" ref="C25"/>
-    <hyperlink r:id="rId29" ref="C26"/>
-    <hyperlink r:id="rId30" ref="C27"/>
-    <hyperlink r:id="rId31" ref="C28"/>
-    <hyperlink r:id="rId32" ref="C29"/>
-    <hyperlink r:id="rId33" ref="C30"/>
-    <hyperlink r:id="rId34" ref="C31"/>
-    <hyperlink r:id="rId35" ref="C32"/>
-    <hyperlink r:id="rId36" ref="C33"/>
-    <hyperlink r:id="rId37" ref="C34"/>
-    <hyperlink r:id="rId38" ref="C35"/>
-    <hyperlink r:id="rId39" ref="C36"/>
-    <hyperlink r:id="rId40" ref="C37"/>
-    <hyperlink r:id="rId41" ref="C38"/>
-    <hyperlink r:id="rId42" ref="C39"/>
-    <hyperlink r:id="rId43" ref="C40"/>
-    <hyperlink r:id="rId44" ref="C41"/>
-    <hyperlink r:id="rId45" ref="C42"/>
-    <hyperlink r:id="rId46" ref="C43"/>
-    <hyperlink r:id="rId47" ref="C44"/>
-    <hyperlink r:id="rId48" ref="C45"/>
-    <hyperlink r:id="rId49" ref="C46"/>
-    <hyperlink r:id="rId50" ref="C47"/>
+    <hyperlink r:id="rId1" ref="A1"/>
+    <hyperlink r:id="rId2" ref="C2"/>
+    <hyperlink r:id="rId3" ref="C3"/>
+    <hyperlink r:id="rId4" ref="C4"/>
+    <hyperlink r:id="rId5" ref="C5"/>
+    <hyperlink r:id="rId6" ref="C6"/>
+    <hyperlink r:id="rId7" ref="C7"/>
+    <hyperlink r:id="rId8" ref="C8"/>
+    <hyperlink r:id="rId9" ref="C9"/>
+    <hyperlink r:id="rId10" ref="C10"/>
+    <hyperlink r:id="rId11" ref="E10"/>
+    <hyperlink r:id="rId12" ref="C11"/>
+    <hyperlink r:id="rId13" ref="C12"/>
+    <hyperlink r:id="rId14" ref="E12"/>
+    <hyperlink r:id="rId15" ref="C13"/>
+    <hyperlink r:id="rId16" ref="E13"/>
+    <hyperlink r:id="rId17" ref="C14"/>
+    <hyperlink r:id="rId18" ref="C15"/>
+    <hyperlink r:id="rId19" ref="C16"/>
+    <hyperlink r:id="rId20" ref="C17"/>
+    <hyperlink r:id="rId21" ref="C18"/>
+    <hyperlink r:id="rId22" ref="C19"/>
+    <hyperlink r:id="rId23" ref="C20"/>
+    <hyperlink r:id="rId24" ref="C21"/>
+    <hyperlink r:id="rId25" ref="C22"/>
+    <hyperlink r:id="rId26" ref="C23"/>
+    <hyperlink r:id="rId27" ref="C24"/>
+    <hyperlink r:id="rId28" ref="E24"/>
+    <hyperlink r:id="rId29" ref="C25"/>
+    <hyperlink r:id="rId30" ref="C26"/>
+    <hyperlink r:id="rId31" ref="C27"/>
+    <hyperlink r:id="rId32" ref="C28"/>
+    <hyperlink r:id="rId33" ref="C29"/>
+    <hyperlink r:id="rId34" ref="C30"/>
+    <hyperlink r:id="rId35" ref="C31"/>
+    <hyperlink r:id="rId36" ref="C32"/>
+    <hyperlink r:id="rId37" ref="C33"/>
+    <hyperlink r:id="rId38" ref="C34"/>
+    <hyperlink r:id="rId39" ref="C35"/>
+    <hyperlink r:id="rId40" ref="C36"/>
+    <hyperlink r:id="rId41" ref="C37"/>
+    <hyperlink r:id="rId42" ref="C38"/>
+    <hyperlink r:id="rId43" ref="C39"/>
+    <hyperlink r:id="rId44" ref="C40"/>
+    <hyperlink r:id="rId45" ref="C41"/>
+    <hyperlink r:id="rId46" ref="C42"/>
+    <hyperlink r:id="rId47" ref="C43"/>
+    <hyperlink r:id="rId48" ref="C44"/>
+    <hyperlink r:id="rId49" ref="C45"/>
+    <hyperlink r:id="rId50" ref="C46"/>
+    <hyperlink r:id="rId51" ref="C47"/>
+    <hyperlink r:id="rId52" ref="C48"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId51"/>
+  <drawing r:id="rId53"/>
 </worksheet>
 </file>
 
@@ -2577,216 +2595,216 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="4" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="J2" s="5">
+      <c r="J2" s="6">
         <v>6.0</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="J4" s="5">
+      <c r="J4" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6" s="6">
         <v>2.0</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="J8" s="5">
+      <c r="J8" s="6">
         <v>1.0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J14" s="5">
+      <c r="J14" s="6">
         <v>2.0</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="J15" s="5">
+      <c r="J15" s="6">
         <v>2.0</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="s">
+      <c r="A17" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="I17" s="5" t="s">
+      <c r="I17" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="J17" s="5">
+      <c r="J17" s="6">
         <v>3.0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="s">
+      <c r="A18" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="I18" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="6">
         <v>2.0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>147</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add entrenamiento hasta 24-04 correg
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="149">
   <si>
     <t>https://youtu.be/_8Jx9h36Sp8</t>
   </si>
@@ -417,6 +417,9 @@
   </si>
   <si>
     <t>Cambios de orientacion - Centros y Definicion</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_8Jx9h36Sp8</t>
   </si>
   <si>
     <t>3ER TURNO- 3:00 P.M</t>
@@ -1554,14 +1557,14 @@
       <c r="A48" s="13">
         <v>46136.0</v>
       </c>
-      <c r="C48" s="7" t="s">
-        <v>0</v>
+      <c r="C48" s="19" t="s">
+        <v>115</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1"/>
@@ -2596,18 +2599,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J2" s="6">
         <v>6.0</v>
@@ -2615,13 +2618,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J3" s="6">
         <v>1.0</v>
@@ -2629,13 +2632,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J4" s="6">
         <v>1.0</v>
@@ -2643,21 +2646,21 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="J6" s="6">
         <v>2.0</v>
@@ -2665,13 +2668,13 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J7" s="6">
         <v>1.0</v>
@@ -2679,13 +2682,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J8" s="6">
         <v>1.0</v>
@@ -2693,42 +2696,42 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J14" s="6">
         <v>2.0</v>
@@ -2736,13 +2739,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J15" s="6">
         <v>2.0</v>
@@ -2750,21 +2753,21 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J17" s="6">
         <v>3.0</v>
@@ -2772,13 +2775,13 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="J18" s="6">
         <v>2.0</v>
@@ -2786,26 +2789,26 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 24-04 corregir
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -10,16 +10,16 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="hei4pOW1qlb/hUfW6D3P3iKZbMqCsgEoQXCCdosrhzU="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="dkY05cCPST3br7bT/fI0DYKAB5OCJ/Rx3XvbzAtHjok="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="146">
-  <si>
-    <t>https://youtu.be/_8Jx9h36Sp8</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="149">
+  <si>
+    <t>date</t>
   </si>
   <si>
     <t>parte_entreno</t>
@@ -419,6 +419,21 @@
     <t>Cambios de orientacion - Centros y Definicion</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>3er Turno 24 04 2026</t>
+    </r>
+  </si>
+  <si>
+    <t>3ER TURNO- 3:00 P.M</t>
+  </si>
+  <si>
+    <t>Juego 11 VS 11</t>
+  </si>
+  <si>
     <t>VERDE</t>
   </si>
   <si>
@@ -530,9 +545,8 @@
     </font>
     <font>
       <b/>
-      <u/>
       <sz val="11.0"/>
-      <color theme="1"/>
+      <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1544,7 +1558,20 @@
         <v>114</v>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="13">
+        <v>46136.0</v>
+      </c>
+      <c r="C48" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
@@ -2502,59 +2529,60 @@
     <row r="1003" ht="15.75" customHeight="1"/>
     <row r="1004" ht="15.75" customHeight="1"/>
     <row r="1005" ht="15.75" customHeight="1"/>
+    <row r="1006" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="A1"/>
-    <hyperlink r:id="rId2" ref="C2"/>
-    <hyperlink r:id="rId3" ref="C3"/>
-    <hyperlink r:id="rId4" ref="C4"/>
-    <hyperlink r:id="rId5" ref="C5"/>
-    <hyperlink r:id="rId6" ref="C6"/>
-    <hyperlink r:id="rId7" ref="C7"/>
-    <hyperlink r:id="rId8" ref="C8"/>
-    <hyperlink r:id="rId9" ref="C9"/>
-    <hyperlink r:id="rId10" ref="C10"/>
-    <hyperlink r:id="rId11" ref="E10"/>
-    <hyperlink r:id="rId12" ref="C11"/>
-    <hyperlink r:id="rId13" ref="C12"/>
-    <hyperlink r:id="rId14" ref="E12"/>
-    <hyperlink r:id="rId15" ref="C13"/>
-    <hyperlink r:id="rId16" ref="E13"/>
-    <hyperlink r:id="rId17" ref="C14"/>
-    <hyperlink r:id="rId18" ref="C15"/>
-    <hyperlink r:id="rId19" ref="C16"/>
-    <hyperlink r:id="rId20" ref="C17"/>
-    <hyperlink r:id="rId21" ref="C18"/>
-    <hyperlink r:id="rId22" ref="C19"/>
-    <hyperlink r:id="rId23" ref="C20"/>
-    <hyperlink r:id="rId24" ref="C21"/>
-    <hyperlink r:id="rId25" ref="C22"/>
-    <hyperlink r:id="rId26" ref="C23"/>
-    <hyperlink r:id="rId27" ref="C24"/>
-    <hyperlink r:id="rId28" ref="E24"/>
-    <hyperlink r:id="rId29" ref="C25"/>
-    <hyperlink r:id="rId30" ref="C26"/>
-    <hyperlink r:id="rId31" ref="C27"/>
-    <hyperlink r:id="rId32" ref="C28"/>
-    <hyperlink r:id="rId33" ref="C29"/>
-    <hyperlink r:id="rId34" ref="C30"/>
-    <hyperlink r:id="rId35" ref="C31"/>
-    <hyperlink r:id="rId36" ref="C32"/>
-    <hyperlink r:id="rId37" ref="C33"/>
-    <hyperlink r:id="rId38" ref="C34"/>
-    <hyperlink r:id="rId39" ref="C35"/>
-    <hyperlink r:id="rId40" ref="C36"/>
-    <hyperlink r:id="rId41" ref="C37"/>
-    <hyperlink r:id="rId42" ref="C38"/>
-    <hyperlink r:id="rId43" ref="C39"/>
-    <hyperlink r:id="rId44" ref="C40"/>
-    <hyperlink r:id="rId45" ref="C41"/>
-    <hyperlink r:id="rId46" ref="C42"/>
-    <hyperlink r:id="rId47" ref="C43"/>
-    <hyperlink r:id="rId48" ref="C44"/>
-    <hyperlink r:id="rId49" ref="C45"/>
-    <hyperlink r:id="rId50" ref="C46"/>
-    <hyperlink r:id="rId51" ref="C47"/>
+    <hyperlink r:id="rId1" ref="C2"/>
+    <hyperlink r:id="rId2" ref="C3"/>
+    <hyperlink r:id="rId3" ref="C4"/>
+    <hyperlink r:id="rId4" ref="C5"/>
+    <hyperlink r:id="rId5" ref="C6"/>
+    <hyperlink r:id="rId6" ref="C7"/>
+    <hyperlink r:id="rId7" ref="C8"/>
+    <hyperlink r:id="rId8" ref="C9"/>
+    <hyperlink r:id="rId9" ref="C10"/>
+    <hyperlink r:id="rId10" ref="E10"/>
+    <hyperlink r:id="rId11" ref="C11"/>
+    <hyperlink r:id="rId12" ref="C12"/>
+    <hyperlink r:id="rId13" ref="E12"/>
+    <hyperlink r:id="rId14" ref="C13"/>
+    <hyperlink r:id="rId15" ref="E13"/>
+    <hyperlink r:id="rId16" ref="C14"/>
+    <hyperlink r:id="rId17" ref="C15"/>
+    <hyperlink r:id="rId18" ref="C16"/>
+    <hyperlink r:id="rId19" ref="C17"/>
+    <hyperlink r:id="rId20" ref="C18"/>
+    <hyperlink r:id="rId21" ref="C19"/>
+    <hyperlink r:id="rId22" ref="C20"/>
+    <hyperlink r:id="rId23" ref="C21"/>
+    <hyperlink r:id="rId24" ref="C22"/>
+    <hyperlink r:id="rId25" ref="C23"/>
+    <hyperlink r:id="rId26" ref="C24"/>
+    <hyperlink r:id="rId27" ref="E24"/>
+    <hyperlink r:id="rId28" ref="C25"/>
+    <hyperlink r:id="rId29" ref="C26"/>
+    <hyperlink r:id="rId30" ref="C27"/>
+    <hyperlink r:id="rId31" ref="C28"/>
+    <hyperlink r:id="rId32" ref="C29"/>
+    <hyperlink r:id="rId33" ref="C30"/>
+    <hyperlink r:id="rId34" ref="C31"/>
+    <hyperlink r:id="rId35" ref="C32"/>
+    <hyperlink r:id="rId36" ref="C33"/>
+    <hyperlink r:id="rId37" ref="C34"/>
+    <hyperlink r:id="rId38" ref="C35"/>
+    <hyperlink r:id="rId39" ref="C36"/>
+    <hyperlink r:id="rId40" ref="C37"/>
+    <hyperlink r:id="rId41" ref="C38"/>
+    <hyperlink r:id="rId42" ref="C39"/>
+    <hyperlink r:id="rId43" ref="C40"/>
+    <hyperlink r:id="rId44" ref="C41"/>
+    <hyperlink r:id="rId45" ref="C42"/>
+    <hyperlink r:id="rId46" ref="C43"/>
+    <hyperlink r:id="rId47" ref="C44"/>
+    <hyperlink r:id="rId48" ref="C45"/>
+    <hyperlink r:id="rId49" ref="C46"/>
+    <hyperlink r:id="rId50" ref="C47"/>
+    <hyperlink r:id="rId51" ref="C48"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
@@ -2575,18 +2603,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J2" s="6">
         <v>6.0</v>
@@ -2594,13 +2622,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="J3" s="6">
         <v>1.0</v>
@@ -2608,13 +2636,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="J4" s="6">
         <v>1.0</v>
@@ -2622,21 +2650,21 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="I6" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>124</v>
       </c>
       <c r="J6" s="6">
         <v>2.0</v>
@@ -2644,13 +2672,13 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="J7" s="6">
         <v>1.0</v>
@@ -2658,13 +2686,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J8" s="6">
         <v>1.0</v>
@@ -2672,42 +2700,42 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="J14" s="6">
         <v>2.0</v>
@@ -2715,13 +2743,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J15" s="6">
         <v>2.0</v>
@@ -2729,21 +2757,21 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="J17" s="6">
         <v>3.0</v>
@@ -2751,13 +2779,13 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="J18" s="6">
         <v>2.0</v>
@@ -2765,26 +2793,26 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 24-04 corregir2
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -419,13 +419,7 @@
     <t>Cambios de orientacion - Centros y Definicion</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <color rgb="FF1155CC"/>
-        <u/>
-      </rPr>
-      <t>3er Turno 24 04 2026</t>
-    </r>
+    <t>https://www.youtube.com/watch?v=_8Jx9h36Sp8</t>
   </si>
   <si>
     <t>3ER TURNO- 3:00 P.M</t>

</xml_diff>

<commit_message>
add entrenamiento hasta 26-04
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="157">
   <si>
     <t>date</t>
   </si>
@@ -426,6 +426,30 @@
   </si>
   <si>
     <t>Juego 11 VS 11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/lqXWQO7BcHI</t>
+  </si>
+  <si>
+    <t>Turno único 10:00 am</t>
+  </si>
+  <si>
+    <t>https://youtu.be/pn7qxeSxgVc</t>
+  </si>
+  <si>
+    <t>Turno único 8am</t>
+  </si>
+  <si>
+    <t>Porteros</t>
+  </si>
+  <si>
+    <t>https://youtu.be/05XeMi_68Mo</t>
+  </si>
+  <si>
+    <t>Cambios de orientación, centros y definición</t>
+  </si>
+  <si>
+    <t>https://youtu.be/KHLU3IBqzs4</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -1566,10 +1590,62 @@
         <v>117</v>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1"/>
-    <row r="50" ht="15.75" customHeight="1"/>
-    <row r="51" ht="15.75" customHeight="1"/>
-    <row r="52" ht="15.75" customHeight="1"/>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" s="13">
+        <v>46137.0</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="13">
+        <v>46138.0</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="A51" s="13">
+        <v>46138.0</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="A52" s="13">
+        <v>46138.0</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
     <row r="53" ht="15.75" customHeight="1"/>
     <row r="54" ht="15.75" customHeight="1"/>
     <row r="55" ht="15.75" customHeight="1"/>
@@ -2577,11 +2653,15 @@
     <hyperlink r:id="rId49" ref="C46"/>
     <hyperlink r:id="rId50" ref="C47"/>
     <hyperlink r:id="rId51" ref="C48"/>
+    <hyperlink r:id="rId52" ref="C49"/>
+    <hyperlink r:id="rId53" ref="C50"/>
+    <hyperlink r:id="rId54" ref="C51"/>
+    <hyperlink r:id="rId55" ref="C52"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId52"/>
+  <drawing r:id="rId56"/>
 </worksheet>
 </file>
 
@@ -2597,18 +2677,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J2" s="6">
         <v>6.0</v>
@@ -2616,13 +2696,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="J3" s="6">
         <v>1.0</v>
@@ -2630,13 +2710,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J4" s="6">
         <v>1.0</v>
@@ -2644,21 +2724,21 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="J6" s="6">
         <v>2.0</v>
@@ -2666,13 +2746,13 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>124</v>
       </c>
       <c r="J7" s="6">
         <v>1.0</v>
@@ -2680,13 +2760,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J8" s="6">
         <v>1.0</v>
@@ -2694,42 +2774,42 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="J14" s="6">
         <v>2.0</v>
@@ -2737,13 +2817,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="J15" s="6">
         <v>2.0</v>
@@ -2751,21 +2831,21 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>129</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>121</v>
       </c>
       <c r="J17" s="6">
         <v>3.0</v>
@@ -2773,13 +2853,13 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="J18" s="6">
         <v>2.0</v>
@@ -2787,26 +2867,26 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 01-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -4,22 +4,23 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Hoja1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Hoja x" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="Copia de Hoja1" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="Hoja x" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="dkY05cCPST3br7bT/fI0DYKAB5OCJ/Rx3XvbzAtHjok="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="nVGqFylxOMnrMPQ+QhULhUoor+EoekNxf7YmYmFKK2k="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="157">
-  <si>
-    <t>date</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="169">
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>parte_entreno</t>
@@ -450,6 +451,71 @@
   </si>
   <si>
     <t>https://youtu.be/KHLU3IBqzs4</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ppDobsGo3Yg</t>
+  </si>
+  <si>
+    <t>Turno Unico 3pm</t>
+  </si>
+  <si>
+    <t>Entrenamiento de resistencia, rueda de pases, juego de posesion</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Hod9nJ9w4gM</t>
+  </si>
+  <si>
+    <t>Amistoso vs Real Católica</t>
+  </si>
+  <si>
+    <t>Partido Amistoso VS Catolica</t>
+  </si>
+  <si>
+    <t>https://youtu.be/O_RFkTcApiY</t>
+  </si>
+  <si>
+    <t>1re Turno  09:00 am</t>
+  </si>
+  <si>
+    <t>Trabajo de Fuerza, Juego de Centros y Transiciones D-A , A-D</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>VERDE</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">: 8 de 12 veces terminó la jugada (6 por derecha, 1 por el medio y 1 por la izquierda). 4 pérdidas en zona baja (2 por el medio, 1 izq. 1 derecha). </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>NARANJA</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+      </rPr>
+      <t>: 4 de 9 veces terminó la jugada (2 izq. y 2 derecha) y un gol marcado. 5 pérdidas (3 por derecha y 2 por izquierda)</t>
+    </r>
+  </si>
+  <si>
+    <t>Turno unico 3pm</t>
+  </si>
+  <si>
+    <t>Juego de Patrones, Juego a 11 dirigido</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -720,6 +786,10 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -1646,11 +1716,1852 @@
         <v>18</v>
       </c>
     </row>
-    <row r="53" ht="15.75" customHeight="1"/>
-    <row r="54" ht="15.75" customHeight="1"/>
-    <row r="55" ht="15.75" customHeight="1"/>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="13">
+        <v>46140.0</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="A54" s="13">
+        <v>46113.0</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="A55" s="13">
+        <v>46146.0</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
     <row r="56" ht="15.75" customHeight="1"/>
     <row r="57" ht="15.75" customHeight="1"/>
+    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1"/>
+    <row r="60" ht="15.75" customHeight="1"/>
+    <row r="61" ht="15.75" customHeight="1"/>
+    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="63" ht="15.75" customHeight="1"/>
+    <row r="64" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="70" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="72" ht="15.75" customHeight="1"/>
+    <row r="73" ht="15.75" customHeight="1"/>
+    <row r="74" ht="15.75" customHeight="1"/>
+    <row r="75" ht="15.75" customHeight="1"/>
+    <row r="76" ht="15.75" customHeight="1"/>
+    <row r="77" ht="15.75" customHeight="1"/>
+    <row r="78" ht="15.75" customHeight="1"/>
+    <row r="79" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1"/>
+    <row r="81" ht="15.75" customHeight="1"/>
+    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1"/>
+    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1"/>
+    <row r="86" ht="15.75" customHeight="1"/>
+    <row r="87" ht="15.75" customHeight="1"/>
+    <row r="88" ht="15.75" customHeight="1"/>
+    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="90" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1"/>
+    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1"/>
+    <row r="94" ht="15.75" customHeight="1"/>
+    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1"/>
+    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1"/>
+    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1"/>
+    <row r="101" ht="15.75" customHeight="1"/>
+    <row r="102" ht="15.75" customHeight="1"/>
+    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1"/>
+    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1"/>
+    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1"/>
+    <row r="109" ht="15.75" customHeight="1"/>
+    <row r="110" ht="15.75" customHeight="1"/>
+    <row r="111" ht="15.75" customHeight="1"/>
+    <row r="112" ht="15.75" customHeight="1"/>
+    <row r="113" ht="15.75" customHeight="1"/>
+    <row r="114" ht="15.75" customHeight="1"/>
+    <row r="115" ht="15.75" customHeight="1"/>
+    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="117" ht="15.75" customHeight="1"/>
+    <row r="118" ht="15.75" customHeight="1"/>
+    <row r="119" ht="15.75" customHeight="1"/>
+    <row r="120" ht="15.75" customHeight="1"/>
+    <row r="121" ht="15.75" customHeight="1"/>
+    <row r="122" ht="15.75" customHeight="1"/>
+    <row r="123" ht="15.75" customHeight="1"/>
+    <row r="124" ht="15.75" customHeight="1"/>
+    <row r="125" ht="15.75" customHeight="1"/>
+    <row r="126" ht="15.75" customHeight="1"/>
+    <row r="127" ht="15.75" customHeight="1"/>
+    <row r="128" ht="15.75" customHeight="1"/>
+    <row r="129" ht="15.75" customHeight="1"/>
+    <row r="130" ht="15.75" customHeight="1"/>
+    <row r="131" ht="15.75" customHeight="1"/>
+    <row r="132" ht="15.75" customHeight="1"/>
+    <row r="133" ht="15.75" customHeight="1"/>
+    <row r="134" ht="15.75" customHeight="1"/>
+    <row r="135" ht="15.75" customHeight="1"/>
+    <row r="136" ht="15.75" customHeight="1"/>
+    <row r="137" ht="15.75" customHeight="1"/>
+    <row r="138" ht="15.75" customHeight="1"/>
+    <row r="139" ht="15.75" customHeight="1"/>
+    <row r="140" ht="15.75" customHeight="1"/>
+    <row r="141" ht="15.75" customHeight="1"/>
+    <row r="142" ht="15.75" customHeight="1"/>
+    <row r="143" ht="15.75" customHeight="1"/>
+    <row r="144" ht="15.75" customHeight="1"/>
+    <row r="145" ht="15.75" customHeight="1"/>
+    <row r="146" ht="15.75" customHeight="1"/>
+    <row r="147" ht="15.75" customHeight="1"/>
+    <row r="148" ht="15.75" customHeight="1"/>
+    <row r="149" ht="15.75" customHeight="1"/>
+    <row r="150" ht="15.75" customHeight="1"/>
+    <row r="151" ht="15.75" customHeight="1"/>
+    <row r="152" ht="15.75" customHeight="1"/>
+    <row r="153" ht="15.75" customHeight="1"/>
+    <row r="154" ht="15.75" customHeight="1"/>
+    <row r="155" ht="15.75" customHeight="1"/>
+    <row r="156" ht="15.75" customHeight="1"/>
+    <row r="157" ht="15.75" customHeight="1"/>
+    <row r="158" ht="15.75" customHeight="1"/>
+    <row r="159" ht="15.75" customHeight="1"/>
+    <row r="160" ht="15.75" customHeight="1"/>
+    <row r="161" ht="15.75" customHeight="1"/>
+    <row r="162" ht="15.75" customHeight="1"/>
+    <row r="163" ht="15.75" customHeight="1"/>
+    <row r="164" ht="15.75" customHeight="1"/>
+    <row r="165" ht="15.75" customHeight="1"/>
+    <row r="166" ht="15.75" customHeight="1"/>
+    <row r="167" ht="15.75" customHeight="1"/>
+    <row r="168" ht="15.75" customHeight="1"/>
+    <row r="169" ht="15.75" customHeight="1"/>
+    <row r="170" ht="15.75" customHeight="1"/>
+    <row r="171" ht="15.75" customHeight="1"/>
+    <row r="172" ht="15.75" customHeight="1"/>
+    <row r="173" ht="15.75" customHeight="1"/>
+    <row r="174" ht="15.75" customHeight="1"/>
+    <row r="175" ht="15.75" customHeight="1"/>
+    <row r="176" ht="15.75" customHeight="1"/>
+    <row r="177" ht="15.75" customHeight="1"/>
+    <row r="178" ht="15.75" customHeight="1"/>
+    <row r="179" ht="15.75" customHeight="1"/>
+    <row r="180" ht="15.75" customHeight="1"/>
+    <row r="181" ht="15.75" customHeight="1"/>
+    <row r="182" ht="15.75" customHeight="1"/>
+    <row r="183" ht="15.75" customHeight="1"/>
+    <row r="184" ht="15.75" customHeight="1"/>
+    <row r="185" ht="15.75" customHeight="1"/>
+    <row r="186" ht="15.75" customHeight="1"/>
+    <row r="187" ht="15.75" customHeight="1"/>
+    <row r="188" ht="15.75" customHeight="1"/>
+    <row r="189" ht="15.75" customHeight="1"/>
+    <row r="190" ht="15.75" customHeight="1"/>
+    <row r="191" ht="15.75" customHeight="1"/>
+    <row r="192" ht="15.75" customHeight="1"/>
+    <row r="193" ht="15.75" customHeight="1"/>
+    <row r="194" ht="15.75" customHeight="1"/>
+    <row r="195" ht="15.75" customHeight="1"/>
+    <row r="196" ht="15.75" customHeight="1"/>
+    <row r="197" ht="15.75" customHeight="1"/>
+    <row r="198" ht="15.75" customHeight="1"/>
+    <row r="199" ht="15.75" customHeight="1"/>
+    <row r="200" ht="15.75" customHeight="1"/>
+    <row r="201" ht="15.75" customHeight="1"/>
+    <row r="202" ht="15.75" customHeight="1"/>
+    <row r="203" ht="15.75" customHeight="1"/>
+    <row r="204" ht="15.75" customHeight="1"/>
+    <row r="205" ht="15.75" customHeight="1"/>
+    <row r="206" ht="15.75" customHeight="1"/>
+    <row r="207" ht="15.75" customHeight="1"/>
+    <row r="208" ht="15.75" customHeight="1"/>
+    <row r="209" ht="15.75" customHeight="1"/>
+    <row r="210" ht="15.75" customHeight="1"/>
+    <row r="211" ht="15.75" customHeight="1"/>
+    <row r="212" ht="15.75" customHeight="1"/>
+    <row r="213" ht="15.75" customHeight="1"/>
+    <row r="214" ht="15.75" customHeight="1"/>
+    <row r="215" ht="15.75" customHeight="1"/>
+    <row r="216" ht="15.75" customHeight="1"/>
+    <row r="217" ht="15.75" customHeight="1"/>
+    <row r="218" ht="15.75" customHeight="1"/>
+    <row r="219" ht="15.75" customHeight="1"/>
+    <row r="220" ht="15.75" customHeight="1"/>
+    <row r="221" ht="15.75" customHeight="1"/>
+    <row r="222" ht="15.75" customHeight="1"/>
+    <row r="223" ht="15.75" customHeight="1"/>
+    <row r="224" ht="15.75" customHeight="1"/>
+    <row r="225" ht="15.75" customHeight="1"/>
+    <row r="226" ht="15.75" customHeight="1"/>
+    <row r="227" ht="15.75" customHeight="1"/>
+    <row r="228" ht="15.75" customHeight="1"/>
+    <row r="229" ht="15.75" customHeight="1"/>
+    <row r="230" ht="15.75" customHeight="1"/>
+    <row r="231" ht="15.75" customHeight="1"/>
+    <row r="232" ht="15.75" customHeight="1"/>
+    <row r="233" ht="15.75" customHeight="1"/>
+    <row r="234" ht="15.75" customHeight="1"/>
+    <row r="235" ht="15.75" customHeight="1"/>
+    <row r="236" ht="15.75" customHeight="1"/>
+    <row r="237" ht="15.75" customHeight="1"/>
+    <row r="238" ht="15.75" customHeight="1"/>
+    <row r="239" ht="15.75" customHeight="1"/>
+    <row r="240" ht="15.75" customHeight="1"/>
+    <row r="241" ht="15.75" customHeight="1"/>
+    <row r="242" ht="15.75" customHeight="1"/>
+    <row r="243" ht="15.75" customHeight="1"/>
+    <row r="244" ht="15.75" customHeight="1"/>
+    <row r="245" ht="15.75" customHeight="1"/>
+    <row r="246" ht="15.75" customHeight="1"/>
+    <row r="247" ht="15.75" customHeight="1"/>
+    <row r="248" ht="15.75" customHeight="1"/>
+    <row r="249" ht="15.75" customHeight="1"/>
+    <row r="250" ht="15.75" customHeight="1"/>
+    <row r="251" ht="15.75" customHeight="1"/>
+    <row r="252" ht="15.75" customHeight="1"/>
+    <row r="253" ht="15.75" customHeight="1"/>
+    <row r="254" ht="15.75" customHeight="1"/>
+    <row r="255" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="258" ht="15.75" customHeight="1"/>
+    <row r="259" ht="15.75" customHeight="1"/>
+    <row r="260" ht="15.75" customHeight="1"/>
+    <row r="261" ht="15.75" customHeight="1"/>
+    <row r="262" ht="15.75" customHeight="1"/>
+    <row r="263" ht="15.75" customHeight="1"/>
+    <row r="264" ht="15.75" customHeight="1"/>
+    <row r="265" ht="15.75" customHeight="1"/>
+    <row r="266" ht="15.75" customHeight="1"/>
+    <row r="267" ht="15.75" customHeight="1"/>
+    <row r="268" ht="15.75" customHeight="1"/>
+    <row r="269" ht="15.75" customHeight="1"/>
+    <row r="270" ht="15.75" customHeight="1"/>
+    <row r="271" ht="15.75" customHeight="1"/>
+    <row r="272" ht="15.75" customHeight="1"/>
+    <row r="273" ht="15.75" customHeight="1"/>
+    <row r="274" ht="15.75" customHeight="1"/>
+    <row r="275" ht="15.75" customHeight="1"/>
+    <row r="276" ht="15.75" customHeight="1"/>
+    <row r="277" ht="15.75" customHeight="1"/>
+    <row r="278" ht="15.75" customHeight="1"/>
+    <row r="279" ht="15.75" customHeight="1"/>
+    <row r="280" ht="15.75" customHeight="1"/>
+    <row r="281" ht="15.75" customHeight="1"/>
+    <row r="282" ht="15.75" customHeight="1"/>
+    <row r="283" ht="15.75" customHeight="1"/>
+    <row r="284" ht="15.75" customHeight="1"/>
+    <row r="285" ht="15.75" customHeight="1"/>
+    <row r="286" ht="15.75" customHeight="1"/>
+    <row r="287" ht="15.75" customHeight="1"/>
+    <row r="288" ht="15.75" customHeight="1"/>
+    <row r="289" ht="15.75" customHeight="1"/>
+    <row r="290" ht="15.75" customHeight="1"/>
+    <row r="291" ht="15.75" customHeight="1"/>
+    <row r="292" ht="15.75" customHeight="1"/>
+    <row r="293" ht="15.75" customHeight="1"/>
+    <row r="294" ht="15.75" customHeight="1"/>
+    <row r="295" ht="15.75" customHeight="1"/>
+    <row r="296" ht="15.75" customHeight="1"/>
+    <row r="297" ht="15.75" customHeight="1"/>
+    <row r="298" ht="15.75" customHeight="1"/>
+    <row r="299" ht="15.75" customHeight="1"/>
+    <row r="300" ht="15.75" customHeight="1"/>
+    <row r="301" ht="15.75" customHeight="1"/>
+    <row r="302" ht="15.75" customHeight="1"/>
+    <row r="303" ht="15.75" customHeight="1"/>
+    <row r="304" ht="15.75" customHeight="1"/>
+    <row r="305" ht="15.75" customHeight="1"/>
+    <row r="306" ht="15.75" customHeight="1"/>
+    <row r="307" ht="15.75" customHeight="1"/>
+    <row r="308" ht="15.75" customHeight="1"/>
+    <row r="309" ht="15.75" customHeight="1"/>
+    <row r="310" ht="15.75" customHeight="1"/>
+    <row r="311" ht="15.75" customHeight="1"/>
+    <row r="312" ht="15.75" customHeight="1"/>
+    <row r="313" ht="15.75" customHeight="1"/>
+    <row r="314" ht="15.75" customHeight="1"/>
+    <row r="315" ht="15.75" customHeight="1"/>
+    <row r="316" ht="15.75" customHeight="1"/>
+    <row r="317" ht="15.75" customHeight="1"/>
+    <row r="318" ht="15.75" customHeight="1"/>
+    <row r="319" ht="15.75" customHeight="1"/>
+    <row r="320" ht="15.75" customHeight="1"/>
+    <row r="321" ht="15.75" customHeight="1"/>
+    <row r="322" ht="15.75" customHeight="1"/>
+    <row r="323" ht="15.75" customHeight="1"/>
+    <row r="324" ht="15.75" customHeight="1"/>
+    <row r="325" ht="15.75" customHeight="1"/>
+    <row r="326" ht="15.75" customHeight="1"/>
+    <row r="327" ht="15.75" customHeight="1"/>
+    <row r="328" ht="15.75" customHeight="1"/>
+    <row r="329" ht="15.75" customHeight="1"/>
+    <row r="330" ht="15.75" customHeight="1"/>
+    <row r="331" ht="15.75" customHeight="1"/>
+    <row r="332" ht="15.75" customHeight="1"/>
+    <row r="333" ht="15.75" customHeight="1"/>
+    <row r="334" ht="15.75" customHeight="1"/>
+    <row r="335" ht="15.75" customHeight="1"/>
+    <row r="336" ht="15.75" customHeight="1"/>
+    <row r="337" ht="15.75" customHeight="1"/>
+    <row r="338" ht="15.75" customHeight="1"/>
+    <row r="339" ht="15.75" customHeight="1"/>
+    <row r="340" ht="15.75" customHeight="1"/>
+    <row r="341" ht="15.75" customHeight="1"/>
+    <row r="342" ht="15.75" customHeight="1"/>
+    <row r="343" ht="15.75" customHeight="1"/>
+    <row r="344" ht="15.75" customHeight="1"/>
+    <row r="345" ht="15.75" customHeight="1"/>
+    <row r="346" ht="15.75" customHeight="1"/>
+    <row r="347" ht="15.75" customHeight="1"/>
+    <row r="348" ht="15.75" customHeight="1"/>
+    <row r="349" ht="15.75" customHeight="1"/>
+    <row r="350" ht="15.75" customHeight="1"/>
+    <row r="351" ht="15.75" customHeight="1"/>
+    <row r="352" ht="15.75" customHeight="1"/>
+    <row r="353" ht="15.75" customHeight="1"/>
+    <row r="354" ht="15.75" customHeight="1"/>
+    <row r="355" ht="15.75" customHeight="1"/>
+    <row r="356" ht="15.75" customHeight="1"/>
+    <row r="357" ht="15.75" customHeight="1"/>
+    <row r="358" ht="15.75" customHeight="1"/>
+    <row r="359" ht="15.75" customHeight="1"/>
+    <row r="360" ht="15.75" customHeight="1"/>
+    <row r="361" ht="15.75" customHeight="1"/>
+    <row r="362" ht="15.75" customHeight="1"/>
+    <row r="363" ht="15.75" customHeight="1"/>
+    <row r="364" ht="15.75" customHeight="1"/>
+    <row r="365" ht="15.75" customHeight="1"/>
+    <row r="366" ht="15.75" customHeight="1"/>
+    <row r="367" ht="15.75" customHeight="1"/>
+    <row r="368" ht="15.75" customHeight="1"/>
+    <row r="369" ht="15.75" customHeight="1"/>
+    <row r="370" ht="15.75" customHeight="1"/>
+    <row r="371" ht="15.75" customHeight="1"/>
+    <row r="372" ht="15.75" customHeight="1"/>
+    <row r="373" ht="15.75" customHeight="1"/>
+    <row r="374" ht="15.75" customHeight="1"/>
+    <row r="375" ht="15.75" customHeight="1"/>
+    <row r="376" ht="15.75" customHeight="1"/>
+    <row r="377" ht="15.75" customHeight="1"/>
+    <row r="378" ht="15.75" customHeight="1"/>
+    <row r="379" ht="15.75" customHeight="1"/>
+    <row r="380" ht="15.75" customHeight="1"/>
+    <row r="381" ht="15.75" customHeight="1"/>
+    <row r="382" ht="15.75" customHeight="1"/>
+    <row r="383" ht="15.75" customHeight="1"/>
+    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="385" ht="15.75" customHeight="1"/>
+    <row r="386" ht="15.75" customHeight="1"/>
+    <row r="387" ht="15.75" customHeight="1"/>
+    <row r="388" ht="15.75" customHeight="1"/>
+    <row r="389" ht="15.75" customHeight="1"/>
+    <row r="390" ht="15.75" customHeight="1"/>
+    <row r="391" ht="15.75" customHeight="1"/>
+    <row r="392" ht="15.75" customHeight="1"/>
+    <row r="393" ht="15.75" customHeight="1"/>
+    <row r="394" ht="15.75" customHeight="1"/>
+    <row r="395" ht="15.75" customHeight="1"/>
+    <row r="396" ht="15.75" customHeight="1"/>
+    <row r="397" ht="15.75" customHeight="1"/>
+    <row r="398" ht="15.75" customHeight="1"/>
+    <row r="399" ht="15.75" customHeight="1"/>
+    <row r="400" ht="15.75" customHeight="1"/>
+    <row r="401" ht="15.75" customHeight="1"/>
+    <row r="402" ht="15.75" customHeight="1"/>
+    <row r="403" ht="15.75" customHeight="1"/>
+    <row r="404" ht="15.75" customHeight="1"/>
+    <row r="405" ht="15.75" customHeight="1"/>
+    <row r="406" ht="15.75" customHeight="1"/>
+    <row r="407" ht="15.75" customHeight="1"/>
+    <row r="408" ht="15.75" customHeight="1"/>
+    <row r="409" ht="15.75" customHeight="1"/>
+    <row r="410" ht="15.75" customHeight="1"/>
+    <row r="411" ht="15.75" customHeight="1"/>
+    <row r="412" ht="15.75" customHeight="1"/>
+    <row r="413" ht="15.75" customHeight="1"/>
+    <row r="414" ht="15.75" customHeight="1"/>
+    <row r="415" ht="15.75" customHeight="1"/>
+    <row r="416" ht="15.75" customHeight="1"/>
+    <row r="417" ht="15.75" customHeight="1"/>
+    <row r="418" ht="15.75" customHeight="1"/>
+    <row r="419" ht="15.75" customHeight="1"/>
+    <row r="420" ht="15.75" customHeight="1"/>
+    <row r="421" ht="15.75" customHeight="1"/>
+    <row r="422" ht="15.75" customHeight="1"/>
+    <row r="423" ht="15.75" customHeight="1"/>
+    <row r="424" ht="15.75" customHeight="1"/>
+    <row r="425" ht="15.75" customHeight="1"/>
+    <row r="426" ht="15.75" customHeight="1"/>
+    <row r="427" ht="15.75" customHeight="1"/>
+    <row r="428" ht="15.75" customHeight="1"/>
+    <row r="429" ht="15.75" customHeight="1"/>
+    <row r="430" ht="15.75" customHeight="1"/>
+    <row r="431" ht="15.75" customHeight="1"/>
+    <row r="432" ht="15.75" customHeight="1"/>
+    <row r="433" ht="15.75" customHeight="1"/>
+    <row r="434" ht="15.75" customHeight="1"/>
+    <row r="435" ht="15.75" customHeight="1"/>
+    <row r="436" ht="15.75" customHeight="1"/>
+    <row r="437" ht="15.75" customHeight="1"/>
+    <row r="438" ht="15.75" customHeight="1"/>
+    <row r="439" ht="15.75" customHeight="1"/>
+    <row r="440" ht="15.75" customHeight="1"/>
+    <row r="441" ht="15.75" customHeight="1"/>
+    <row r="442" ht="15.75" customHeight="1"/>
+    <row r="443" ht="15.75" customHeight="1"/>
+    <row r="444" ht="15.75" customHeight="1"/>
+    <row r="445" ht="15.75" customHeight="1"/>
+    <row r="446" ht="15.75" customHeight="1"/>
+    <row r="447" ht="15.75" customHeight="1"/>
+    <row r="448" ht="15.75" customHeight="1"/>
+    <row r="449" ht="15.75" customHeight="1"/>
+    <row r="450" ht="15.75" customHeight="1"/>
+    <row r="451" ht="15.75" customHeight="1"/>
+    <row r="452" ht="15.75" customHeight="1"/>
+    <row r="453" ht="15.75" customHeight="1"/>
+    <row r="454" ht="15.75" customHeight="1"/>
+    <row r="455" ht="15.75" customHeight="1"/>
+    <row r="456" ht="15.75" customHeight="1"/>
+    <row r="457" ht="15.75" customHeight="1"/>
+    <row r="458" ht="15.75" customHeight="1"/>
+    <row r="459" ht="15.75" customHeight="1"/>
+    <row r="460" ht="15.75" customHeight="1"/>
+    <row r="461" ht="15.75" customHeight="1"/>
+    <row r="462" ht="15.75" customHeight="1"/>
+    <row r="463" ht="15.75" customHeight="1"/>
+    <row r="464" ht="15.75" customHeight="1"/>
+    <row r="465" ht="15.75" customHeight="1"/>
+    <row r="466" ht="15.75" customHeight="1"/>
+    <row r="467" ht="15.75" customHeight="1"/>
+    <row r="468" ht="15.75" customHeight="1"/>
+    <row r="469" ht="15.75" customHeight="1"/>
+    <row r="470" ht="15.75" customHeight="1"/>
+    <row r="471" ht="15.75" customHeight="1"/>
+    <row r="472" ht="15.75" customHeight="1"/>
+    <row r="473" ht="15.75" customHeight="1"/>
+    <row r="474" ht="15.75" customHeight="1"/>
+    <row r="475" ht="15.75" customHeight="1"/>
+    <row r="476" ht="15.75" customHeight="1"/>
+    <row r="477" ht="15.75" customHeight="1"/>
+    <row r="478" ht="15.75" customHeight="1"/>
+    <row r="479" ht="15.75" customHeight="1"/>
+    <row r="480" ht="15.75" customHeight="1"/>
+    <row r="481" ht="15.75" customHeight="1"/>
+    <row r="482" ht="15.75" customHeight="1"/>
+    <row r="483" ht="15.75" customHeight="1"/>
+    <row r="484" ht="15.75" customHeight="1"/>
+    <row r="485" ht="15.75" customHeight="1"/>
+    <row r="486" ht="15.75" customHeight="1"/>
+    <row r="487" ht="15.75" customHeight="1"/>
+    <row r="488" ht="15.75" customHeight="1"/>
+    <row r="489" ht="15.75" customHeight="1"/>
+    <row r="490" ht="15.75" customHeight="1"/>
+    <row r="491" ht="15.75" customHeight="1"/>
+    <row r="492" ht="15.75" customHeight="1"/>
+    <row r="493" ht="15.75" customHeight="1"/>
+    <row r="494" ht="15.75" customHeight="1"/>
+    <row r="495" ht="15.75" customHeight="1"/>
+    <row r="496" ht="15.75" customHeight="1"/>
+    <row r="497" ht="15.75" customHeight="1"/>
+    <row r="498" ht="15.75" customHeight="1"/>
+    <row r="499" ht="15.75" customHeight="1"/>
+    <row r="500" ht="15.75" customHeight="1"/>
+    <row r="501" ht="15.75" customHeight="1"/>
+    <row r="502" ht="15.75" customHeight="1"/>
+    <row r="503" ht="15.75" customHeight="1"/>
+    <row r="504" ht="15.75" customHeight="1"/>
+    <row r="505" ht="15.75" customHeight="1"/>
+    <row r="506" ht="15.75" customHeight="1"/>
+    <row r="507" ht="15.75" customHeight="1"/>
+    <row r="508" ht="15.75" customHeight="1"/>
+    <row r="509" ht="15.75" customHeight="1"/>
+    <row r="510" ht="15.75" customHeight="1"/>
+    <row r="511" ht="15.75" customHeight="1"/>
+    <row r="512" ht="15.75" customHeight="1"/>
+    <row r="513" ht="15.75" customHeight="1"/>
+    <row r="514" ht="15.75" customHeight="1"/>
+    <row r="515" ht="15.75" customHeight="1"/>
+    <row r="516" ht="15.75" customHeight="1"/>
+    <row r="517" ht="15.75" customHeight="1"/>
+    <row r="518" ht="15.75" customHeight="1"/>
+    <row r="519" ht="15.75" customHeight="1"/>
+    <row r="520" ht="15.75" customHeight="1"/>
+    <row r="521" ht="15.75" customHeight="1"/>
+    <row r="522" ht="15.75" customHeight="1"/>
+    <row r="523" ht="15.75" customHeight="1"/>
+    <row r="524" ht="15.75" customHeight="1"/>
+    <row r="525" ht="15.75" customHeight="1"/>
+    <row r="526" ht="15.75" customHeight="1"/>
+    <row r="527" ht="15.75" customHeight="1"/>
+    <row r="528" ht="15.75" customHeight="1"/>
+    <row r="529" ht="15.75" customHeight="1"/>
+    <row r="530" ht="15.75" customHeight="1"/>
+    <row r="531" ht="15.75" customHeight="1"/>
+    <row r="532" ht="15.75" customHeight="1"/>
+    <row r="533" ht="15.75" customHeight="1"/>
+    <row r="534" ht="15.75" customHeight="1"/>
+    <row r="535" ht="15.75" customHeight="1"/>
+    <row r="536" ht="15.75" customHeight="1"/>
+    <row r="537" ht="15.75" customHeight="1"/>
+    <row r="538" ht="15.75" customHeight="1"/>
+    <row r="539" ht="15.75" customHeight="1"/>
+    <row r="540" ht="15.75" customHeight="1"/>
+    <row r="541" ht="15.75" customHeight="1"/>
+    <row r="542" ht="15.75" customHeight="1"/>
+    <row r="543" ht="15.75" customHeight="1"/>
+    <row r="544" ht="15.75" customHeight="1"/>
+    <row r="545" ht="15.75" customHeight="1"/>
+    <row r="546" ht="15.75" customHeight="1"/>
+    <row r="547" ht="15.75" customHeight="1"/>
+    <row r="548" ht="15.75" customHeight="1"/>
+    <row r="549" ht="15.75" customHeight="1"/>
+    <row r="550" ht="15.75" customHeight="1"/>
+    <row r="551" ht="15.75" customHeight="1"/>
+    <row r="552" ht="15.75" customHeight="1"/>
+    <row r="553" ht="15.75" customHeight="1"/>
+    <row r="554" ht="15.75" customHeight="1"/>
+    <row r="555" ht="15.75" customHeight="1"/>
+    <row r="556" ht="15.75" customHeight="1"/>
+    <row r="557" ht="15.75" customHeight="1"/>
+    <row r="558" ht="15.75" customHeight="1"/>
+    <row r="559" ht="15.75" customHeight="1"/>
+    <row r="560" ht="15.75" customHeight="1"/>
+    <row r="561" ht="15.75" customHeight="1"/>
+    <row r="562" ht="15.75" customHeight="1"/>
+    <row r="563" ht="15.75" customHeight="1"/>
+    <row r="564" ht="15.75" customHeight="1"/>
+    <row r="565" ht="15.75" customHeight="1"/>
+    <row r="566" ht="15.75" customHeight="1"/>
+    <row r="567" ht="15.75" customHeight="1"/>
+    <row r="568" ht="15.75" customHeight="1"/>
+    <row r="569" ht="15.75" customHeight="1"/>
+    <row r="570" ht="15.75" customHeight="1"/>
+    <row r="571" ht="15.75" customHeight="1"/>
+    <row r="572" ht="15.75" customHeight="1"/>
+    <row r="573" ht="15.75" customHeight="1"/>
+    <row r="574" ht="15.75" customHeight="1"/>
+    <row r="575" ht="15.75" customHeight="1"/>
+    <row r="576" ht="15.75" customHeight="1"/>
+    <row r="577" ht="15.75" customHeight="1"/>
+    <row r="578" ht="15.75" customHeight="1"/>
+    <row r="579" ht="15.75" customHeight="1"/>
+    <row r="580" ht="15.75" customHeight="1"/>
+    <row r="581" ht="15.75" customHeight="1"/>
+    <row r="582" ht="15.75" customHeight="1"/>
+    <row r="583" ht="15.75" customHeight="1"/>
+    <row r="584" ht="15.75" customHeight="1"/>
+    <row r="585" ht="15.75" customHeight="1"/>
+    <row r="586" ht="15.75" customHeight="1"/>
+    <row r="587" ht="15.75" customHeight="1"/>
+    <row r="588" ht="15.75" customHeight="1"/>
+    <row r="589" ht="15.75" customHeight="1"/>
+    <row r="590" ht="15.75" customHeight="1"/>
+    <row r="591" ht="15.75" customHeight="1"/>
+    <row r="592" ht="15.75" customHeight="1"/>
+    <row r="593" ht="15.75" customHeight="1"/>
+    <row r="594" ht="15.75" customHeight="1"/>
+    <row r="595" ht="15.75" customHeight="1"/>
+    <row r="596" ht="15.75" customHeight="1"/>
+    <row r="597" ht="15.75" customHeight="1"/>
+    <row r="598" ht="15.75" customHeight="1"/>
+    <row r="599" ht="15.75" customHeight="1"/>
+    <row r="600" ht="15.75" customHeight="1"/>
+    <row r="601" ht="15.75" customHeight="1"/>
+    <row r="602" ht="15.75" customHeight="1"/>
+    <row r="603" ht="15.75" customHeight="1"/>
+    <row r="604" ht="15.75" customHeight="1"/>
+    <row r="605" ht="15.75" customHeight="1"/>
+    <row r="606" ht="15.75" customHeight="1"/>
+    <row r="607" ht="15.75" customHeight="1"/>
+    <row r="608" ht="15.75" customHeight="1"/>
+    <row r="609" ht="15.75" customHeight="1"/>
+    <row r="610" ht="15.75" customHeight="1"/>
+    <row r="611" ht="15.75" customHeight="1"/>
+    <row r="612" ht="15.75" customHeight="1"/>
+    <row r="613" ht="15.75" customHeight="1"/>
+    <row r="614" ht="15.75" customHeight="1"/>
+    <row r="615" ht="15.75" customHeight="1"/>
+    <row r="616" ht="15.75" customHeight="1"/>
+    <row r="617" ht="15.75" customHeight="1"/>
+    <row r="618" ht="15.75" customHeight="1"/>
+    <row r="619" ht="15.75" customHeight="1"/>
+    <row r="620" ht="15.75" customHeight="1"/>
+    <row r="621" ht="15.75" customHeight="1"/>
+    <row r="622" ht="15.75" customHeight="1"/>
+    <row r="623" ht="15.75" customHeight="1"/>
+    <row r="624" ht="15.75" customHeight="1"/>
+    <row r="625" ht="15.75" customHeight="1"/>
+    <row r="626" ht="15.75" customHeight="1"/>
+    <row r="627" ht="15.75" customHeight="1"/>
+    <row r="628" ht="15.75" customHeight="1"/>
+    <row r="629" ht="15.75" customHeight="1"/>
+    <row r="630" ht="15.75" customHeight="1"/>
+    <row r="631" ht="15.75" customHeight="1"/>
+    <row r="632" ht="15.75" customHeight="1"/>
+    <row r="633" ht="15.75" customHeight="1"/>
+    <row r="634" ht="15.75" customHeight="1"/>
+    <row r="635" ht="15.75" customHeight="1"/>
+    <row r="636" ht="15.75" customHeight="1"/>
+    <row r="637" ht="15.75" customHeight="1"/>
+    <row r="638" ht="15.75" customHeight="1"/>
+    <row r="639" ht="15.75" customHeight="1"/>
+    <row r="640" ht="15.75" customHeight="1"/>
+    <row r="641" ht="15.75" customHeight="1"/>
+    <row r="642" ht="15.75" customHeight="1"/>
+    <row r="643" ht="15.75" customHeight="1"/>
+    <row r="644" ht="15.75" customHeight="1"/>
+    <row r="645" ht="15.75" customHeight="1"/>
+    <row r="646" ht="15.75" customHeight="1"/>
+    <row r="647" ht="15.75" customHeight="1"/>
+    <row r="648" ht="15.75" customHeight="1"/>
+    <row r="649" ht="15.75" customHeight="1"/>
+    <row r="650" ht="15.75" customHeight="1"/>
+    <row r="651" ht="15.75" customHeight="1"/>
+    <row r="652" ht="15.75" customHeight="1"/>
+    <row r="653" ht="15.75" customHeight="1"/>
+    <row r="654" ht="15.75" customHeight="1"/>
+    <row r="655" ht="15.75" customHeight="1"/>
+    <row r="656" ht="15.75" customHeight="1"/>
+    <row r="657" ht="15.75" customHeight="1"/>
+    <row r="658" ht="15.75" customHeight="1"/>
+    <row r="659" ht="15.75" customHeight="1"/>
+    <row r="660" ht="15.75" customHeight="1"/>
+    <row r="661" ht="15.75" customHeight="1"/>
+    <row r="662" ht="15.75" customHeight="1"/>
+    <row r="663" ht="15.75" customHeight="1"/>
+    <row r="664" ht="15.75" customHeight="1"/>
+    <row r="665" ht="15.75" customHeight="1"/>
+    <row r="666" ht="15.75" customHeight="1"/>
+    <row r="667" ht="15.75" customHeight="1"/>
+    <row r="668" ht="15.75" customHeight="1"/>
+    <row r="669" ht="15.75" customHeight="1"/>
+    <row r="670" ht="15.75" customHeight="1"/>
+    <row r="671" ht="15.75" customHeight="1"/>
+    <row r="672" ht="15.75" customHeight="1"/>
+    <row r="673" ht="15.75" customHeight="1"/>
+    <row r="674" ht="15.75" customHeight="1"/>
+    <row r="675" ht="15.75" customHeight="1"/>
+    <row r="676" ht="15.75" customHeight="1"/>
+    <row r="677" ht="15.75" customHeight="1"/>
+    <row r="678" ht="15.75" customHeight="1"/>
+    <row r="679" ht="15.75" customHeight="1"/>
+    <row r="680" ht="15.75" customHeight="1"/>
+    <row r="681" ht="15.75" customHeight="1"/>
+    <row r="682" ht="15.75" customHeight="1"/>
+    <row r="683" ht="15.75" customHeight="1"/>
+    <row r="684" ht="15.75" customHeight="1"/>
+    <row r="685" ht="15.75" customHeight="1"/>
+    <row r="686" ht="15.75" customHeight="1"/>
+    <row r="687" ht="15.75" customHeight="1"/>
+    <row r="688" ht="15.75" customHeight="1"/>
+    <row r="689" ht="15.75" customHeight="1"/>
+    <row r="690" ht="15.75" customHeight="1"/>
+    <row r="691" ht="15.75" customHeight="1"/>
+    <row r="692" ht="15.75" customHeight="1"/>
+    <row r="693" ht="15.75" customHeight="1"/>
+    <row r="694" ht="15.75" customHeight="1"/>
+    <row r="695" ht="15.75" customHeight="1"/>
+    <row r="696" ht="15.75" customHeight="1"/>
+    <row r="697" ht="15.75" customHeight="1"/>
+    <row r="698" ht="15.75" customHeight="1"/>
+    <row r="699" ht="15.75" customHeight="1"/>
+    <row r="700" ht="15.75" customHeight="1"/>
+    <row r="701" ht="15.75" customHeight="1"/>
+    <row r="702" ht="15.75" customHeight="1"/>
+    <row r="703" ht="15.75" customHeight="1"/>
+    <row r="704" ht="15.75" customHeight="1"/>
+    <row r="705" ht="15.75" customHeight="1"/>
+    <row r="706" ht="15.75" customHeight="1"/>
+    <row r="707" ht="15.75" customHeight="1"/>
+    <row r="708" ht="15.75" customHeight="1"/>
+    <row r="709" ht="15.75" customHeight="1"/>
+    <row r="710" ht="15.75" customHeight="1"/>
+    <row r="711" ht="15.75" customHeight="1"/>
+    <row r="712" ht="15.75" customHeight="1"/>
+    <row r="713" ht="15.75" customHeight="1"/>
+    <row r="714" ht="15.75" customHeight="1"/>
+    <row r="715" ht="15.75" customHeight="1"/>
+    <row r="716" ht="15.75" customHeight="1"/>
+    <row r="717" ht="15.75" customHeight="1"/>
+    <row r="718" ht="15.75" customHeight="1"/>
+    <row r="719" ht="15.75" customHeight="1"/>
+    <row r="720" ht="15.75" customHeight="1"/>
+    <row r="721" ht="15.75" customHeight="1"/>
+    <row r="722" ht="15.75" customHeight="1"/>
+    <row r="723" ht="15.75" customHeight="1"/>
+    <row r="724" ht="15.75" customHeight="1"/>
+    <row r="725" ht="15.75" customHeight="1"/>
+    <row r="726" ht="15.75" customHeight="1"/>
+    <row r="727" ht="15.75" customHeight="1"/>
+    <row r="728" ht="15.75" customHeight="1"/>
+    <row r="729" ht="15.75" customHeight="1"/>
+    <row r="730" ht="15.75" customHeight="1"/>
+    <row r="731" ht="15.75" customHeight="1"/>
+    <row r="732" ht="15.75" customHeight="1"/>
+    <row r="733" ht="15.75" customHeight="1"/>
+    <row r="734" ht="15.75" customHeight="1"/>
+    <row r="735" ht="15.75" customHeight="1"/>
+    <row r="736" ht="15.75" customHeight="1"/>
+    <row r="737" ht="15.75" customHeight="1"/>
+    <row r="738" ht="15.75" customHeight="1"/>
+    <row r="739" ht="15.75" customHeight="1"/>
+    <row r="740" ht="15.75" customHeight="1"/>
+    <row r="741" ht="15.75" customHeight="1"/>
+    <row r="742" ht="15.75" customHeight="1"/>
+    <row r="743" ht="15.75" customHeight="1"/>
+    <row r="744" ht="15.75" customHeight="1"/>
+    <row r="745" ht="15.75" customHeight="1"/>
+    <row r="746" ht="15.75" customHeight="1"/>
+    <row r="747" ht="15.75" customHeight="1"/>
+    <row r="748" ht="15.75" customHeight="1"/>
+    <row r="749" ht="15.75" customHeight="1"/>
+    <row r="750" ht="15.75" customHeight="1"/>
+    <row r="751" ht="15.75" customHeight="1"/>
+    <row r="752" ht="15.75" customHeight="1"/>
+    <row r="753" ht="15.75" customHeight="1"/>
+    <row r="754" ht="15.75" customHeight="1"/>
+    <row r="755" ht="15.75" customHeight="1"/>
+    <row r="756" ht="15.75" customHeight="1"/>
+    <row r="757" ht="15.75" customHeight="1"/>
+    <row r="758" ht="15.75" customHeight="1"/>
+    <row r="759" ht="15.75" customHeight="1"/>
+    <row r="760" ht="15.75" customHeight="1"/>
+    <row r="761" ht="15.75" customHeight="1"/>
+    <row r="762" ht="15.75" customHeight="1"/>
+    <row r="763" ht="15.75" customHeight="1"/>
+    <row r="764" ht="15.75" customHeight="1"/>
+    <row r="765" ht="15.75" customHeight="1"/>
+    <row r="766" ht="15.75" customHeight="1"/>
+    <row r="767" ht="15.75" customHeight="1"/>
+    <row r="768" ht="15.75" customHeight="1"/>
+    <row r="769" ht="15.75" customHeight="1"/>
+    <row r="770" ht="15.75" customHeight="1"/>
+    <row r="771" ht="15.75" customHeight="1"/>
+    <row r="772" ht="15.75" customHeight="1"/>
+    <row r="773" ht="15.75" customHeight="1"/>
+    <row r="774" ht="15.75" customHeight="1"/>
+    <row r="775" ht="15.75" customHeight="1"/>
+    <row r="776" ht="15.75" customHeight="1"/>
+    <row r="777" ht="15.75" customHeight="1"/>
+    <row r="778" ht="15.75" customHeight="1"/>
+    <row r="779" ht="15.75" customHeight="1"/>
+    <row r="780" ht="15.75" customHeight="1"/>
+    <row r="781" ht="15.75" customHeight="1"/>
+    <row r="782" ht="15.75" customHeight="1"/>
+    <row r="783" ht="15.75" customHeight="1"/>
+    <row r="784" ht="15.75" customHeight="1"/>
+    <row r="785" ht="15.75" customHeight="1"/>
+    <row r="786" ht="15.75" customHeight="1"/>
+    <row r="787" ht="15.75" customHeight="1"/>
+    <row r="788" ht="15.75" customHeight="1"/>
+    <row r="789" ht="15.75" customHeight="1"/>
+    <row r="790" ht="15.75" customHeight="1"/>
+    <row r="791" ht="15.75" customHeight="1"/>
+    <row r="792" ht="15.75" customHeight="1"/>
+    <row r="793" ht="15.75" customHeight="1"/>
+    <row r="794" ht="15.75" customHeight="1"/>
+    <row r="795" ht="15.75" customHeight="1"/>
+    <row r="796" ht="15.75" customHeight="1"/>
+    <row r="797" ht="15.75" customHeight="1"/>
+    <row r="798" ht="15.75" customHeight="1"/>
+    <row r="799" ht="15.75" customHeight="1"/>
+    <row r="800" ht="15.75" customHeight="1"/>
+    <row r="801" ht="15.75" customHeight="1"/>
+    <row r="802" ht="15.75" customHeight="1"/>
+    <row r="803" ht="15.75" customHeight="1"/>
+    <row r="804" ht="15.75" customHeight="1"/>
+    <row r="805" ht="15.75" customHeight="1"/>
+    <row r="806" ht="15.75" customHeight="1"/>
+    <row r="807" ht="15.75" customHeight="1"/>
+    <row r="808" ht="15.75" customHeight="1"/>
+    <row r="809" ht="15.75" customHeight="1"/>
+    <row r="810" ht="15.75" customHeight="1"/>
+    <row r="811" ht="15.75" customHeight="1"/>
+    <row r="812" ht="15.75" customHeight="1"/>
+    <row r="813" ht="15.75" customHeight="1"/>
+    <row r="814" ht="15.75" customHeight="1"/>
+    <row r="815" ht="15.75" customHeight="1"/>
+    <row r="816" ht="15.75" customHeight="1"/>
+    <row r="817" ht="15.75" customHeight="1"/>
+    <row r="818" ht="15.75" customHeight="1"/>
+    <row r="819" ht="15.75" customHeight="1"/>
+    <row r="820" ht="15.75" customHeight="1"/>
+    <row r="821" ht="15.75" customHeight="1"/>
+    <row r="822" ht="15.75" customHeight="1"/>
+    <row r="823" ht="15.75" customHeight="1"/>
+    <row r="824" ht="15.75" customHeight="1"/>
+    <row r="825" ht="15.75" customHeight="1"/>
+    <row r="826" ht="15.75" customHeight="1"/>
+    <row r="827" ht="15.75" customHeight="1"/>
+    <row r="828" ht="15.75" customHeight="1"/>
+    <row r="829" ht="15.75" customHeight="1"/>
+    <row r="830" ht="15.75" customHeight="1"/>
+    <row r="831" ht="15.75" customHeight="1"/>
+    <row r="832" ht="15.75" customHeight="1"/>
+    <row r="833" ht="15.75" customHeight="1"/>
+    <row r="834" ht="15.75" customHeight="1"/>
+    <row r="835" ht="15.75" customHeight="1"/>
+    <row r="836" ht="15.75" customHeight="1"/>
+    <row r="837" ht="15.75" customHeight="1"/>
+    <row r="838" ht="15.75" customHeight="1"/>
+    <row r="839" ht="15.75" customHeight="1"/>
+    <row r="840" ht="15.75" customHeight="1"/>
+    <row r="841" ht="15.75" customHeight="1"/>
+    <row r="842" ht="15.75" customHeight="1"/>
+    <row r="843" ht="15.75" customHeight="1"/>
+    <row r="844" ht="15.75" customHeight="1"/>
+    <row r="845" ht="15.75" customHeight="1"/>
+    <row r="846" ht="15.75" customHeight="1"/>
+    <row r="847" ht="15.75" customHeight="1"/>
+    <row r="848" ht="15.75" customHeight="1"/>
+    <row r="849" ht="15.75" customHeight="1"/>
+    <row r="850" ht="15.75" customHeight="1"/>
+    <row r="851" ht="15.75" customHeight="1"/>
+    <row r="852" ht="15.75" customHeight="1"/>
+    <row r="853" ht="15.75" customHeight="1"/>
+    <row r="854" ht="15.75" customHeight="1"/>
+    <row r="855" ht="15.75" customHeight="1"/>
+    <row r="856" ht="15.75" customHeight="1"/>
+    <row r="857" ht="15.75" customHeight="1"/>
+    <row r="858" ht="15.75" customHeight="1"/>
+    <row r="859" ht="15.75" customHeight="1"/>
+    <row r="860" ht="15.75" customHeight="1"/>
+    <row r="861" ht="15.75" customHeight="1"/>
+    <row r="862" ht="15.75" customHeight="1"/>
+    <row r="863" ht="15.75" customHeight="1"/>
+    <row r="864" ht="15.75" customHeight="1"/>
+    <row r="865" ht="15.75" customHeight="1"/>
+    <row r="866" ht="15.75" customHeight="1"/>
+    <row r="867" ht="15.75" customHeight="1"/>
+    <row r="868" ht="15.75" customHeight="1"/>
+    <row r="869" ht="15.75" customHeight="1"/>
+    <row r="870" ht="15.75" customHeight="1"/>
+    <row r="871" ht="15.75" customHeight="1"/>
+    <row r="872" ht="15.75" customHeight="1"/>
+    <row r="873" ht="15.75" customHeight="1"/>
+    <row r="874" ht="15.75" customHeight="1"/>
+    <row r="875" ht="15.75" customHeight="1"/>
+    <row r="876" ht="15.75" customHeight="1"/>
+    <row r="877" ht="15.75" customHeight="1"/>
+    <row r="878" ht="15.75" customHeight="1"/>
+    <row r="879" ht="15.75" customHeight="1"/>
+    <row r="880" ht="15.75" customHeight="1"/>
+    <row r="881" ht="15.75" customHeight="1"/>
+    <row r="882" ht="15.75" customHeight="1"/>
+    <row r="883" ht="15.75" customHeight="1"/>
+    <row r="884" ht="15.75" customHeight="1"/>
+    <row r="885" ht="15.75" customHeight="1"/>
+    <row r="886" ht="15.75" customHeight="1"/>
+    <row r="887" ht="15.75" customHeight="1"/>
+    <row r="888" ht="15.75" customHeight="1"/>
+    <row r="889" ht="15.75" customHeight="1"/>
+    <row r="890" ht="15.75" customHeight="1"/>
+    <row r="891" ht="15.75" customHeight="1"/>
+    <row r="892" ht="15.75" customHeight="1"/>
+    <row r="893" ht="15.75" customHeight="1"/>
+    <row r="894" ht="15.75" customHeight="1"/>
+    <row r="895" ht="15.75" customHeight="1"/>
+    <row r="896" ht="15.75" customHeight="1"/>
+    <row r="897" ht="15.75" customHeight="1"/>
+    <row r="898" ht="15.75" customHeight="1"/>
+    <row r="899" ht="15.75" customHeight="1"/>
+    <row r="900" ht="15.75" customHeight="1"/>
+    <row r="901" ht="15.75" customHeight="1"/>
+    <row r="902" ht="15.75" customHeight="1"/>
+    <row r="903" ht="15.75" customHeight="1"/>
+    <row r="904" ht="15.75" customHeight="1"/>
+    <row r="905" ht="15.75" customHeight="1"/>
+    <row r="906" ht="15.75" customHeight="1"/>
+    <row r="907" ht="15.75" customHeight="1"/>
+    <row r="908" ht="15.75" customHeight="1"/>
+    <row r="909" ht="15.75" customHeight="1"/>
+    <row r="910" ht="15.75" customHeight="1"/>
+    <row r="911" ht="15.75" customHeight="1"/>
+    <row r="912" ht="15.75" customHeight="1"/>
+    <row r="913" ht="15.75" customHeight="1"/>
+    <row r="914" ht="15.75" customHeight="1"/>
+    <row r="915" ht="15.75" customHeight="1"/>
+    <row r="916" ht="15.75" customHeight="1"/>
+    <row r="917" ht="15.75" customHeight="1"/>
+    <row r="918" ht="15.75" customHeight="1"/>
+    <row r="919" ht="15.75" customHeight="1"/>
+    <row r="920" ht="15.75" customHeight="1"/>
+    <row r="921" ht="15.75" customHeight="1"/>
+    <row r="922" ht="15.75" customHeight="1"/>
+    <row r="923" ht="15.75" customHeight="1"/>
+    <row r="924" ht="15.75" customHeight="1"/>
+    <row r="925" ht="15.75" customHeight="1"/>
+    <row r="926" ht="15.75" customHeight="1"/>
+    <row r="927" ht="15.75" customHeight="1"/>
+    <row r="928" ht="15.75" customHeight="1"/>
+    <row r="929" ht="15.75" customHeight="1"/>
+    <row r="930" ht="15.75" customHeight="1"/>
+    <row r="931" ht="15.75" customHeight="1"/>
+    <row r="932" ht="15.75" customHeight="1"/>
+    <row r="933" ht="15.75" customHeight="1"/>
+    <row r="934" ht="15.75" customHeight="1"/>
+    <row r="935" ht="15.75" customHeight="1"/>
+    <row r="936" ht="15.75" customHeight="1"/>
+    <row r="937" ht="15.75" customHeight="1"/>
+    <row r="938" ht="15.75" customHeight="1"/>
+    <row r="939" ht="15.75" customHeight="1"/>
+    <row r="940" ht="15.75" customHeight="1"/>
+    <row r="941" ht="15.75" customHeight="1"/>
+    <row r="942" ht="15.75" customHeight="1"/>
+    <row r="943" ht="15.75" customHeight="1"/>
+    <row r="944" ht="15.75" customHeight="1"/>
+    <row r="945" ht="15.75" customHeight="1"/>
+    <row r="946" ht="15.75" customHeight="1"/>
+    <row r="947" ht="15.75" customHeight="1"/>
+    <row r="948" ht="15.75" customHeight="1"/>
+    <row r="949" ht="15.75" customHeight="1"/>
+    <row r="950" ht="15.75" customHeight="1"/>
+    <row r="951" ht="15.75" customHeight="1"/>
+    <row r="952" ht="15.75" customHeight="1"/>
+    <row r="953" ht="15.75" customHeight="1"/>
+    <row r="954" ht="15.75" customHeight="1"/>
+    <row r="955" ht="15.75" customHeight="1"/>
+    <row r="956" ht="15.75" customHeight="1"/>
+    <row r="957" ht="15.75" customHeight="1"/>
+    <row r="958" ht="15.75" customHeight="1"/>
+    <row r="959" ht="15.75" customHeight="1"/>
+    <row r="960" ht="15.75" customHeight="1"/>
+    <row r="961" ht="15.75" customHeight="1"/>
+    <row r="962" ht="15.75" customHeight="1"/>
+    <row r="963" ht="15.75" customHeight="1"/>
+    <row r="964" ht="15.75" customHeight="1"/>
+    <row r="965" ht="15.75" customHeight="1"/>
+    <row r="966" ht="15.75" customHeight="1"/>
+    <row r="967" ht="15.75" customHeight="1"/>
+    <row r="968" ht="15.75" customHeight="1"/>
+    <row r="969" ht="15.75" customHeight="1"/>
+    <row r="970" ht="15.75" customHeight="1"/>
+    <row r="971" ht="15.75" customHeight="1"/>
+    <row r="972" ht="15.75" customHeight="1"/>
+    <row r="973" ht="15.75" customHeight="1"/>
+    <row r="974" ht="15.75" customHeight="1"/>
+    <row r="975" ht="15.75" customHeight="1"/>
+    <row r="976" ht="15.75" customHeight="1"/>
+    <row r="977" ht="15.75" customHeight="1"/>
+    <row r="978" ht="15.75" customHeight="1"/>
+    <row r="979" ht="15.75" customHeight="1"/>
+    <row r="980" ht="15.75" customHeight="1"/>
+    <row r="981" ht="15.75" customHeight="1"/>
+    <row r="982" ht="15.75" customHeight="1"/>
+    <row r="983" ht="15.75" customHeight="1"/>
+    <row r="984" ht="15.75" customHeight="1"/>
+    <row r="985" ht="15.75" customHeight="1"/>
+    <row r="986" ht="15.75" customHeight="1"/>
+    <row r="987" ht="15.75" customHeight="1"/>
+    <row r="988" ht="15.75" customHeight="1"/>
+    <row r="989" ht="15.75" customHeight="1"/>
+    <row r="990" ht="15.75" customHeight="1"/>
+    <row r="991" ht="15.75" customHeight="1"/>
+    <row r="992" ht="15.75" customHeight="1"/>
+    <row r="993" ht="15.75" customHeight="1"/>
+    <row r="994" ht="15.75" customHeight="1"/>
+    <row r="995" ht="15.75" customHeight="1"/>
+    <row r="996" ht="15.75" customHeight="1"/>
+    <row r="997" ht="15.75" customHeight="1"/>
+    <row r="998" ht="15.75" customHeight="1"/>
+    <row r="999" ht="15.75" customHeight="1"/>
+    <row r="1000" ht="15.75" customHeight="1"/>
+    <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="C2"/>
+    <hyperlink r:id="rId2" ref="C3"/>
+    <hyperlink r:id="rId3" ref="C4"/>
+    <hyperlink r:id="rId4" ref="C5"/>
+    <hyperlink r:id="rId5" ref="C6"/>
+    <hyperlink r:id="rId6" ref="C7"/>
+    <hyperlink r:id="rId7" ref="C8"/>
+    <hyperlink r:id="rId8" ref="C9"/>
+    <hyperlink r:id="rId9" ref="C10"/>
+    <hyperlink r:id="rId10" ref="E10"/>
+    <hyperlink r:id="rId11" ref="C11"/>
+    <hyperlink r:id="rId12" ref="C12"/>
+    <hyperlink r:id="rId13" ref="E12"/>
+    <hyperlink r:id="rId14" ref="C13"/>
+    <hyperlink r:id="rId15" ref="E13"/>
+    <hyperlink r:id="rId16" ref="C14"/>
+    <hyperlink r:id="rId17" ref="C15"/>
+    <hyperlink r:id="rId18" ref="C16"/>
+    <hyperlink r:id="rId19" ref="C17"/>
+    <hyperlink r:id="rId20" ref="C18"/>
+    <hyperlink r:id="rId21" ref="C19"/>
+    <hyperlink r:id="rId22" ref="C20"/>
+    <hyperlink r:id="rId23" ref="C21"/>
+    <hyperlink r:id="rId24" ref="C22"/>
+    <hyperlink r:id="rId25" ref="C23"/>
+    <hyperlink r:id="rId26" ref="C24"/>
+    <hyperlink r:id="rId27" ref="E24"/>
+    <hyperlink r:id="rId28" ref="C25"/>
+    <hyperlink r:id="rId29" ref="C26"/>
+    <hyperlink r:id="rId30" ref="C27"/>
+    <hyperlink r:id="rId31" ref="C28"/>
+    <hyperlink r:id="rId32" ref="C29"/>
+    <hyperlink r:id="rId33" ref="C30"/>
+    <hyperlink r:id="rId34" ref="C31"/>
+    <hyperlink r:id="rId35" ref="C32"/>
+    <hyperlink r:id="rId36" ref="C33"/>
+    <hyperlink r:id="rId37" ref="C34"/>
+    <hyperlink r:id="rId38" ref="C35"/>
+    <hyperlink r:id="rId39" ref="C36"/>
+    <hyperlink r:id="rId40" ref="C37"/>
+    <hyperlink r:id="rId41" ref="C38"/>
+    <hyperlink r:id="rId42" ref="C39"/>
+    <hyperlink r:id="rId43" ref="C40"/>
+    <hyperlink r:id="rId44" ref="C41"/>
+    <hyperlink r:id="rId45" ref="C42"/>
+    <hyperlink r:id="rId46" ref="C43"/>
+    <hyperlink r:id="rId47" ref="C44"/>
+    <hyperlink r:id="rId48" ref="C45"/>
+    <hyperlink r:id="rId49" ref="C46"/>
+    <hyperlink r:id="rId50" ref="C47"/>
+    <hyperlink r:id="rId51" ref="C48"/>
+    <hyperlink r:id="rId52" ref="C49"/>
+    <hyperlink r:id="rId53" ref="C50"/>
+    <hyperlink r:id="rId54" ref="C51"/>
+    <hyperlink r:id="rId55" ref="C52"/>
+    <hyperlink r:id="rId56" ref="C53"/>
+    <hyperlink r:id="rId57" ref="C54"/>
+    <hyperlink r:id="rId58" ref="C55"/>
+  </hyperlinks>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId59"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <pageSetUpPr/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="10.71"/>
+    <col customWidth="1" min="2" max="2" width="14.71"/>
+    <col customWidth="1" min="3" max="3" width="45.43"/>
+    <col customWidth="1" min="4" max="4" width="36.57"/>
+    <col customWidth="1" min="5" max="5" width="12.0"/>
+    <col customWidth="1" min="6" max="15" width="9.14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5">
+        <v>46087.0</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5">
+        <v>46087.0</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5">
+        <v>46087.0</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11">
+        <v>46092.0</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="11">
+        <v>46092.0</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11">
+        <v>46093.0</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11">
+        <v>46093.0</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11">
+        <v>46093.0</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11">
+        <v>46093.0</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11">
+        <v>46094.0</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11">
+        <v>46094.0</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="11">
+        <v>46095.0</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13">
+        <v>46097.0</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13">
+        <v>46098.0</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13">
+        <v>46098.0</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13">
+        <v>46098.0</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13">
+        <v>46099.0</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E18" s="14"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="13">
+        <v>46099.0</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="15">
+        <v>46102.0</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E20" s="18"/>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="13">
+        <v>46103.0</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="14"/>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="13">
+        <v>46104.0</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E22" s="18"/>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="13">
+        <v>46105.0</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E23" s="14"/>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="13">
+        <v>46106.0</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="13">
+        <v>46108.0</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="13">
+        <v>46108.0</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="13">
+        <v>46108.0</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="15">
+        <v>46109.0</v>
+      </c>
+      <c r="B28" s="20"/>
+      <c r="C28" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="A29" s="15">
+        <v>46113.0</v>
+      </c>
+      <c r="B29" s="20"/>
+      <c r="C29" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" s="16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="15">
+        <v>46114.0</v>
+      </c>
+      <c r="B30" s="20"/>
+      <c r="C30" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="D30" s="16" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="13">
+        <v>46116.0</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="13">
+        <v>46119.0</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="15">
+        <v>46120.0</v>
+      </c>
+      <c r="B33" s="20"/>
+      <c r="C33" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="16" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="A34" s="13">
+        <v>46127.0</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="A35" s="13">
+        <v>46127.0</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="13">
+        <v>46128.0</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="A37" s="13">
+        <v>46129.0</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="A38" s="13">
+        <v>46130.0</v>
+      </c>
+      <c r="C38" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="39" ht="15.75" customHeight="1">
+      <c r="A39" s="13">
+        <v>46131.0</v>
+      </c>
+      <c r="C39" s="19" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40" ht="15.75" customHeight="1">
+      <c r="A40" s="13">
+        <v>46131.0</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="A41" s="13">
+        <v>46132.0</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="A42" s="13">
+        <v>46133.0</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="A43" s="13">
+        <v>46133.0</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="A44" s="13">
+        <v>46135.0</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H44" s="6"/>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="13">
+        <v>46135.0</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="13">
+        <v>46136.0</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="13">
+        <v>46136.0</v>
+      </c>
+      <c r="C47" s="21" t="s">
+        <v>112</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="13">
+        <v>46136.0</v>
+      </c>
+      <c r="C48" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E48" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="A49" s="13">
+        <v>46137.0</v>
+      </c>
+      <c r="C49" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customHeight="1">
+      <c r="A50" s="13">
+        <v>46138.0</v>
+      </c>
+      <c r="C50" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="D50" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E50" s="6" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customHeight="1">
+      <c r="A51" s="13">
+        <v>46138.0</v>
+      </c>
+      <c r="C51" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="D51" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customHeight="1">
+      <c r="A52" s="13">
+        <v>46138.0</v>
+      </c>
+      <c r="C52" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customHeight="1">
+      <c r="A53" s="13">
+        <v>46140.0</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customHeight="1">
+      <c r="A54" s="13">
+        <v>46141.0</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customHeight="1">
+      <c r="A55" s="13">
+        <v>46142.0</v>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="13">
+        <v>46113.0</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="13">
+        <v>46146.0</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
     <row r="58" ht="15.75" customHeight="1"/>
     <row r="59" ht="15.75" customHeight="1"/>
     <row r="60" ht="15.75" customHeight="1"/>
@@ -2657,15 +4568,18 @@
     <hyperlink r:id="rId53" ref="C50"/>
     <hyperlink r:id="rId54" ref="C51"/>
     <hyperlink r:id="rId55" ref="C52"/>
+    <hyperlink r:id="rId56" ref="C53"/>
+    <hyperlink r:id="rId57" ref="C56"/>
+    <hyperlink r:id="rId58" ref="C57"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId56"/>
+  <drawing r:id="rId59"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -2677,18 +4591,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>126</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="J2" s="6">
         <v>6.0</v>
@@ -2696,13 +4610,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="J3" s="6">
         <v>1.0</v>
@@ -2710,13 +4624,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="J4" s="6">
         <v>1.0</v>
@@ -2724,21 +4638,21 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>135</v>
+        <v>147</v>
       </c>
       <c r="J6" s="6">
         <v>2.0</v>
@@ -2746,13 +4660,13 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="J7" s="6">
         <v>1.0</v>
@@ -2760,13 +4674,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="I8" s="6" t="s">
         <v>141</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="J8" s="6">
         <v>1.0</v>
@@ -2774,42 +4688,42 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="J14" s="6">
         <v>2.0</v>
@@ -2817,13 +4731,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="J15" s="6">
         <v>2.0</v>
@@ -2831,21 +4745,21 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>129</v>
+        <v>141</v>
       </c>
       <c r="J17" s="6">
         <v>3.0</v>
@@ -2853,13 +4767,13 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="J18" s="6">
         <v>2.0</v>
@@ -2867,26 +4781,26 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 04-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -4,21 +4,20 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Hoja1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Copia de Hoja1" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="Hoja x" sheetId="3" r:id="rId6"/>
+    <sheet state="visible" name="Hoja x" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="nVGqFylxOMnrMPQ+QhULhUoor+EoekNxf7YmYmFKK2k="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="hoF12/XSjhOFQCYc+u+CyOYasShuanztpa6csxB8U0U="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="166">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -474,48 +473,10 @@
     <t>https://youtu.be/O_RFkTcApiY</t>
   </si>
   <si>
-    <t>1re Turno  09:00 am</t>
+    <t>1er Turno  09:00 am</t>
   </si>
   <si>
     <t>Trabajo de Fuerza, Juego de Centros y Transiciones D-A , A-D</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>VERDE</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-      </rPr>
-      <t xml:space="preserve">: 8 de 12 veces terminó la jugada (6 por derecha, 1 por el medio y 1 por la izquierda). 4 pérdidas en zona baja (2 por el medio, 1 izq. 1 derecha). </t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <b/>
-        <color theme="1"/>
-      </rPr>
-      <t>NARANJA</t>
-    </r>
-    <r>
-      <rPr>
-        <rFont val="Calibri"/>
-        <color theme="1"/>
-      </rPr>
-      <t>: 4 de 9 veces terminó la jugada (2 izq. y 2 derecha) y un gol marcado. 5 pérdidas (3 por derecha y 2 por izquierda)</t>
-    </r>
-  </si>
-  <si>
-    <t>Turno unico 3pm</t>
-  </si>
-  <si>
-    <t>Juego de Patrones, Juego a 11 dirigido</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -786,10 +747,6 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -2778,1810 +2735,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <pageSetUpPr/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="10.71"/>
-    <col customWidth="1" min="2" max="2" width="14.71"/>
-    <col customWidth="1" min="3" max="3" width="45.43"/>
-    <col customWidth="1" min="4" max="4" width="36.57"/>
-    <col customWidth="1" min="5" max="5" width="12.0"/>
-    <col customWidth="1" min="6" max="15" width="9.14"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5">
-        <v>46087.0</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5">
-        <v>46087.0</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5">
-        <v>46087.0</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="11">
-        <v>46092.0</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="11">
-        <v>46092.0</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="11">
-        <v>46093.0</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="11">
-        <v>46093.0</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11">
-        <v>46093.0</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11">
-        <v>46093.0</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11">
-        <v>46094.0</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11">
-        <v>46094.0</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11">
-        <v>46095.0</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="13">
-        <v>46097.0</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="13">
-        <v>46098.0</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="13">
-        <v>46098.0</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="13">
-        <v>46098.0</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="13">
-        <v>46099.0</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="E18" s="14"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="13">
-        <v>46099.0</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="15">
-        <v>46102.0</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="E20" s="18"/>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="13">
-        <v>46103.0</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="E21" s="14"/>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="13">
-        <v>46104.0</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="E22" s="18"/>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="13">
-        <v>46105.0</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="14"/>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="13">
-        <v>46106.0</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="13">
-        <v>46108.0</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="13">
-        <v>46108.0</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="13">
-        <v>46108.0</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="15">
-        <v>46109.0</v>
-      </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="15">
-        <v>46113.0</v>
-      </c>
-      <c r="B29" s="20"/>
-      <c r="C29" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="D29" s="16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="15">
-        <v>46114.0</v>
-      </c>
-      <c r="B30" s="20"/>
-      <c r="C30" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="D30" s="16" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="13">
-        <v>46116.0</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="13">
-        <v>46119.0</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="15">
-        <v>46120.0</v>
-      </c>
-      <c r="B33" s="20"/>
-      <c r="C33" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="D33" s="16" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="13">
-        <v>46127.0</v>
-      </c>
-      <c r="C34" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="13">
-        <v>46127.0</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="13">
-        <v>46128.0</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="13">
-        <v>46129.0</v>
-      </c>
-      <c r="C37" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="13">
-        <v>46130.0</v>
-      </c>
-      <c r="C38" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="13">
-        <v>46131.0</v>
-      </c>
-      <c r="C39" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="13">
-        <v>46131.0</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="13">
-        <v>46132.0</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="13">
-        <v>46133.0</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="13">
-        <v>46133.0</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="13">
-        <v>46135.0</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="H44" s="6"/>
-    </row>
-    <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="13">
-        <v>46135.0</v>
-      </c>
-      <c r="C45" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="13">
-        <v>46136.0</v>
-      </c>
-      <c r="C46" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="13">
-        <v>46136.0</v>
-      </c>
-      <c r="C47" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="13">
-        <v>46136.0</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>115</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="13">
-        <v>46137.0</v>
-      </c>
-      <c r="C49" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="13">
-        <v>46138.0</v>
-      </c>
-      <c r="C50" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="13">
-        <v>46138.0</v>
-      </c>
-      <c r="C51" s="7" t="s">
-        <v>123</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="13">
-        <v>46138.0</v>
-      </c>
-      <c r="C52" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="13">
-        <v>46140.0</v>
-      </c>
-      <c r="C53" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="13">
-        <v>46141.0</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="13">
-        <v>46142.0</v>
-      </c>
-    </row>
-    <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="13">
-        <v>46113.0</v>
-      </c>
-      <c r="C56" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="13">
-        <v>46146.0</v>
-      </c>
-      <c r="C57" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="E57" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="58" ht="15.75" customHeight="1"/>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
-    <row r="65" ht="15.75" customHeight="1"/>
-    <row r="66" ht="15.75" customHeight="1"/>
-    <row r="67" ht="15.75" customHeight="1"/>
-    <row r="68" ht="15.75" customHeight="1"/>
-    <row r="69" ht="15.75" customHeight="1"/>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
-    <row r="117" ht="15.75" customHeight="1"/>
-    <row r="118" ht="15.75" customHeight="1"/>
-    <row r="119" ht="15.75" customHeight="1"/>
-    <row r="120" ht="15.75" customHeight="1"/>
-    <row r="121" ht="15.75" customHeight="1"/>
-    <row r="122" ht="15.75" customHeight="1"/>
-    <row r="123" ht="15.75" customHeight="1"/>
-    <row r="124" ht="15.75" customHeight="1"/>
-    <row r="125" ht="15.75" customHeight="1"/>
-    <row r="126" ht="15.75" customHeight="1"/>
-    <row r="127" ht="15.75" customHeight="1"/>
-    <row r="128" ht="15.75" customHeight="1"/>
-    <row r="129" ht="15.75" customHeight="1"/>
-    <row r="130" ht="15.75" customHeight="1"/>
-    <row r="131" ht="15.75" customHeight="1"/>
-    <row r="132" ht="15.75" customHeight="1"/>
-    <row r="133" ht="15.75" customHeight="1"/>
-    <row r="134" ht="15.75" customHeight="1"/>
-    <row r="135" ht="15.75" customHeight="1"/>
-    <row r="136" ht="15.75" customHeight="1"/>
-    <row r="137" ht="15.75" customHeight="1"/>
-    <row r="138" ht="15.75" customHeight="1"/>
-    <row r="139" ht="15.75" customHeight="1"/>
-    <row r="140" ht="15.75" customHeight="1"/>
-    <row r="141" ht="15.75" customHeight="1"/>
-    <row r="142" ht="15.75" customHeight="1"/>
-    <row r="143" ht="15.75" customHeight="1"/>
-    <row r="144" ht="15.75" customHeight="1"/>
-    <row r="145" ht="15.75" customHeight="1"/>
-    <row r="146" ht="15.75" customHeight="1"/>
-    <row r="147" ht="15.75" customHeight="1"/>
-    <row r="148" ht="15.75" customHeight="1"/>
-    <row r="149" ht="15.75" customHeight="1"/>
-    <row r="150" ht="15.75" customHeight="1"/>
-    <row r="151" ht="15.75" customHeight="1"/>
-    <row r="152" ht="15.75" customHeight="1"/>
-    <row r="153" ht="15.75" customHeight="1"/>
-    <row r="154" ht="15.75" customHeight="1"/>
-    <row r="155" ht="15.75" customHeight="1"/>
-    <row r="156" ht="15.75" customHeight="1"/>
-    <row r="157" ht="15.75" customHeight="1"/>
-    <row r="158" ht="15.75" customHeight="1"/>
-    <row r="159" ht="15.75" customHeight="1"/>
-    <row r="160" ht="15.75" customHeight="1"/>
-    <row r="161" ht="15.75" customHeight="1"/>
-    <row r="162" ht="15.75" customHeight="1"/>
-    <row r="163" ht="15.75" customHeight="1"/>
-    <row r="164" ht="15.75" customHeight="1"/>
-    <row r="165" ht="15.75" customHeight="1"/>
-    <row r="166" ht="15.75" customHeight="1"/>
-    <row r="167" ht="15.75" customHeight="1"/>
-    <row r="168" ht="15.75" customHeight="1"/>
-    <row r="169" ht="15.75" customHeight="1"/>
-    <row r="170" ht="15.75" customHeight="1"/>
-    <row r="171" ht="15.75" customHeight="1"/>
-    <row r="172" ht="15.75" customHeight="1"/>
-    <row r="173" ht="15.75" customHeight="1"/>
-    <row r="174" ht="15.75" customHeight="1"/>
-    <row r="175" ht="15.75" customHeight="1"/>
-    <row r="176" ht="15.75" customHeight="1"/>
-    <row r="177" ht="15.75" customHeight="1"/>
-    <row r="178" ht="15.75" customHeight="1"/>
-    <row r="179" ht="15.75" customHeight="1"/>
-    <row r="180" ht="15.75" customHeight="1"/>
-    <row r="181" ht="15.75" customHeight="1"/>
-    <row r="182" ht="15.75" customHeight="1"/>
-    <row r="183" ht="15.75" customHeight="1"/>
-    <row r="184" ht="15.75" customHeight="1"/>
-    <row r="185" ht="15.75" customHeight="1"/>
-    <row r="186" ht="15.75" customHeight="1"/>
-    <row r="187" ht="15.75" customHeight="1"/>
-    <row r="188" ht="15.75" customHeight="1"/>
-    <row r="189" ht="15.75" customHeight="1"/>
-    <row r="190" ht="15.75" customHeight="1"/>
-    <row r="191" ht="15.75" customHeight="1"/>
-    <row r="192" ht="15.75" customHeight="1"/>
-    <row r="193" ht="15.75" customHeight="1"/>
-    <row r="194" ht="15.75" customHeight="1"/>
-    <row r="195" ht="15.75" customHeight="1"/>
-    <row r="196" ht="15.75" customHeight="1"/>
-    <row r="197" ht="15.75" customHeight="1"/>
-    <row r="198" ht="15.75" customHeight="1"/>
-    <row r="199" ht="15.75" customHeight="1"/>
-    <row r="200" ht="15.75" customHeight="1"/>
-    <row r="201" ht="15.75" customHeight="1"/>
-    <row r="202" ht="15.75" customHeight="1"/>
-    <row r="203" ht="15.75" customHeight="1"/>
-    <row r="204" ht="15.75" customHeight="1"/>
-    <row r="205" ht="15.75" customHeight="1"/>
-    <row r="206" ht="15.75" customHeight="1"/>
-    <row r="207" ht="15.75" customHeight="1"/>
-    <row r="208" ht="15.75" customHeight="1"/>
-    <row r="209" ht="15.75" customHeight="1"/>
-    <row r="210" ht="15.75" customHeight="1"/>
-    <row r="211" ht="15.75" customHeight="1"/>
-    <row r="212" ht="15.75" customHeight="1"/>
-    <row r="213" ht="15.75" customHeight="1"/>
-    <row r="214" ht="15.75" customHeight="1"/>
-    <row r="215" ht="15.75" customHeight="1"/>
-    <row r="216" ht="15.75" customHeight="1"/>
-    <row r="217" ht="15.75" customHeight="1"/>
-    <row r="218" ht="15.75" customHeight="1"/>
-    <row r="219" ht="15.75" customHeight="1"/>
-    <row r="220" ht="15.75" customHeight="1"/>
-    <row r="221" ht="15.75" customHeight="1"/>
-    <row r="222" ht="15.75" customHeight="1"/>
-    <row r="223" ht="15.75" customHeight="1"/>
-    <row r="224" ht="15.75" customHeight="1"/>
-    <row r="225" ht="15.75" customHeight="1"/>
-    <row r="226" ht="15.75" customHeight="1"/>
-    <row r="227" ht="15.75" customHeight="1"/>
-    <row r="228" ht="15.75" customHeight="1"/>
-    <row r="229" ht="15.75" customHeight="1"/>
-    <row r="230" ht="15.75" customHeight="1"/>
-    <row r="231" ht="15.75" customHeight="1"/>
-    <row r="232" ht="15.75" customHeight="1"/>
-    <row r="233" ht="15.75" customHeight="1"/>
-    <row r="234" ht="15.75" customHeight="1"/>
-    <row r="235" ht="15.75" customHeight="1"/>
-    <row r="236" ht="15.75" customHeight="1"/>
-    <row r="237" ht="15.75" customHeight="1"/>
-    <row r="238" ht="15.75" customHeight="1"/>
-    <row r="239" ht="15.75" customHeight="1"/>
-    <row r="240" ht="15.75" customHeight="1"/>
-    <row r="241" ht="15.75" customHeight="1"/>
-    <row r="242" ht="15.75" customHeight="1"/>
-    <row r="243" ht="15.75" customHeight="1"/>
-    <row r="244" ht="15.75" customHeight="1"/>
-    <row r="245" ht="15.75" customHeight="1"/>
-    <row r="246" ht="15.75" customHeight="1"/>
-    <row r="247" ht="15.75" customHeight="1"/>
-    <row r="248" ht="15.75" customHeight="1"/>
-    <row r="249" ht="15.75" customHeight="1"/>
-    <row r="250" ht="15.75" customHeight="1"/>
-    <row r="251" ht="15.75" customHeight="1"/>
-    <row r="252" ht="15.75" customHeight="1"/>
-    <row r="253" ht="15.75" customHeight="1"/>
-    <row r="254" ht="15.75" customHeight="1"/>
-    <row r="255" ht="15.75" customHeight="1"/>
-    <row r="256" ht="15.75" customHeight="1"/>
-    <row r="257" ht="15.75" customHeight="1"/>
-    <row r="258" ht="15.75" customHeight="1"/>
-    <row r="259" ht="15.75" customHeight="1"/>
-    <row r="260" ht="15.75" customHeight="1"/>
-    <row r="261" ht="15.75" customHeight="1"/>
-    <row r="262" ht="15.75" customHeight="1"/>
-    <row r="263" ht="15.75" customHeight="1"/>
-    <row r="264" ht="15.75" customHeight="1"/>
-    <row r="265" ht="15.75" customHeight="1"/>
-    <row r="266" ht="15.75" customHeight="1"/>
-    <row r="267" ht="15.75" customHeight="1"/>
-    <row r="268" ht="15.75" customHeight="1"/>
-    <row r="269" ht="15.75" customHeight="1"/>
-    <row r="270" ht="15.75" customHeight="1"/>
-    <row r="271" ht="15.75" customHeight="1"/>
-    <row r="272" ht="15.75" customHeight="1"/>
-    <row r="273" ht="15.75" customHeight="1"/>
-    <row r="274" ht="15.75" customHeight="1"/>
-    <row r="275" ht="15.75" customHeight="1"/>
-    <row r="276" ht="15.75" customHeight="1"/>
-    <row r="277" ht="15.75" customHeight="1"/>
-    <row r="278" ht="15.75" customHeight="1"/>
-    <row r="279" ht="15.75" customHeight="1"/>
-    <row r="280" ht="15.75" customHeight="1"/>
-    <row r="281" ht="15.75" customHeight="1"/>
-    <row r="282" ht="15.75" customHeight="1"/>
-    <row r="283" ht="15.75" customHeight="1"/>
-    <row r="284" ht="15.75" customHeight="1"/>
-    <row r="285" ht="15.75" customHeight="1"/>
-    <row r="286" ht="15.75" customHeight="1"/>
-    <row r="287" ht="15.75" customHeight="1"/>
-    <row r="288" ht="15.75" customHeight="1"/>
-    <row r="289" ht="15.75" customHeight="1"/>
-    <row r="290" ht="15.75" customHeight="1"/>
-    <row r="291" ht="15.75" customHeight="1"/>
-    <row r="292" ht="15.75" customHeight="1"/>
-    <row r="293" ht="15.75" customHeight="1"/>
-    <row r="294" ht="15.75" customHeight="1"/>
-    <row r="295" ht="15.75" customHeight="1"/>
-    <row r="296" ht="15.75" customHeight="1"/>
-    <row r="297" ht="15.75" customHeight="1"/>
-    <row r="298" ht="15.75" customHeight="1"/>
-    <row r="299" ht="15.75" customHeight="1"/>
-    <row r="300" ht="15.75" customHeight="1"/>
-    <row r="301" ht="15.75" customHeight="1"/>
-    <row r="302" ht="15.75" customHeight="1"/>
-    <row r="303" ht="15.75" customHeight="1"/>
-    <row r="304" ht="15.75" customHeight="1"/>
-    <row r="305" ht="15.75" customHeight="1"/>
-    <row r="306" ht="15.75" customHeight="1"/>
-    <row r="307" ht="15.75" customHeight="1"/>
-    <row r="308" ht="15.75" customHeight="1"/>
-    <row r="309" ht="15.75" customHeight="1"/>
-    <row r="310" ht="15.75" customHeight="1"/>
-    <row r="311" ht="15.75" customHeight="1"/>
-    <row r="312" ht="15.75" customHeight="1"/>
-    <row r="313" ht="15.75" customHeight="1"/>
-    <row r="314" ht="15.75" customHeight="1"/>
-    <row r="315" ht="15.75" customHeight="1"/>
-    <row r="316" ht="15.75" customHeight="1"/>
-    <row r="317" ht="15.75" customHeight="1"/>
-    <row r="318" ht="15.75" customHeight="1"/>
-    <row r="319" ht="15.75" customHeight="1"/>
-    <row r="320" ht="15.75" customHeight="1"/>
-    <row r="321" ht="15.75" customHeight="1"/>
-    <row r="322" ht="15.75" customHeight="1"/>
-    <row r="323" ht="15.75" customHeight="1"/>
-    <row r="324" ht="15.75" customHeight="1"/>
-    <row r="325" ht="15.75" customHeight="1"/>
-    <row r="326" ht="15.75" customHeight="1"/>
-    <row r="327" ht="15.75" customHeight="1"/>
-    <row r="328" ht="15.75" customHeight="1"/>
-    <row r="329" ht="15.75" customHeight="1"/>
-    <row r="330" ht="15.75" customHeight="1"/>
-    <row r="331" ht="15.75" customHeight="1"/>
-    <row r="332" ht="15.75" customHeight="1"/>
-    <row r="333" ht="15.75" customHeight="1"/>
-    <row r="334" ht="15.75" customHeight="1"/>
-    <row r="335" ht="15.75" customHeight="1"/>
-    <row r="336" ht="15.75" customHeight="1"/>
-    <row r="337" ht="15.75" customHeight="1"/>
-    <row r="338" ht="15.75" customHeight="1"/>
-    <row r="339" ht="15.75" customHeight="1"/>
-    <row r="340" ht="15.75" customHeight="1"/>
-    <row r="341" ht="15.75" customHeight="1"/>
-    <row r="342" ht="15.75" customHeight="1"/>
-    <row r="343" ht="15.75" customHeight="1"/>
-    <row r="344" ht="15.75" customHeight="1"/>
-    <row r="345" ht="15.75" customHeight="1"/>
-    <row r="346" ht="15.75" customHeight="1"/>
-    <row r="347" ht="15.75" customHeight="1"/>
-    <row r="348" ht="15.75" customHeight="1"/>
-    <row r="349" ht="15.75" customHeight="1"/>
-    <row r="350" ht="15.75" customHeight="1"/>
-    <row r="351" ht="15.75" customHeight="1"/>
-    <row r="352" ht="15.75" customHeight="1"/>
-    <row r="353" ht="15.75" customHeight="1"/>
-    <row r="354" ht="15.75" customHeight="1"/>
-    <row r="355" ht="15.75" customHeight="1"/>
-    <row r="356" ht="15.75" customHeight="1"/>
-    <row r="357" ht="15.75" customHeight="1"/>
-    <row r="358" ht="15.75" customHeight="1"/>
-    <row r="359" ht="15.75" customHeight="1"/>
-    <row r="360" ht="15.75" customHeight="1"/>
-    <row r="361" ht="15.75" customHeight="1"/>
-    <row r="362" ht="15.75" customHeight="1"/>
-    <row r="363" ht="15.75" customHeight="1"/>
-    <row r="364" ht="15.75" customHeight="1"/>
-    <row r="365" ht="15.75" customHeight="1"/>
-    <row r="366" ht="15.75" customHeight="1"/>
-    <row r="367" ht="15.75" customHeight="1"/>
-    <row r="368" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
-    <row r="385" ht="15.75" customHeight="1"/>
-    <row r="386" ht="15.75" customHeight="1"/>
-    <row r="387" ht="15.75" customHeight="1"/>
-    <row r="388" ht="15.75" customHeight="1"/>
-    <row r="389" ht="15.75" customHeight="1"/>
-    <row r="390" ht="15.75" customHeight="1"/>
-    <row r="391" ht="15.75" customHeight="1"/>
-    <row r="392" ht="15.75" customHeight="1"/>
-    <row r="393" ht="15.75" customHeight="1"/>
-    <row r="394" ht="15.75" customHeight="1"/>
-    <row r="395" ht="15.75" customHeight="1"/>
-    <row r="396" ht="15.75" customHeight="1"/>
-    <row r="397" ht="15.75" customHeight="1"/>
-    <row r="398" ht="15.75" customHeight="1"/>
-    <row r="399" ht="15.75" customHeight="1"/>
-    <row r="400" ht="15.75" customHeight="1"/>
-    <row r="401" ht="15.75" customHeight="1"/>
-    <row r="402" ht="15.75" customHeight="1"/>
-    <row r="403" ht="15.75" customHeight="1"/>
-    <row r="404" ht="15.75" customHeight="1"/>
-    <row r="405" ht="15.75" customHeight="1"/>
-    <row r="406" ht="15.75" customHeight="1"/>
-    <row r="407" ht="15.75" customHeight="1"/>
-    <row r="408" ht="15.75" customHeight="1"/>
-    <row r="409" ht="15.75" customHeight="1"/>
-    <row r="410" ht="15.75" customHeight="1"/>
-    <row r="411" ht="15.75" customHeight="1"/>
-    <row r="412" ht="15.75" customHeight="1"/>
-    <row r="413" ht="15.75" customHeight="1"/>
-    <row r="414" ht="15.75" customHeight="1"/>
-    <row r="415" ht="15.75" customHeight="1"/>
-    <row r="416" ht="15.75" customHeight="1"/>
-    <row r="417" ht="15.75" customHeight="1"/>
-    <row r="418" ht="15.75" customHeight="1"/>
-    <row r="419" ht="15.75" customHeight="1"/>
-    <row r="420" ht="15.75" customHeight="1"/>
-    <row r="421" ht="15.75" customHeight="1"/>
-    <row r="422" ht="15.75" customHeight="1"/>
-    <row r="423" ht="15.75" customHeight="1"/>
-    <row r="424" ht="15.75" customHeight="1"/>
-    <row r="425" ht="15.75" customHeight="1"/>
-    <row r="426" ht="15.75" customHeight="1"/>
-    <row r="427" ht="15.75" customHeight="1"/>
-    <row r="428" ht="15.75" customHeight="1"/>
-    <row r="429" ht="15.75" customHeight="1"/>
-    <row r="430" ht="15.75" customHeight="1"/>
-    <row r="431" ht="15.75" customHeight="1"/>
-    <row r="432" ht="15.75" customHeight="1"/>
-    <row r="433" ht="15.75" customHeight="1"/>
-    <row r="434" ht="15.75" customHeight="1"/>
-    <row r="435" ht="15.75" customHeight="1"/>
-    <row r="436" ht="15.75" customHeight="1"/>
-    <row r="437" ht="15.75" customHeight="1"/>
-    <row r="438" ht="15.75" customHeight="1"/>
-    <row r="439" ht="15.75" customHeight="1"/>
-    <row r="440" ht="15.75" customHeight="1"/>
-    <row r="441" ht="15.75" customHeight="1"/>
-    <row r="442" ht="15.75" customHeight="1"/>
-    <row r="443" ht="15.75" customHeight="1"/>
-    <row r="444" ht="15.75" customHeight="1"/>
-    <row r="445" ht="15.75" customHeight="1"/>
-    <row r="446" ht="15.75" customHeight="1"/>
-    <row r="447" ht="15.75" customHeight="1"/>
-    <row r="448" ht="15.75" customHeight="1"/>
-    <row r="449" ht="15.75" customHeight="1"/>
-    <row r="450" ht="15.75" customHeight="1"/>
-    <row r="451" ht="15.75" customHeight="1"/>
-    <row r="452" ht="15.75" customHeight="1"/>
-    <row r="453" ht="15.75" customHeight="1"/>
-    <row r="454" ht="15.75" customHeight="1"/>
-    <row r="455" ht="15.75" customHeight="1"/>
-    <row r="456" ht="15.75" customHeight="1"/>
-    <row r="457" ht="15.75" customHeight="1"/>
-    <row r="458" ht="15.75" customHeight="1"/>
-    <row r="459" ht="15.75" customHeight="1"/>
-    <row r="460" ht="15.75" customHeight="1"/>
-    <row r="461" ht="15.75" customHeight="1"/>
-    <row r="462" ht="15.75" customHeight="1"/>
-    <row r="463" ht="15.75" customHeight="1"/>
-    <row r="464" ht="15.75" customHeight="1"/>
-    <row r="465" ht="15.75" customHeight="1"/>
-    <row r="466" ht="15.75" customHeight="1"/>
-    <row r="467" ht="15.75" customHeight="1"/>
-    <row r="468" ht="15.75" customHeight="1"/>
-    <row r="469" ht="15.75" customHeight="1"/>
-    <row r="470" ht="15.75" customHeight="1"/>
-    <row r="471" ht="15.75" customHeight="1"/>
-    <row r="472" ht="15.75" customHeight="1"/>
-    <row r="473" ht="15.75" customHeight="1"/>
-    <row r="474" ht="15.75" customHeight="1"/>
-    <row r="475" ht="15.75" customHeight="1"/>
-    <row r="476" ht="15.75" customHeight="1"/>
-    <row r="477" ht="15.75" customHeight="1"/>
-    <row r="478" ht="15.75" customHeight="1"/>
-    <row r="479" ht="15.75" customHeight="1"/>
-    <row r="480" ht="15.75" customHeight="1"/>
-    <row r="481" ht="15.75" customHeight="1"/>
-    <row r="482" ht="15.75" customHeight="1"/>
-    <row r="483" ht="15.75" customHeight="1"/>
-    <row r="484" ht="15.75" customHeight="1"/>
-    <row r="485" ht="15.75" customHeight="1"/>
-    <row r="486" ht="15.75" customHeight="1"/>
-    <row r="487" ht="15.75" customHeight="1"/>
-    <row r="488" ht="15.75" customHeight="1"/>
-    <row r="489" ht="15.75" customHeight="1"/>
-    <row r="490" ht="15.75" customHeight="1"/>
-    <row r="491" ht="15.75" customHeight="1"/>
-    <row r="492" ht="15.75" customHeight="1"/>
-    <row r="493" ht="15.75" customHeight="1"/>
-    <row r="494" ht="15.75" customHeight="1"/>
-    <row r="495" ht="15.75" customHeight="1"/>
-    <row r="496" ht="15.75" customHeight="1"/>
-    <row r="497" ht="15.75" customHeight="1"/>
-    <row r="498" ht="15.75" customHeight="1"/>
-    <row r="499" ht="15.75" customHeight="1"/>
-    <row r="500" ht="15.75" customHeight="1"/>
-    <row r="501" ht="15.75" customHeight="1"/>
-    <row r="502" ht="15.75" customHeight="1"/>
-    <row r="503" ht="15.75" customHeight="1"/>
-    <row r="504" ht="15.75" customHeight="1"/>
-    <row r="505" ht="15.75" customHeight="1"/>
-    <row r="506" ht="15.75" customHeight="1"/>
-    <row r="507" ht="15.75" customHeight="1"/>
-    <row r="508" ht="15.75" customHeight="1"/>
-    <row r="509" ht="15.75" customHeight="1"/>
-    <row r="510" ht="15.75" customHeight="1"/>
-    <row r="511" ht="15.75" customHeight="1"/>
-    <row r="512" ht="15.75" customHeight="1"/>
-    <row r="513" ht="15.75" customHeight="1"/>
-    <row r="514" ht="15.75" customHeight="1"/>
-    <row r="515" ht="15.75" customHeight="1"/>
-    <row r="516" ht="15.75" customHeight="1"/>
-    <row r="517" ht="15.75" customHeight="1"/>
-    <row r="518" ht="15.75" customHeight="1"/>
-    <row r="519" ht="15.75" customHeight="1"/>
-    <row r="520" ht="15.75" customHeight="1"/>
-    <row r="521" ht="15.75" customHeight="1"/>
-    <row r="522" ht="15.75" customHeight="1"/>
-    <row r="523" ht="15.75" customHeight="1"/>
-    <row r="524" ht="15.75" customHeight="1"/>
-    <row r="525" ht="15.75" customHeight="1"/>
-    <row r="526" ht="15.75" customHeight="1"/>
-    <row r="527" ht="15.75" customHeight="1"/>
-    <row r="528" ht="15.75" customHeight="1"/>
-    <row r="529" ht="15.75" customHeight="1"/>
-    <row r="530" ht="15.75" customHeight="1"/>
-    <row r="531" ht="15.75" customHeight="1"/>
-    <row r="532" ht="15.75" customHeight="1"/>
-    <row r="533" ht="15.75" customHeight="1"/>
-    <row r="534" ht="15.75" customHeight="1"/>
-    <row r="535" ht="15.75" customHeight="1"/>
-    <row r="536" ht="15.75" customHeight="1"/>
-    <row r="537" ht="15.75" customHeight="1"/>
-    <row r="538" ht="15.75" customHeight="1"/>
-    <row r="539" ht="15.75" customHeight="1"/>
-    <row r="540" ht="15.75" customHeight="1"/>
-    <row r="541" ht="15.75" customHeight="1"/>
-    <row r="542" ht="15.75" customHeight="1"/>
-    <row r="543" ht="15.75" customHeight="1"/>
-    <row r="544" ht="15.75" customHeight="1"/>
-    <row r="545" ht="15.75" customHeight="1"/>
-    <row r="546" ht="15.75" customHeight="1"/>
-    <row r="547" ht="15.75" customHeight="1"/>
-    <row r="548" ht="15.75" customHeight="1"/>
-    <row r="549" ht="15.75" customHeight="1"/>
-    <row r="550" ht="15.75" customHeight="1"/>
-    <row r="551" ht="15.75" customHeight="1"/>
-    <row r="552" ht="15.75" customHeight="1"/>
-    <row r="553" ht="15.75" customHeight="1"/>
-    <row r="554" ht="15.75" customHeight="1"/>
-    <row r="555" ht="15.75" customHeight="1"/>
-    <row r="556" ht="15.75" customHeight="1"/>
-    <row r="557" ht="15.75" customHeight="1"/>
-    <row r="558" ht="15.75" customHeight="1"/>
-    <row r="559" ht="15.75" customHeight="1"/>
-    <row r="560" ht="15.75" customHeight="1"/>
-    <row r="561" ht="15.75" customHeight="1"/>
-    <row r="562" ht="15.75" customHeight="1"/>
-    <row r="563" ht="15.75" customHeight="1"/>
-    <row r="564" ht="15.75" customHeight="1"/>
-    <row r="565" ht="15.75" customHeight="1"/>
-    <row r="566" ht="15.75" customHeight="1"/>
-    <row r="567" ht="15.75" customHeight="1"/>
-    <row r="568" ht="15.75" customHeight="1"/>
-    <row r="569" ht="15.75" customHeight="1"/>
-    <row r="570" ht="15.75" customHeight="1"/>
-    <row r="571" ht="15.75" customHeight="1"/>
-    <row r="572" ht="15.75" customHeight="1"/>
-    <row r="573" ht="15.75" customHeight="1"/>
-    <row r="574" ht="15.75" customHeight="1"/>
-    <row r="575" ht="15.75" customHeight="1"/>
-    <row r="576" ht="15.75" customHeight="1"/>
-    <row r="577" ht="15.75" customHeight="1"/>
-    <row r="578" ht="15.75" customHeight="1"/>
-    <row r="579" ht="15.75" customHeight="1"/>
-    <row r="580" ht="15.75" customHeight="1"/>
-    <row r="581" ht="15.75" customHeight="1"/>
-    <row r="582" ht="15.75" customHeight="1"/>
-    <row r="583" ht="15.75" customHeight="1"/>
-    <row r="584" ht="15.75" customHeight="1"/>
-    <row r="585" ht="15.75" customHeight="1"/>
-    <row r="586" ht="15.75" customHeight="1"/>
-    <row r="587" ht="15.75" customHeight="1"/>
-    <row r="588" ht="15.75" customHeight="1"/>
-    <row r="589" ht="15.75" customHeight="1"/>
-    <row r="590" ht="15.75" customHeight="1"/>
-    <row r="591" ht="15.75" customHeight="1"/>
-    <row r="592" ht="15.75" customHeight="1"/>
-    <row r="593" ht="15.75" customHeight="1"/>
-    <row r="594" ht="15.75" customHeight="1"/>
-    <row r="595" ht="15.75" customHeight="1"/>
-    <row r="596" ht="15.75" customHeight="1"/>
-    <row r="597" ht="15.75" customHeight="1"/>
-    <row r="598" ht="15.75" customHeight="1"/>
-    <row r="599" ht="15.75" customHeight="1"/>
-    <row r="600" ht="15.75" customHeight="1"/>
-    <row r="601" ht="15.75" customHeight="1"/>
-    <row r="602" ht="15.75" customHeight="1"/>
-    <row r="603" ht="15.75" customHeight="1"/>
-    <row r="604" ht="15.75" customHeight="1"/>
-    <row r="605" ht="15.75" customHeight="1"/>
-    <row r="606" ht="15.75" customHeight="1"/>
-    <row r="607" ht="15.75" customHeight="1"/>
-    <row r="608" ht="15.75" customHeight="1"/>
-    <row r="609" ht="15.75" customHeight="1"/>
-    <row r="610" ht="15.75" customHeight="1"/>
-    <row r="611" ht="15.75" customHeight="1"/>
-    <row r="612" ht="15.75" customHeight="1"/>
-    <row r="613" ht="15.75" customHeight="1"/>
-    <row r="614" ht="15.75" customHeight="1"/>
-    <row r="615" ht="15.75" customHeight="1"/>
-    <row r="616" ht="15.75" customHeight="1"/>
-    <row r="617" ht="15.75" customHeight="1"/>
-    <row r="618" ht="15.75" customHeight="1"/>
-    <row r="619" ht="15.75" customHeight="1"/>
-    <row r="620" ht="15.75" customHeight="1"/>
-    <row r="621" ht="15.75" customHeight="1"/>
-    <row r="622" ht="15.75" customHeight="1"/>
-    <row r="623" ht="15.75" customHeight="1"/>
-    <row r="624" ht="15.75" customHeight="1"/>
-    <row r="625" ht="15.75" customHeight="1"/>
-    <row r="626" ht="15.75" customHeight="1"/>
-    <row r="627" ht="15.75" customHeight="1"/>
-    <row r="628" ht="15.75" customHeight="1"/>
-    <row r="629" ht="15.75" customHeight="1"/>
-    <row r="630" ht="15.75" customHeight="1"/>
-    <row r="631" ht="15.75" customHeight="1"/>
-    <row r="632" ht="15.75" customHeight="1"/>
-    <row r="633" ht="15.75" customHeight="1"/>
-    <row r="634" ht="15.75" customHeight="1"/>
-    <row r="635" ht="15.75" customHeight="1"/>
-    <row r="636" ht="15.75" customHeight="1"/>
-    <row r="637" ht="15.75" customHeight="1"/>
-    <row r="638" ht="15.75" customHeight="1"/>
-    <row r="639" ht="15.75" customHeight="1"/>
-    <row r="640" ht="15.75" customHeight="1"/>
-    <row r="641" ht="15.75" customHeight="1"/>
-    <row r="642" ht="15.75" customHeight="1"/>
-    <row r="643" ht="15.75" customHeight="1"/>
-    <row r="644" ht="15.75" customHeight="1"/>
-    <row r="645" ht="15.75" customHeight="1"/>
-    <row r="646" ht="15.75" customHeight="1"/>
-    <row r="647" ht="15.75" customHeight="1"/>
-    <row r="648" ht="15.75" customHeight="1"/>
-    <row r="649" ht="15.75" customHeight="1"/>
-    <row r="650" ht="15.75" customHeight="1"/>
-    <row r="651" ht="15.75" customHeight="1"/>
-    <row r="652" ht="15.75" customHeight="1"/>
-    <row r="653" ht="15.75" customHeight="1"/>
-    <row r="654" ht="15.75" customHeight="1"/>
-    <row r="655" ht="15.75" customHeight="1"/>
-    <row r="656" ht="15.75" customHeight="1"/>
-    <row r="657" ht="15.75" customHeight="1"/>
-    <row r="658" ht="15.75" customHeight="1"/>
-    <row r="659" ht="15.75" customHeight="1"/>
-    <row r="660" ht="15.75" customHeight="1"/>
-    <row r="661" ht="15.75" customHeight="1"/>
-    <row r="662" ht="15.75" customHeight="1"/>
-    <row r="663" ht="15.75" customHeight="1"/>
-    <row r="664" ht="15.75" customHeight="1"/>
-    <row r="665" ht="15.75" customHeight="1"/>
-    <row r="666" ht="15.75" customHeight="1"/>
-    <row r="667" ht="15.75" customHeight="1"/>
-    <row r="668" ht="15.75" customHeight="1"/>
-    <row r="669" ht="15.75" customHeight="1"/>
-    <row r="670" ht="15.75" customHeight="1"/>
-    <row r="671" ht="15.75" customHeight="1"/>
-    <row r="672" ht="15.75" customHeight="1"/>
-    <row r="673" ht="15.75" customHeight="1"/>
-    <row r="674" ht="15.75" customHeight="1"/>
-    <row r="675" ht="15.75" customHeight="1"/>
-    <row r="676" ht="15.75" customHeight="1"/>
-    <row r="677" ht="15.75" customHeight="1"/>
-    <row r="678" ht="15.75" customHeight="1"/>
-    <row r="679" ht="15.75" customHeight="1"/>
-    <row r="680" ht="15.75" customHeight="1"/>
-    <row r="681" ht="15.75" customHeight="1"/>
-    <row r="682" ht="15.75" customHeight="1"/>
-    <row r="683" ht="15.75" customHeight="1"/>
-    <row r="684" ht="15.75" customHeight="1"/>
-    <row r="685" ht="15.75" customHeight="1"/>
-    <row r="686" ht="15.75" customHeight="1"/>
-    <row r="687" ht="15.75" customHeight="1"/>
-    <row r="688" ht="15.75" customHeight="1"/>
-    <row r="689" ht="15.75" customHeight="1"/>
-    <row r="690" ht="15.75" customHeight="1"/>
-    <row r="691" ht="15.75" customHeight="1"/>
-    <row r="692" ht="15.75" customHeight="1"/>
-    <row r="693" ht="15.75" customHeight="1"/>
-    <row r="694" ht="15.75" customHeight="1"/>
-    <row r="695" ht="15.75" customHeight="1"/>
-    <row r="696" ht="15.75" customHeight="1"/>
-    <row r="697" ht="15.75" customHeight="1"/>
-    <row r="698" ht="15.75" customHeight="1"/>
-    <row r="699" ht="15.75" customHeight="1"/>
-    <row r="700" ht="15.75" customHeight="1"/>
-    <row r="701" ht="15.75" customHeight="1"/>
-    <row r="702" ht="15.75" customHeight="1"/>
-    <row r="703" ht="15.75" customHeight="1"/>
-    <row r="704" ht="15.75" customHeight="1"/>
-    <row r="705" ht="15.75" customHeight="1"/>
-    <row r="706" ht="15.75" customHeight="1"/>
-    <row r="707" ht="15.75" customHeight="1"/>
-    <row r="708" ht="15.75" customHeight="1"/>
-    <row r="709" ht="15.75" customHeight="1"/>
-    <row r="710" ht="15.75" customHeight="1"/>
-    <row r="711" ht="15.75" customHeight="1"/>
-    <row r="712" ht="15.75" customHeight="1"/>
-    <row r="713" ht="15.75" customHeight="1"/>
-    <row r="714" ht="15.75" customHeight="1"/>
-    <row r="715" ht="15.75" customHeight="1"/>
-    <row r="716" ht="15.75" customHeight="1"/>
-    <row r="717" ht="15.75" customHeight="1"/>
-    <row r="718" ht="15.75" customHeight="1"/>
-    <row r="719" ht="15.75" customHeight="1"/>
-    <row r="720" ht="15.75" customHeight="1"/>
-    <row r="721" ht="15.75" customHeight="1"/>
-    <row r="722" ht="15.75" customHeight="1"/>
-    <row r="723" ht="15.75" customHeight="1"/>
-    <row r="724" ht="15.75" customHeight="1"/>
-    <row r="725" ht="15.75" customHeight="1"/>
-    <row r="726" ht="15.75" customHeight="1"/>
-    <row r="727" ht="15.75" customHeight="1"/>
-    <row r="728" ht="15.75" customHeight="1"/>
-    <row r="729" ht="15.75" customHeight="1"/>
-    <row r="730" ht="15.75" customHeight="1"/>
-    <row r="731" ht="15.75" customHeight="1"/>
-    <row r="732" ht="15.75" customHeight="1"/>
-    <row r="733" ht="15.75" customHeight="1"/>
-    <row r="734" ht="15.75" customHeight="1"/>
-    <row r="735" ht="15.75" customHeight="1"/>
-    <row r="736" ht="15.75" customHeight="1"/>
-    <row r="737" ht="15.75" customHeight="1"/>
-    <row r="738" ht="15.75" customHeight="1"/>
-    <row r="739" ht="15.75" customHeight="1"/>
-    <row r="740" ht="15.75" customHeight="1"/>
-    <row r="741" ht="15.75" customHeight="1"/>
-    <row r="742" ht="15.75" customHeight="1"/>
-    <row r="743" ht="15.75" customHeight="1"/>
-    <row r="744" ht="15.75" customHeight="1"/>
-    <row r="745" ht="15.75" customHeight="1"/>
-    <row r="746" ht="15.75" customHeight="1"/>
-    <row r="747" ht="15.75" customHeight="1"/>
-    <row r="748" ht="15.75" customHeight="1"/>
-    <row r="749" ht="15.75" customHeight="1"/>
-    <row r="750" ht="15.75" customHeight="1"/>
-    <row r="751" ht="15.75" customHeight="1"/>
-    <row r="752" ht="15.75" customHeight="1"/>
-    <row r="753" ht="15.75" customHeight="1"/>
-    <row r="754" ht="15.75" customHeight="1"/>
-    <row r="755" ht="15.75" customHeight="1"/>
-    <row r="756" ht="15.75" customHeight="1"/>
-    <row r="757" ht="15.75" customHeight="1"/>
-    <row r="758" ht="15.75" customHeight="1"/>
-    <row r="759" ht="15.75" customHeight="1"/>
-    <row r="760" ht="15.75" customHeight="1"/>
-    <row r="761" ht="15.75" customHeight="1"/>
-    <row r="762" ht="15.75" customHeight="1"/>
-    <row r="763" ht="15.75" customHeight="1"/>
-    <row r="764" ht="15.75" customHeight="1"/>
-    <row r="765" ht="15.75" customHeight="1"/>
-    <row r="766" ht="15.75" customHeight="1"/>
-    <row r="767" ht="15.75" customHeight="1"/>
-    <row r="768" ht="15.75" customHeight="1"/>
-    <row r="769" ht="15.75" customHeight="1"/>
-    <row r="770" ht="15.75" customHeight="1"/>
-    <row r="771" ht="15.75" customHeight="1"/>
-    <row r="772" ht="15.75" customHeight="1"/>
-    <row r="773" ht="15.75" customHeight="1"/>
-    <row r="774" ht="15.75" customHeight="1"/>
-    <row r="775" ht="15.75" customHeight="1"/>
-    <row r="776" ht="15.75" customHeight="1"/>
-    <row r="777" ht="15.75" customHeight="1"/>
-    <row r="778" ht="15.75" customHeight="1"/>
-    <row r="779" ht="15.75" customHeight="1"/>
-    <row r="780" ht="15.75" customHeight="1"/>
-    <row r="781" ht="15.75" customHeight="1"/>
-    <row r="782" ht="15.75" customHeight="1"/>
-    <row r="783" ht="15.75" customHeight="1"/>
-    <row r="784" ht="15.75" customHeight="1"/>
-    <row r="785" ht="15.75" customHeight="1"/>
-    <row r="786" ht="15.75" customHeight="1"/>
-    <row r="787" ht="15.75" customHeight="1"/>
-    <row r="788" ht="15.75" customHeight="1"/>
-    <row r="789" ht="15.75" customHeight="1"/>
-    <row r="790" ht="15.75" customHeight="1"/>
-    <row r="791" ht="15.75" customHeight="1"/>
-    <row r="792" ht="15.75" customHeight="1"/>
-    <row r="793" ht="15.75" customHeight="1"/>
-    <row r="794" ht="15.75" customHeight="1"/>
-    <row r="795" ht="15.75" customHeight="1"/>
-    <row r="796" ht="15.75" customHeight="1"/>
-    <row r="797" ht="15.75" customHeight="1"/>
-    <row r="798" ht="15.75" customHeight="1"/>
-    <row r="799" ht="15.75" customHeight="1"/>
-    <row r="800" ht="15.75" customHeight="1"/>
-    <row r="801" ht="15.75" customHeight="1"/>
-    <row r="802" ht="15.75" customHeight="1"/>
-    <row r="803" ht="15.75" customHeight="1"/>
-    <row r="804" ht="15.75" customHeight="1"/>
-    <row r="805" ht="15.75" customHeight="1"/>
-    <row r="806" ht="15.75" customHeight="1"/>
-    <row r="807" ht="15.75" customHeight="1"/>
-    <row r="808" ht="15.75" customHeight="1"/>
-    <row r="809" ht="15.75" customHeight="1"/>
-    <row r="810" ht="15.75" customHeight="1"/>
-    <row r="811" ht="15.75" customHeight="1"/>
-    <row r="812" ht="15.75" customHeight="1"/>
-    <row r="813" ht="15.75" customHeight="1"/>
-    <row r="814" ht="15.75" customHeight="1"/>
-    <row r="815" ht="15.75" customHeight="1"/>
-    <row r="816" ht="15.75" customHeight="1"/>
-    <row r="817" ht="15.75" customHeight="1"/>
-    <row r="818" ht="15.75" customHeight="1"/>
-    <row r="819" ht="15.75" customHeight="1"/>
-    <row r="820" ht="15.75" customHeight="1"/>
-    <row r="821" ht="15.75" customHeight="1"/>
-    <row r="822" ht="15.75" customHeight="1"/>
-    <row r="823" ht="15.75" customHeight="1"/>
-    <row r="824" ht="15.75" customHeight="1"/>
-    <row r="825" ht="15.75" customHeight="1"/>
-    <row r="826" ht="15.75" customHeight="1"/>
-    <row r="827" ht="15.75" customHeight="1"/>
-    <row r="828" ht="15.75" customHeight="1"/>
-    <row r="829" ht="15.75" customHeight="1"/>
-    <row r="830" ht="15.75" customHeight="1"/>
-    <row r="831" ht="15.75" customHeight="1"/>
-    <row r="832" ht="15.75" customHeight="1"/>
-    <row r="833" ht="15.75" customHeight="1"/>
-    <row r="834" ht="15.75" customHeight="1"/>
-    <row r="835" ht="15.75" customHeight="1"/>
-    <row r="836" ht="15.75" customHeight="1"/>
-    <row r="837" ht="15.75" customHeight="1"/>
-    <row r="838" ht="15.75" customHeight="1"/>
-    <row r="839" ht="15.75" customHeight="1"/>
-    <row r="840" ht="15.75" customHeight="1"/>
-    <row r="841" ht="15.75" customHeight="1"/>
-    <row r="842" ht="15.75" customHeight="1"/>
-    <row r="843" ht="15.75" customHeight="1"/>
-    <row r="844" ht="15.75" customHeight="1"/>
-    <row r="845" ht="15.75" customHeight="1"/>
-    <row r="846" ht="15.75" customHeight="1"/>
-    <row r="847" ht="15.75" customHeight="1"/>
-    <row r="848" ht="15.75" customHeight="1"/>
-    <row r="849" ht="15.75" customHeight="1"/>
-    <row r="850" ht="15.75" customHeight="1"/>
-    <row r="851" ht="15.75" customHeight="1"/>
-    <row r="852" ht="15.75" customHeight="1"/>
-    <row r="853" ht="15.75" customHeight="1"/>
-    <row r="854" ht="15.75" customHeight="1"/>
-    <row r="855" ht="15.75" customHeight="1"/>
-    <row r="856" ht="15.75" customHeight="1"/>
-    <row r="857" ht="15.75" customHeight="1"/>
-    <row r="858" ht="15.75" customHeight="1"/>
-    <row r="859" ht="15.75" customHeight="1"/>
-    <row r="860" ht="15.75" customHeight="1"/>
-    <row r="861" ht="15.75" customHeight="1"/>
-    <row r="862" ht="15.75" customHeight="1"/>
-    <row r="863" ht="15.75" customHeight="1"/>
-    <row r="864" ht="15.75" customHeight="1"/>
-    <row r="865" ht="15.75" customHeight="1"/>
-    <row r="866" ht="15.75" customHeight="1"/>
-    <row r="867" ht="15.75" customHeight="1"/>
-    <row r="868" ht="15.75" customHeight="1"/>
-    <row r="869" ht="15.75" customHeight="1"/>
-    <row r="870" ht="15.75" customHeight="1"/>
-    <row r="871" ht="15.75" customHeight="1"/>
-    <row r="872" ht="15.75" customHeight="1"/>
-    <row r="873" ht="15.75" customHeight="1"/>
-    <row r="874" ht="15.75" customHeight="1"/>
-    <row r="875" ht="15.75" customHeight="1"/>
-    <row r="876" ht="15.75" customHeight="1"/>
-    <row r="877" ht="15.75" customHeight="1"/>
-    <row r="878" ht="15.75" customHeight="1"/>
-    <row r="879" ht="15.75" customHeight="1"/>
-    <row r="880" ht="15.75" customHeight="1"/>
-    <row r="881" ht="15.75" customHeight="1"/>
-    <row r="882" ht="15.75" customHeight="1"/>
-    <row r="883" ht="15.75" customHeight="1"/>
-    <row r="884" ht="15.75" customHeight="1"/>
-    <row r="885" ht="15.75" customHeight="1"/>
-    <row r="886" ht="15.75" customHeight="1"/>
-    <row r="887" ht="15.75" customHeight="1"/>
-    <row r="888" ht="15.75" customHeight="1"/>
-    <row r="889" ht="15.75" customHeight="1"/>
-    <row r="890" ht="15.75" customHeight="1"/>
-    <row r="891" ht="15.75" customHeight="1"/>
-    <row r="892" ht="15.75" customHeight="1"/>
-    <row r="893" ht="15.75" customHeight="1"/>
-    <row r="894" ht="15.75" customHeight="1"/>
-    <row r="895" ht="15.75" customHeight="1"/>
-    <row r="896" ht="15.75" customHeight="1"/>
-    <row r="897" ht="15.75" customHeight="1"/>
-    <row r="898" ht="15.75" customHeight="1"/>
-    <row r="899" ht="15.75" customHeight="1"/>
-    <row r="900" ht="15.75" customHeight="1"/>
-    <row r="901" ht="15.75" customHeight="1"/>
-    <row r="902" ht="15.75" customHeight="1"/>
-    <row r="903" ht="15.75" customHeight="1"/>
-    <row r="904" ht="15.75" customHeight="1"/>
-    <row r="905" ht="15.75" customHeight="1"/>
-    <row r="906" ht="15.75" customHeight="1"/>
-    <row r="907" ht="15.75" customHeight="1"/>
-    <row r="908" ht="15.75" customHeight="1"/>
-    <row r="909" ht="15.75" customHeight="1"/>
-    <row r="910" ht="15.75" customHeight="1"/>
-    <row r="911" ht="15.75" customHeight="1"/>
-    <row r="912" ht="15.75" customHeight="1"/>
-    <row r="913" ht="15.75" customHeight="1"/>
-    <row r="914" ht="15.75" customHeight="1"/>
-    <row r="915" ht="15.75" customHeight="1"/>
-    <row r="916" ht="15.75" customHeight="1"/>
-    <row r="917" ht="15.75" customHeight="1"/>
-    <row r="918" ht="15.75" customHeight="1"/>
-    <row r="919" ht="15.75" customHeight="1"/>
-    <row r="920" ht="15.75" customHeight="1"/>
-    <row r="921" ht="15.75" customHeight="1"/>
-    <row r="922" ht="15.75" customHeight="1"/>
-    <row r="923" ht="15.75" customHeight="1"/>
-    <row r="924" ht="15.75" customHeight="1"/>
-    <row r="925" ht="15.75" customHeight="1"/>
-    <row r="926" ht="15.75" customHeight="1"/>
-    <row r="927" ht="15.75" customHeight="1"/>
-    <row r="928" ht="15.75" customHeight="1"/>
-    <row r="929" ht="15.75" customHeight="1"/>
-    <row r="930" ht="15.75" customHeight="1"/>
-    <row r="931" ht="15.75" customHeight="1"/>
-    <row r="932" ht="15.75" customHeight="1"/>
-    <row r="933" ht="15.75" customHeight="1"/>
-    <row r="934" ht="15.75" customHeight="1"/>
-    <row r="935" ht="15.75" customHeight="1"/>
-    <row r="936" ht="15.75" customHeight="1"/>
-    <row r="937" ht="15.75" customHeight="1"/>
-    <row r="938" ht="15.75" customHeight="1"/>
-    <row r="939" ht="15.75" customHeight="1"/>
-    <row r="940" ht="15.75" customHeight="1"/>
-    <row r="941" ht="15.75" customHeight="1"/>
-    <row r="942" ht="15.75" customHeight="1"/>
-    <row r="943" ht="15.75" customHeight="1"/>
-    <row r="944" ht="15.75" customHeight="1"/>
-    <row r="945" ht="15.75" customHeight="1"/>
-    <row r="946" ht="15.75" customHeight="1"/>
-    <row r="947" ht="15.75" customHeight="1"/>
-    <row r="948" ht="15.75" customHeight="1"/>
-    <row r="949" ht="15.75" customHeight="1"/>
-    <row r="950" ht="15.75" customHeight="1"/>
-    <row r="951" ht="15.75" customHeight="1"/>
-    <row r="952" ht="15.75" customHeight="1"/>
-    <row r="953" ht="15.75" customHeight="1"/>
-    <row r="954" ht="15.75" customHeight="1"/>
-    <row r="955" ht="15.75" customHeight="1"/>
-    <row r="956" ht="15.75" customHeight="1"/>
-    <row r="957" ht="15.75" customHeight="1"/>
-    <row r="958" ht="15.75" customHeight="1"/>
-    <row r="959" ht="15.75" customHeight="1"/>
-    <row r="960" ht="15.75" customHeight="1"/>
-    <row r="961" ht="15.75" customHeight="1"/>
-    <row r="962" ht="15.75" customHeight="1"/>
-    <row r="963" ht="15.75" customHeight="1"/>
-    <row r="964" ht="15.75" customHeight="1"/>
-    <row r="965" ht="15.75" customHeight="1"/>
-    <row r="966" ht="15.75" customHeight="1"/>
-    <row r="967" ht="15.75" customHeight="1"/>
-    <row r="968" ht="15.75" customHeight="1"/>
-    <row r="969" ht="15.75" customHeight="1"/>
-    <row r="970" ht="15.75" customHeight="1"/>
-    <row r="971" ht="15.75" customHeight="1"/>
-    <row r="972" ht="15.75" customHeight="1"/>
-    <row r="973" ht="15.75" customHeight="1"/>
-    <row r="974" ht="15.75" customHeight="1"/>
-    <row r="975" ht="15.75" customHeight="1"/>
-    <row r="976" ht="15.75" customHeight="1"/>
-    <row r="977" ht="15.75" customHeight="1"/>
-    <row r="978" ht="15.75" customHeight="1"/>
-    <row r="979" ht="15.75" customHeight="1"/>
-    <row r="980" ht="15.75" customHeight="1"/>
-    <row r="981" ht="15.75" customHeight="1"/>
-    <row r="982" ht="15.75" customHeight="1"/>
-    <row r="983" ht="15.75" customHeight="1"/>
-    <row r="984" ht="15.75" customHeight="1"/>
-    <row r="985" ht="15.75" customHeight="1"/>
-    <row r="986" ht="15.75" customHeight="1"/>
-    <row r="987" ht="15.75" customHeight="1"/>
-    <row r="988" ht="15.75" customHeight="1"/>
-    <row r="989" ht="15.75" customHeight="1"/>
-    <row r="990" ht="15.75" customHeight="1"/>
-    <row r="991" ht="15.75" customHeight="1"/>
-    <row r="992" ht="15.75" customHeight="1"/>
-    <row r="993" ht="15.75" customHeight="1"/>
-    <row r="994" ht="15.75" customHeight="1"/>
-    <row r="995" ht="15.75" customHeight="1"/>
-    <row r="996" ht="15.75" customHeight="1"/>
-    <row r="997" ht="15.75" customHeight="1"/>
-    <row r="998" ht="15.75" customHeight="1"/>
-    <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
-    <row r="1001" ht="15.75" customHeight="1"/>
-    <row r="1002" ht="15.75" customHeight="1"/>
-    <row r="1003" ht="15.75" customHeight="1"/>
-    <row r="1004" ht="15.75" customHeight="1"/>
-    <row r="1005" ht="15.75" customHeight="1"/>
-    <row r="1006" ht="15.75" customHeight="1"/>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink r:id="rId1" ref="C2"/>
-    <hyperlink r:id="rId2" ref="C3"/>
-    <hyperlink r:id="rId3" ref="C4"/>
-    <hyperlink r:id="rId4" ref="C5"/>
-    <hyperlink r:id="rId5" ref="C6"/>
-    <hyperlink r:id="rId6" ref="C7"/>
-    <hyperlink r:id="rId7" ref="C8"/>
-    <hyperlink r:id="rId8" ref="C9"/>
-    <hyperlink r:id="rId9" ref="C10"/>
-    <hyperlink r:id="rId10" ref="E10"/>
-    <hyperlink r:id="rId11" ref="C11"/>
-    <hyperlink r:id="rId12" ref="C12"/>
-    <hyperlink r:id="rId13" ref="E12"/>
-    <hyperlink r:id="rId14" ref="C13"/>
-    <hyperlink r:id="rId15" ref="E13"/>
-    <hyperlink r:id="rId16" ref="C14"/>
-    <hyperlink r:id="rId17" ref="C15"/>
-    <hyperlink r:id="rId18" ref="C16"/>
-    <hyperlink r:id="rId19" ref="C17"/>
-    <hyperlink r:id="rId20" ref="C18"/>
-    <hyperlink r:id="rId21" ref="C19"/>
-    <hyperlink r:id="rId22" ref="C20"/>
-    <hyperlink r:id="rId23" ref="C21"/>
-    <hyperlink r:id="rId24" ref="C22"/>
-    <hyperlink r:id="rId25" ref="C23"/>
-    <hyperlink r:id="rId26" ref="C24"/>
-    <hyperlink r:id="rId27" ref="E24"/>
-    <hyperlink r:id="rId28" ref="C25"/>
-    <hyperlink r:id="rId29" ref="C26"/>
-    <hyperlink r:id="rId30" ref="C27"/>
-    <hyperlink r:id="rId31" ref="C28"/>
-    <hyperlink r:id="rId32" ref="C29"/>
-    <hyperlink r:id="rId33" ref="C30"/>
-    <hyperlink r:id="rId34" ref="C31"/>
-    <hyperlink r:id="rId35" ref="C32"/>
-    <hyperlink r:id="rId36" ref="C33"/>
-    <hyperlink r:id="rId37" ref="C34"/>
-    <hyperlink r:id="rId38" ref="C35"/>
-    <hyperlink r:id="rId39" ref="C36"/>
-    <hyperlink r:id="rId40" ref="C37"/>
-    <hyperlink r:id="rId41" ref="C38"/>
-    <hyperlink r:id="rId42" ref="C39"/>
-    <hyperlink r:id="rId43" ref="C40"/>
-    <hyperlink r:id="rId44" ref="C41"/>
-    <hyperlink r:id="rId45" ref="C42"/>
-    <hyperlink r:id="rId46" ref="C43"/>
-    <hyperlink r:id="rId47" ref="C44"/>
-    <hyperlink r:id="rId48" ref="C45"/>
-    <hyperlink r:id="rId49" ref="C46"/>
-    <hyperlink r:id="rId50" ref="C47"/>
-    <hyperlink r:id="rId51" ref="C48"/>
-    <hyperlink r:id="rId52" ref="C49"/>
-    <hyperlink r:id="rId53" ref="C50"/>
-    <hyperlink r:id="rId54" ref="C51"/>
-    <hyperlink r:id="rId55" ref="C52"/>
-    <hyperlink r:id="rId56" ref="C53"/>
-    <hyperlink r:id="rId57" ref="C56"/>
-    <hyperlink r:id="rId58" ref="C57"/>
-  </hyperlinks>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
-  <drawing r:id="rId59"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
@@ -4591,18 +2744,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J2" s="6">
         <v>6.0</v>
@@ -4610,13 +2763,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J3" s="6">
         <v>1.0</v>
@@ -4624,13 +2777,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J4" s="6">
         <v>1.0</v>
@@ -4638,21 +2791,21 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J6" s="6">
         <v>2.0</v>
@@ -4660,13 +2813,13 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J7" s="6">
         <v>1.0</v>
@@ -4674,13 +2827,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J8" s="6">
         <v>1.0</v>
@@ -4688,42 +2841,42 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J14" s="6">
         <v>2.0</v>
@@ -4731,13 +2884,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J15" s="6">
         <v>2.0</v>
@@ -4745,21 +2898,21 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="J17" s="6">
         <v>3.0</v>
@@ -4767,13 +2920,13 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="J18" s="6">
         <v>2.0</v>
@@ -4781,26 +2934,26 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 06-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="174">
   <si>
     <t>date</t>
   </si>
@@ -477,6 +477,30 @@
   </si>
   <si>
     <t>Trabajo de Fuerza, Juego de Centros y Transiciones D-A , A-D</t>
+  </si>
+  <si>
+    <t>https://youtu.be/7HBr7Vxj_kA</t>
+  </si>
+  <si>
+    <t>Turno unico 2:30 pm</t>
+  </si>
+  <si>
+    <t>Trabajo de velocidad - Juego 11 vs11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/3Z_xecPmSew</t>
+  </si>
+  <si>
+    <t>Activación 06/05</t>
+  </si>
+  <si>
+    <t>https://youtu.be/hC8wydyucPk</t>
+  </si>
+  <si>
+    <t>ABPs</t>
+  </si>
+  <si>
+    <t>Corner y Tiro libre lateral</t>
   </si>
   <si>
     <t>VERDE</t>
@@ -1715,9 +1739,45 @@
         <v>134</v>
       </c>
     </row>
-    <row r="56" ht="15.75" customHeight="1"/>
-    <row r="57" ht="15.75" customHeight="1"/>
-    <row r="58" ht="15.75" customHeight="1"/>
+    <row r="56" ht="15.75" customHeight="1">
+      <c r="A56" s="13">
+        <v>46147.0</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customHeight="1">
+      <c r="A57" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customHeight="1">
+      <c r="A58" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
     <row r="59" ht="15.75" customHeight="1"/>
     <row r="60" ht="15.75" customHeight="1"/>
     <row r="61" ht="15.75" customHeight="1"/>
@@ -2724,11 +2784,14 @@
     <hyperlink r:id="rId56" ref="C53"/>
     <hyperlink r:id="rId57" ref="C54"/>
     <hyperlink r:id="rId58" ref="C55"/>
+    <hyperlink r:id="rId59" ref="C56"/>
+    <hyperlink r:id="rId60" ref="C57"/>
+    <hyperlink r:id="rId61" ref="C58"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId59"/>
+  <drawing r:id="rId62"/>
 </worksheet>
 </file>
 
@@ -2744,18 +2807,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="6" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="J2" s="6">
         <v>6.0</v>
@@ -2763,13 +2826,13 @@
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="J3" s="6">
         <v>1.0</v>
@@ -2777,13 +2840,13 @@
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="J4" s="6">
         <v>1.0</v>
@@ -2791,21 +2854,21 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="J6" s="6">
         <v>2.0</v>
@@ -2813,13 +2876,13 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>141</v>
       </c>
       <c r="J7" s="6">
         <v>1.0</v>
@@ -2827,13 +2890,13 @@
     </row>
     <row r="8">
       <c r="A8" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="J8" s="6">
         <v>1.0</v>
@@ -2841,42 +2904,42 @@
     </row>
     <row r="9">
       <c r="A9" s="6" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="J14" s="6">
         <v>2.0</v>
@@ -2884,13 +2947,13 @@
     </row>
     <row r="15">
       <c r="A15" s="6" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="J15" s="6">
         <v>2.0</v>
@@ -2898,21 +2961,21 @@
     </row>
     <row r="16">
       <c r="A16" s="6" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>146</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="J17" s="6">
         <v>3.0</v>
@@ -2920,13 +2983,13 @@
     </row>
     <row r="18">
       <c r="A18" s="6" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="J18" s="6">
         <v>2.0</v>
@@ -2934,26 +2997,26 @@
     </row>
     <row r="19">
       <c r="A19" s="6" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add entrenamiento hasta 06-05 correct2
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -4,20 +4,19 @@
   <workbookPr/>
   <sheets>
     <sheet state="visible" name="Hoja1" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="Hoja x" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId6" roundtripDataChecksum="hoF12/XSjhOFQCYc+u+CyOYasShuanztpa6csxB8U0U="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="DO90dd5CGuJTL/RrjZQQ/iy4IEtBn3yIhi3moFPZHOo="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="143">
   <si>
     <t>date</t>
   </si>
@@ -501,99 +500,6 @@
   </si>
   <si>
     <t>Corner y Tiro libre lateral</t>
-  </si>
-  <si>
-    <t>VERDE</t>
-  </si>
-  <si>
-    <t>centro-izquierda</t>
-  </si>
-  <si>
-    <t>centro impreciso  desde izquierda</t>
-  </si>
-  <si>
-    <t>derecha</t>
-  </si>
-  <si>
-    <t>centro-derecha</t>
-  </si>
-  <si>
-    <t>centro bloqueado desde derecha</t>
-  </si>
-  <si>
-    <t>izquierda</t>
-  </si>
-  <si>
-    <t>derecha | derecha</t>
-  </si>
-  <si>
-    <t>centro bloqueado derecha, centro impreciso derecha</t>
-  </si>
-  <si>
-    <t>medio</t>
-  </si>
-  <si>
-    <t>perdida, remate en contra</t>
-  </si>
-  <si>
-    <t>centro-derecha baja</t>
-  </si>
-  <si>
-    <t>lanzamiento, segunda bola remate</t>
-  </si>
-  <si>
-    <t>centro-derecha-izquierda-derecha</t>
-  </si>
-  <si>
-    <t>centro y remate</t>
-  </si>
-  <si>
-    <t>centro</t>
-  </si>
-  <si>
-    <t>perdida</t>
-  </si>
-  <si>
-    <t>medio-derecha | derecha-centro-derecha</t>
-  </si>
-  <si>
-    <t>perdida, recuperacion, centro derecha, remate en contra, transicion ofensiva por derecha centro</t>
-  </si>
-  <si>
-    <t>centro-izquierda-derecha-centro</t>
-  </si>
-  <si>
-    <t>offside</t>
-  </si>
-  <si>
-    <t>NARANJA</t>
-  </si>
-  <si>
-    <t>izquierda-izquierda</t>
-  </si>
-  <si>
-    <t>centro y gol</t>
-  </si>
-  <si>
-    <t>medio-izquierda</t>
-  </si>
-  <si>
-    <t>centro impreciso</t>
-  </si>
-  <si>
-    <t>lanzamiento y perdida</t>
-  </si>
-  <si>
-    <t>centro-derecha | izquierd</t>
-  </si>
-  <si>
-    <t>perdida , recuperacio, perdida</t>
-  </si>
-  <si>
-    <t>izquierda-perdida | derecha</t>
-  </si>
-  <si>
-    <t>perdida | recuperacion y perdida en el medio y remate en contra</t>
   </si>
 </sst>
 </file>
@@ -767,10 +673,6 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -2793,233 +2695,4 @@
   <pageSetup orientation="landscape"/>
   <drawing r:id="rId62"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
-  </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="36.57"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="J2" s="6">
-        <v>6.0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="J3" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="J4" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="J6" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="J7" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="J8" s="6">
-        <v>1.0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="J14" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="J15" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="J17" s="6">
-        <v>3.0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="J18" s="6">
-        <v>2.0</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>173</v>
-      </c>
-    </row>
-  </sheetData>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
add entrenamiento hasta 06-05 correct3
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -1657,7 +1657,7 @@
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="13">
-        <v>46179.0</v>
+        <v>46148.0</v>
       </c>
       <c r="C57" s="7" t="s">
         <v>138</v>
@@ -1668,7 +1668,7 @@
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="13">
-        <v>46179.0</v>
+        <v>46148.0</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>140</v>

</xml_diff>

<commit_message>
add entrenamiento hasta 11/05 turno mañana
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="153">
   <si>
     <t>date</t>
   </si>
@@ -500,6 +500,36 @@
   </si>
   <si>
     <t>Corner y Tiro libre lateral</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bey02ugnB4U</t>
+  </si>
+  <si>
+    <t>Amistoso vs Liberty schoool</t>
+  </si>
+  <si>
+    <t>Partido amistos en Moquegua</t>
+  </si>
+  <si>
+    <t>https://youtu.be/VlC2L9ODx1Q</t>
+  </si>
+  <si>
+    <t>Entrenamiento 4:00 p.m</t>
+  </si>
+  <si>
+    <t>https://youtu.be/fh7C4BXJDJg</t>
+  </si>
+  <si>
+    <t>1er Turno 9:00 a.m</t>
+  </si>
+  <si>
+    <t>Entrenamiento de resistencia</t>
+  </si>
+  <si>
+    <t>2do Turno 3:00 pm</t>
+  </si>
+  <si>
+    <t>//</t>
   </si>
 </sst>
 </file>
@@ -1680,10 +1710,56 @@
         <v>142</v>
       </c>
     </row>
-    <row r="59" ht="15.75" customHeight="1"/>
-    <row r="60" ht="15.75" customHeight="1"/>
-    <row r="61" ht="15.75" customHeight="1"/>
-    <row r="62" ht="15.75" customHeight="1"/>
+    <row r="59" ht="15.75" customHeight="1">
+      <c r="A59" s="13">
+        <v>46149.0</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="60" ht="15.75" customHeight="1">
+      <c r="A60" s="13">
+        <v>46150.0</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="61" ht="15.75" customHeight="1">
+      <c r="A61" s="13">
+        <v>46153.0</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="D61" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E61" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="62" ht="15.75" customHeight="1">
+      <c r="A62" s="13">
+        <v>46153.0</v>
+      </c>
+      <c r="D62" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="O62" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
     <row r="63" ht="15.75" customHeight="1"/>
     <row r="64" ht="15.75" customHeight="1"/>
     <row r="65" ht="15.75" customHeight="1"/>
@@ -2689,10 +2765,13 @@
     <hyperlink r:id="rId59" ref="C56"/>
     <hyperlink r:id="rId60" ref="C57"/>
     <hyperlink r:id="rId61" ref="C58"/>
+    <hyperlink r:id="rId62" ref="C59"/>
+    <hyperlink r:id="rId63" ref="C60"/>
+    <hyperlink r:id="rId64" ref="C61"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId62"/>
+  <drawing r:id="rId65"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add entrenamiento hasta 11/05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="156">
   <si>
     <t>date</t>
   </si>
@@ -365,11 +365,31 @@
     <t>1ER TURNO - 9am</t>
   </si>
   <si>
-    <t>Entrenamiento del 23 de abril 
-Fase de Activación: 20 minutos de carrera continua - trabajo de resistencia, arte principal:
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Entrenamiento del 23 de abril 
+Fase de Activación: 20 minutos de carrera continua - trabajo de resistencia. Arte principal:
 Juego reducido 11VS11
-Equipo blanco:
-1. taylor /Bebote 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Equipo blanco
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">1. Taylor /Bebote 
 2. ⁠cueva
 3. ⁠acasiete
 4. ⁠casas 
@@ -380,8 +400,23 @@
 9. ⁠centurión 
 10. ⁠Jair
 11. ⁠Joaquín 
-Equipo verde
-1. Escalante/Eden
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t xml:space="preserve">Equipo verde
+</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+      </rPr>
+      <t>1. Escalante/Eden
 2. ⁠Perea
 3. ⁠Joaquín 
 4. ⁠Fernández
@@ -392,6 +427,7 @@
 9. ⁠Pedro
 10. ⁠Zúñiga 
 11. ⁠castro</t>
+    </r>
   </si>
   <si>
     <t>https://youtu.be/2A5FJYTC-Q0</t>
@@ -400,6 +436,9 @@
     <t>2DO TURNO - 4:30P.M</t>
   </si>
   <si>
+    <t>https://youtu.be/RspyfOY3NLM</t>
+  </si>
+  <si>
     <t>https://youtu.be/bXof8DRI8G0</t>
   </si>
   <si>
@@ -436,7 +475,7 @@
     <t>https://youtu.be/pn7qxeSxgVc</t>
   </si>
   <si>
-    <t>Turno único 8am</t>
+    <t>Porteros - Turno único</t>
   </si>
   <si>
     <t>Porteros</t>
@@ -445,12 +484,32 @@
     <t>https://youtu.be/05XeMi_68Mo</t>
   </si>
   <si>
-    <t>Cambios de orientación, centros y definición</t>
+    <t>Centros - Turno único</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <b/>
+        <color theme="1"/>
+      </rPr>
+      <t>Cambios de orientación, centros y definición</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Calibri"/>
+        <color theme="1"/>
+      </rPr>
+      <t>. El porcentaje de efectividad de los centros (sin oposición) fue de 35.5% a nivel de equipo</t>
+    </r>
   </si>
   <si>
     <t>https://youtu.be/KHLU3IBqzs4</t>
   </si>
   <si>
+    <t>Reducido - Turno único</t>
+  </si>
+  <si>
     <t>https://youtu.be/ppDobsGo3Yg</t>
   </si>
   <si>
@@ -508,7 +567,7 @@
     <t>Amistoso vs Liberty schoool</t>
   </si>
   <si>
-    <t>Partido amistos en Moquegua</t>
+    <t>Partido amistos vs Liberty (Moquegua)</t>
   </si>
   <si>
     <t>https://youtu.be/VlC2L9ODx1Q</t>
@@ -1530,19 +1589,22 @@
       <c r="D45" s="6" t="s">
         <v>108</v>
       </c>
+      <c r="E45" s="7" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="13">
         <v>46136.0</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
@@ -1550,13 +1612,13 @@
         <v>46136.0</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -1564,13 +1626,13 @@
         <v>46136.0</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
@@ -1578,13 +1640,13 @@
         <v>46137.0</v>
       </c>
       <c r="C49" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E49" s="6" t="s">
         <v>118</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
@@ -1592,13 +1654,13 @@
         <v>46138.0</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
@@ -1606,13 +1668,13 @@
         <v>46138.0</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
@@ -1620,27 +1682,25 @@
         <v>46138.0</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>18</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="E52" s="6"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="13">
         <v>46140.0</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
@@ -1648,13 +1708,13 @@
         <v>46143.0</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
@@ -1662,13 +1722,13 @@
         <v>46146.0</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
@@ -1676,13 +1736,13 @@
         <v>46147.0</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -1690,10 +1750,10 @@
         <v>46148.0</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -1701,13 +1761,13 @@
         <v>46148.0</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
@@ -1715,13 +1775,13 @@
         <v>46149.0</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -1729,10 +1789,10 @@
         <v>46150.0</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
@@ -1740,13 +1800,13 @@
         <v>46153.0</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
@@ -1754,10 +1814,10 @@
         <v>46153.0</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1"/>
@@ -2752,26 +2812,27 @@
     <hyperlink r:id="rId46" ref="C43"/>
     <hyperlink r:id="rId47" ref="C44"/>
     <hyperlink r:id="rId48" ref="C45"/>
-    <hyperlink r:id="rId49" ref="C46"/>
-    <hyperlink r:id="rId50" ref="C47"/>
-    <hyperlink r:id="rId51" ref="C48"/>
-    <hyperlink r:id="rId52" ref="C49"/>
-    <hyperlink r:id="rId53" ref="C50"/>
-    <hyperlink r:id="rId54" ref="C51"/>
-    <hyperlink r:id="rId55" ref="C52"/>
-    <hyperlink r:id="rId56" ref="C53"/>
-    <hyperlink r:id="rId57" ref="C54"/>
-    <hyperlink r:id="rId58" ref="C55"/>
-    <hyperlink r:id="rId59" ref="C56"/>
-    <hyperlink r:id="rId60" ref="C57"/>
-    <hyperlink r:id="rId61" ref="C58"/>
-    <hyperlink r:id="rId62" ref="C59"/>
-    <hyperlink r:id="rId63" ref="C60"/>
-    <hyperlink r:id="rId64" ref="C61"/>
+    <hyperlink r:id="rId49" ref="E45"/>
+    <hyperlink r:id="rId50" ref="C46"/>
+    <hyperlink r:id="rId51" ref="C47"/>
+    <hyperlink r:id="rId52" ref="C48"/>
+    <hyperlink r:id="rId53" ref="C49"/>
+    <hyperlink r:id="rId54" ref="C50"/>
+    <hyperlink r:id="rId55" ref="C51"/>
+    <hyperlink r:id="rId56" ref="C52"/>
+    <hyperlink r:id="rId57" ref="C53"/>
+    <hyperlink r:id="rId58" ref="C54"/>
+    <hyperlink r:id="rId59" ref="C55"/>
+    <hyperlink r:id="rId60" ref="C56"/>
+    <hyperlink r:id="rId61" ref="C57"/>
+    <hyperlink r:id="rId62" ref="C58"/>
+    <hyperlink r:id="rId63" ref="C59"/>
+    <hyperlink r:id="rId64" ref="C60"/>
+    <hyperlink r:id="rId65" ref="C61"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId65"/>
+  <drawing r:id="rId66"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add entrenamiento hasta 11/05 2do turno
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="163">
   <si>
     <t>date</t>
   </si>
@@ -585,10 +585,31 @@
     <t>Entrenamiento de resistencia</t>
   </si>
   <si>
-    <t>2do Turno 3:00 pm</t>
+    <t>https://youtu.be/CdhE6Pk3Qvk</t>
+  </si>
+  <si>
+    <t>2do Turno - activación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rondos </t>
   </si>
   <si>
     <t>//</t>
+  </si>
+  <si>
+    <t>2do Turno - Salida (prueba en vacio)</t>
+  </si>
+  <si>
+    <t>Salida de balón - prueba en vació</t>
+  </si>
+  <si>
+    <t>https://youtu.be/cPF7Sij2ZBk</t>
+  </si>
+  <si>
+    <t>2do Turno - Salida real</t>
+  </si>
+  <si>
+    <t>Salida de balón: estructura y movimientos</t>
   </si>
 </sst>
 </file>
@@ -1813,15 +1834,44 @@
       <c r="A62" s="13">
         <v>46153.0</v>
       </c>
+      <c r="C62" s="7" t="s">
+        <v>154</v>
+      </c>
       <c r="D62" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
+      </c>
+      <c r="E62" s="6" t="s">
+        <v>156</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="63" ht="15.75" customHeight="1"/>
-    <row r="64" ht="15.75" customHeight="1"/>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="63" ht="15.75" customHeight="1">
+      <c r="A63" s="13">
+        <v>46153.0</v>
+      </c>
+      <c r="D63" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="E63" s="6" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="64" ht="15.75" customHeight="1">
+      <c r="A64" s="13">
+        <v>46153.0</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="D64" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="E64" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1"/>
@@ -2829,10 +2879,12 @@
     <hyperlink r:id="rId63" ref="C59"/>
     <hyperlink r:id="rId64" ref="C60"/>
     <hyperlink r:id="rId65" ref="C61"/>
+    <hyperlink r:id="rId66" ref="C62"/>
+    <hyperlink r:id="rId67" ref="C64"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId66"/>
+  <drawing r:id="rId68"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add entrenamiento hasta 12/05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="165">
   <si>
     <t>date</t>
   </si>
@@ -610,6 +610,12 @@
   </si>
   <si>
     <t>Salida de balón: estructura y movimientos</t>
+  </si>
+  <si>
+    <t>https://youtu.be/qES7G7-s39Q</t>
+  </si>
+  <si>
+    <t>Turno único</t>
   </si>
 </sst>
 </file>
@@ -1872,7 +1878,17 @@
         <v>162</v>
       </c>
     </row>
-    <row r="65" ht="15.75" customHeight="1"/>
+    <row r="65" ht="15.75" customHeight="1">
+      <c r="A65" s="13">
+        <v>46154.0</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D65" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
     <row r="66" ht="15.75" customHeight="1"/>
     <row r="67" ht="15.75" customHeight="1"/>
     <row r="68" ht="15.75" customHeight="1"/>
@@ -2881,10 +2897,11 @@
     <hyperlink r:id="rId65" ref="C61"/>
     <hyperlink r:id="rId66" ref="C62"/>
     <hyperlink r:id="rId67" ref="C64"/>
+    <hyperlink r:id="rId68" ref="C65"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId68"/>
+  <drawing r:id="rId69"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add entrenamiento hasta 12/05 new video
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -612,7 +612,7 @@
     <t>Salida de balón: estructura y movimientos</t>
   </si>
   <si>
-    <t>https://youtu.be/qES7G7-s39Q</t>
+    <t>https://youtu.be/47_QGKmmLw4</t>
   </si>
   <si>
     <t>Turno único</t>
@@ -627,7 +627,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -698,6 +698,10 @@
       <u/>
       <color rgb="FF0000FF"/>
     </font>
+    <font>
+      <u/>
+      <color rgb="FF0563C1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -719,7 +723,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -778,6 +782,9 @@
     </xf>
     <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1882,7 +1889,7 @@
       <c r="A65" s="13">
         <v>46154.0</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="C65" s="22" t="s">
         <v>163</v>
       </c>
       <c r="D65" s="6" t="s">

</xml_diff>

<commit_message>
videos de entrenamientos hasta 15-05, falta 14-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="167">
   <si>
     <t>date</t>
   </si>
@@ -616,6 +616,12 @@
   </si>
   <si>
     <t>Turno único</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/VSLhcOEX8ho </t>
+  </si>
+  <si>
+    <t>Amistoso A vs B</t>
   </si>
 </sst>
 </file>
@@ -1896,7 +1902,17 @@
         <v>164</v>
       </c>
     </row>
-    <row r="66" ht="15.75" customHeight="1"/>
+    <row r="66" ht="15.75" customHeight="1">
+      <c r="A66" s="13">
+        <v>46157.0</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="D66" s="6" t="s">
+        <v>166</v>
+      </c>
+    </row>
     <row r="67" ht="15.75" customHeight="1"/>
     <row r="68" ht="15.75" customHeight="1"/>
     <row r="69" ht="15.75" customHeight="1"/>
@@ -2905,10 +2921,11 @@
     <hyperlink r:id="rId66" ref="C62"/>
     <hyperlink r:id="rId67" ref="C64"/>
     <hyperlink r:id="rId68" ref="C65"/>
+    <hyperlink r:id="rId69" ref="C66"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId69"/>
+  <drawing r:id="rId70"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamiento hasta 18-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="170">
   <si>
     <t>date</t>
   </si>
@@ -623,6 +623,15 @@
   <si>
     <t>Amistoso A vs B</t>
   </si>
+  <si>
+    <t>https://youtu.be/sVRy3ma9PpQ</t>
+  </si>
+  <si>
+    <t>11 vs 11 - 18/05/26</t>
+  </si>
+  <si>
+    <t>Libre 11 vs 11</t>
+  </si>
 </sst>
 </file>
 
@@ -633,7 +642,7 @@
     <numFmt numFmtId="165" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -708,8 +717,12 @@
       <u/>
       <color rgb="FF0563C1"/>
     </font>
+    <font>
+      <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -722,14 +735,34 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -792,6 +825,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="15" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1913,11 +1949,35 @@
         <v>166</v>
       </c>
     </row>
-    <row r="67" ht="15.75" customHeight="1"/>
+    <row r="67" ht="15.75" customHeight="1">
+      <c r="A67" s="13">
+        <v>46160.0</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="D67" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E67" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
     <row r="68" ht="15.75" customHeight="1"/>
     <row r="69" ht="15.75" customHeight="1"/>
     <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1"/>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="D71" s="23"/>
+      <c r="E71" s="23"/>
+      <c r="F71" s="23"/>
+      <c r="G71" s="23"/>
+      <c r="H71" s="23"/>
+      <c r="I71" s="23"/>
+      <c r="J71" s="23"/>
+      <c r="K71" s="23"/>
+      <c r="L71" s="23"/>
+      <c r="M71" s="23"/>
+    </row>
     <row r="72" ht="15.75" customHeight="1"/>
     <row r="73" ht="15.75" customHeight="1"/>
     <row r="74" ht="15.75" customHeight="1"/>
@@ -2922,10 +2982,11 @@
     <hyperlink r:id="rId67" ref="C64"/>
     <hyperlink r:id="rId68" ref="C65"/>
     <hyperlink r:id="rId69" ref="C66"/>
+    <hyperlink r:id="rId70" ref="C67"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId70"/>
+  <drawing r:id="rId71"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamiento hasta 19-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="173">
   <si>
     <t>date</t>
   </si>
@@ -631,6 +631,15 @@
   </si>
   <si>
     <t>Libre 11 vs 11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/LGVYMTdnvps</t>
+  </si>
+  <si>
+    <t>11 vs 11 - 19/05/26</t>
+  </si>
+  <si>
+    <t>Equipo A  vs Equipo B. Equipo A vs Equipo "aprueba"</t>
   </si>
 </sst>
 </file>
@@ -1963,7 +1972,20 @@
         <v>169</v>
       </c>
     </row>
-    <row r="68" ht="15.75" customHeight="1"/>
+    <row r="68" ht="15.75" customHeight="1">
+      <c r="A68" s="13">
+        <v>46161.0</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="D68" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="E68" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
     <row r="69" ht="15.75" customHeight="1"/>
     <row r="70" ht="15.75" customHeight="1"/>
     <row r="71" ht="15.75" customHeight="1">
@@ -2983,10 +3005,11 @@
     <hyperlink r:id="rId68" ref="C65"/>
     <hyperlink r:id="rId69" ref="C66"/>
     <hyperlink r:id="rId70" ref="C67"/>
+    <hyperlink r:id="rId71" ref="C68"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId71"/>
+  <drawing r:id="rId72"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamiento hasta 21-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="176">
   <si>
     <t>date</t>
   </si>
@@ -640,6 +640,15 @@
   </si>
   <si>
     <t>Equipo A  vs Equipo B. Equipo A vs Equipo "a prueba"</t>
+  </si>
+  <si>
+    <t>https://youtu.be/EK7GF8KsKNo</t>
+  </si>
+  <si>
+    <t>Partido amistoso</t>
+  </si>
+  <si>
+    <t>Amistos vs Sportivo Huracán</t>
   </si>
 </sst>
 </file>
@@ -1986,7 +1995,20 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" ht="15.75" customHeight="1"/>
+    <row r="69" ht="15.75" customHeight="1">
+      <c r="A69" s="13">
+        <v>46163.0</v>
+      </c>
+      <c r="C69" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="D69" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
     <row r="70" ht="15.75" customHeight="1"/>
     <row r="71" ht="15.75" customHeight="1">
       <c r="D71" s="23"/>
@@ -3006,10 +3028,11 @@
     <hyperlink r:id="rId69" ref="C66"/>
     <hyperlink r:id="rId70" ref="C67"/>
     <hyperlink r:id="rId71" ref="C68"/>
+    <hyperlink r:id="rId72" ref="C69"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId72"/>
+  <drawing r:id="rId73"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamiento hasta 23-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="DO90dd5CGuJTL/RrjZQQ/iy4IEtBn3yIhi3moFPZHOo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="QNr4uAtfhwsnYdsjUHW0ONuTij7TZqiGYsaXq6Jz+sA="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="180">
   <si>
     <t>date</t>
   </si>
@@ -597,12 +597,6 @@
     <t>//</t>
   </si>
   <si>
-    <t>2do Turno - Salida (prueba en vacio)</t>
-  </si>
-  <si>
-    <t>Salida de balón - prueba en vació</t>
-  </si>
-  <si>
     <t>https://youtu.be/cPF7Sij2ZBk</t>
   </si>
   <si>
@@ -649,6 +643,24 @@
   </si>
   <si>
     <t>Amistos vs Sportivo Huracán</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-7p876MvXF8</t>
+  </si>
+  <si>
+    <t>Salida 23-05</t>
+  </si>
+  <si>
+    <t>Salida sin oposición</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Vcp_XV58azM</t>
+  </si>
+  <si>
+    <t>ABPs  23-05</t>
+  </si>
+  <si>
+    <t>Practicando ABP (corners, tiros libres y penales)</t>
   </si>
 </sst>
 </file>
@@ -780,7 +792,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -845,6 +857,9 @@
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="1" fillId="3" fontId="15" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="15" numFmtId="49" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment shrinkToFit="0" wrapText="0"/>
     </xf>
   </cellXfs>
@@ -1924,32 +1939,32 @@
       <c r="A63" s="13">
         <v>46153.0</v>
       </c>
+      <c r="C63" s="7" t="s">
+        <v>158</v>
+      </c>
       <c r="D63" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="13">
-        <v>46153.0</v>
-      </c>
-      <c r="C64" s="7" t="s">
-        <v>160</v>
+        <v>46154.0</v>
+      </c>
+      <c r="C64" s="22" t="s">
+        <v>161</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="E64" s="6" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="13">
-        <v>46154.0</v>
-      </c>
-      <c r="C65" s="22" t="s">
+        <v>46157.0</v>
+      </c>
+      <c r="C65" s="7" t="s">
         <v>163</v>
       </c>
       <c r="D65" s="6" t="s">
@@ -1958,7 +1973,7 @@
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="13">
-        <v>46157.0</v>
+        <v>46160.0</v>
       </c>
       <c r="C66" s="7" t="s">
         <v>165</v>
@@ -1966,62 +1981,75 @@
       <c r="D66" s="6" t="s">
         <v>166</v>
       </c>
+      <c r="E66" s="6" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="13">
-        <v>46160.0</v>
+        <v>46161.0</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="13">
-        <v>46161.0</v>
+        <v>46163.0</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="13">
-        <v>46163.0</v>
+        <v>46076.0</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="70" ht="15.75" customHeight="1"/>
-    <row r="71" ht="15.75" customHeight="1">
-      <c r="D71" s="23"/>
-      <c r="E71" s="23"/>
-      <c r="F71" s="23"/>
-      <c r="G71" s="23"/>
-      <c r="H71" s="23"/>
-      <c r="I71" s="23"/>
-      <c r="J71" s="23"/>
-      <c r="K71" s="23"/>
-      <c r="L71" s="23"/>
-      <c r="M71" s="23"/>
-    </row>
+        <v>176</v>
+      </c>
+    </row>
+    <row r="70" ht="15.75" customHeight="1">
+      <c r="A70" s="13">
+        <v>46076.0</v>
+      </c>
+      <c r="C70" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="D70" s="23" t="s">
+        <v>178</v>
+      </c>
+      <c r="E70" s="23" t="s">
+        <v>179</v>
+      </c>
+      <c r="F70" s="24"/>
+      <c r="G70" s="24"/>
+      <c r="H70" s="24"/>
+      <c r="I70" s="24"/>
+      <c r="J70" s="24"/>
+      <c r="K70" s="24"/>
+      <c r="L70" s="24"/>
+      <c r="M70" s="24"/>
+    </row>
+    <row r="71" ht="15.75" customHeight="1"/>
     <row r="72" ht="15.75" customHeight="1"/>
     <row r="73" ht="15.75" customHeight="1"/>
     <row r="74" ht="15.75" customHeight="1"/>
@@ -2954,7 +2982,6 @@
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
     <row r="1003" ht="15.75" customHeight="1"/>
-    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3023,16 +3050,18 @@
     <hyperlink r:id="rId64" ref="C60"/>
     <hyperlink r:id="rId65" ref="C61"/>
     <hyperlink r:id="rId66" ref="C62"/>
-    <hyperlink r:id="rId67" ref="C64"/>
-    <hyperlink r:id="rId68" ref="C65"/>
-    <hyperlink r:id="rId69" ref="C66"/>
-    <hyperlink r:id="rId70" ref="C67"/>
-    <hyperlink r:id="rId71" ref="C68"/>
-    <hyperlink r:id="rId72" ref="C69"/>
+    <hyperlink r:id="rId67" ref="C63"/>
+    <hyperlink r:id="rId68" ref="C64"/>
+    <hyperlink r:id="rId69" ref="C65"/>
+    <hyperlink r:id="rId70" ref="C66"/>
+    <hyperlink r:id="rId71" ref="C67"/>
+    <hyperlink r:id="rId72" ref="C68"/>
+    <hyperlink r:id="rId73" ref="C69"/>
+    <hyperlink r:id="rId74" ref="C70"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId73"/>
+  <drawing r:id="rId75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamiento hasta 23-05 v2
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="QNr4uAtfhwsnYdsjUHW0ONuTij7TZqiGYsaXq6Jz+sA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="DO90dd5CGuJTL/RrjZQQ/iy4IEtBn3yIhi3moFPZHOo="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="183">
   <si>
     <t>date</t>
   </si>
@@ -616,6 +616,15 @@
   </si>
   <si>
     <t>Amistoso A vs B</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-zf5eWAEF_w</t>
+  </si>
+  <si>
+    <t>11 vs 11 con condición</t>
+  </si>
+  <si>
+    <t>11 vs 11 con condición || 23-05-26</t>
   </si>
   <si>
     <t>https://youtu.be/sVRy3ma9PpQ</t>
@@ -1987,7 +1996,7 @@
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="13">
-        <v>46161.0</v>
+        <v>46160.0</v>
       </c>
       <c r="C67" s="7" t="s">
         <v>168</v>
@@ -2001,7 +2010,7 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="13">
-        <v>46163.0</v>
+        <v>46161.0</v>
       </c>
       <c r="C68" s="7" t="s">
         <v>171</v>
@@ -2015,7 +2024,7 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="13">
-        <v>46076.0</v>
+        <v>46163.0</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>174</v>
@@ -2034,22 +2043,35 @@
       <c r="C70" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="D70" s="23" t="s">
+      <c r="D70" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="E70" s="23" t="s">
+      <c r="E70" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="F70" s="24"/>
-      <c r="G70" s="24"/>
-      <c r="H70" s="24"/>
-      <c r="I70" s="24"/>
-      <c r="J70" s="24"/>
-      <c r="K70" s="24"/>
-      <c r="L70" s="24"/>
-      <c r="M70" s="24"/>
-    </row>
-    <row r="71" ht="15.75" customHeight="1"/>
+    </row>
+    <row r="71" ht="15.75" customHeight="1">
+      <c r="A71" s="13">
+        <v>46076.0</v>
+      </c>
+      <c r="C71" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="D71" s="23" t="s">
+        <v>181</v>
+      </c>
+      <c r="E71" s="23" t="s">
+        <v>182</v>
+      </c>
+      <c r="F71" s="24"/>
+      <c r="G71" s="24"/>
+      <c r="H71" s="24"/>
+      <c r="I71" s="24"/>
+      <c r="J71" s="24"/>
+      <c r="K71" s="24"/>
+      <c r="L71" s="24"/>
+      <c r="M71" s="24"/>
+    </row>
     <row r="72" ht="15.75" customHeight="1"/>
     <row r="73" ht="15.75" customHeight="1"/>
     <row r="74" ht="15.75" customHeight="1"/>
@@ -2982,6 +3004,7 @@
     <row r="1001" ht="15.75" customHeight="1"/>
     <row r="1002" ht="15.75" customHeight="1"/>
     <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3058,10 +3081,11 @@
     <hyperlink r:id="rId72" ref="C68"/>
     <hyperlink r:id="rId73" ref="C69"/>
     <hyperlink r:id="rId74" ref="C70"/>
+    <hyperlink r:id="rId75" ref="C71"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId75"/>
+  <drawing r:id="rId76"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamiento hasta 23-05 corregido
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -2038,7 +2038,7 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="13">
-        <v>46076.0</v>
+        <v>46165.0</v>
       </c>
       <c r="C70" s="7" t="s">
         <v>177</v>
@@ -2052,7 +2052,7 @@
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="13">
-        <v>46076.0</v>
+        <v>46165.0</v>
       </c>
       <c r="C71" s="7" t="s">
         <v>180</v>

</xml_diff>

<commit_message>
update entrenamientos hasta 26-05
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="DO90dd5CGuJTL/RrjZQQ/iy4IEtBn3yIhi3moFPZHOo="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="iYnBsaeGnAZvtGM8/noNG3xrTTjpBKqMc/Ub/MqKvT8="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="190">
   <si>
     <t>date</t>
   </si>
@@ -612,6 +612,15 @@
     <t>Turno único</t>
   </si>
   <si>
+    <t>https://youtu.be/OnXQbmlEqUo</t>
+  </si>
+  <si>
+    <t>Definición 14-05</t>
+  </si>
+  <si>
+    <t>Ejercicio de definición 14 de mayo 2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://youtu.be/VSLhcOEX8ho </t>
   </si>
   <si>
@@ -670,6 +679,18 @@
   </si>
   <si>
     <t>Practicando ABP (corners, tiros libres y penales)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/y-_Cd_Pa61k</t>
+  </si>
+  <si>
+    <t>Amistoso vs ANBA</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xy0qpug4-W8</t>
+  </si>
+  <si>
+    <t>Entrenamiento 3pm</t>
   </si>
 </sst>
 </file>
@@ -1971,26 +1992,26 @@
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="13">
-        <v>46157.0</v>
-      </c>
-      <c r="C65" s="7" t="s">
+        <v>46156.0</v>
+      </c>
+      <c r="C65" s="22" t="s">
         <v>163</v>
       </c>
       <c r="D65" s="6" t="s">
         <v>164</v>
       </c>
+      <c r="E65" s="6" t="s">
+        <v>165</v>
+      </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="13">
-        <v>46160.0</v>
+        <v>46157.0</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="E66" s="6" t="s">
         <v>167</v>
       </c>
     </row>
@@ -2010,7 +2031,7 @@
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="13">
-        <v>46161.0</v>
+        <v>46160.0</v>
       </c>
       <c r="C68" s="7" t="s">
         <v>171</v>
@@ -2024,7 +2045,7 @@
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="13">
-        <v>46163.0</v>
+        <v>46161.0</v>
       </c>
       <c r="C69" s="7" t="s">
         <v>174</v>
@@ -2038,7 +2059,7 @@
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="13">
-        <v>46165.0</v>
+        <v>46163.0</v>
       </c>
       <c r="C70" s="7" t="s">
         <v>177</v>
@@ -2057,24 +2078,57 @@
       <c r="C71" s="7" t="s">
         <v>180</v>
       </c>
-      <c r="D71" s="23" t="s">
+      <c r="D71" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E71" s="23" t="s">
+      <c r="E71" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="F71" s="24"/>
-      <c r="G71" s="24"/>
-      <c r="H71" s="24"/>
-      <c r="I71" s="24"/>
-      <c r="J71" s="24"/>
-      <c r="K71" s="24"/>
-      <c r="L71" s="24"/>
-      <c r="M71" s="24"/>
-    </row>
-    <row r="72" ht="15.75" customHeight="1"/>
-    <row r="73" ht="15.75" customHeight="1"/>
-    <row r="74" ht="15.75" customHeight="1"/>
+    </row>
+    <row r="72" ht="15.75" customHeight="1">
+      <c r="A72" s="13">
+        <v>46165.0</v>
+      </c>
+      <c r="C72" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="D72" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="E72" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="F72" s="24"/>
+      <c r="G72" s="24"/>
+      <c r="H72" s="24"/>
+      <c r="I72" s="24"/>
+      <c r="J72" s="24"/>
+      <c r="K72" s="24"/>
+      <c r="L72" s="24"/>
+      <c r="M72" s="24"/>
+    </row>
+    <row r="73" ht="15.75" customHeight="1">
+      <c r="A73" s="13">
+        <v>46166.0</v>
+      </c>
+      <c r="C73" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D73" s="6" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="74" ht="15.75" customHeight="1">
+      <c r="A74" s="13">
+        <v>46168.0</v>
+      </c>
+      <c r="C74" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="D74" s="6" t="s">
+        <v>189</v>
+      </c>
+    </row>
     <row r="75" ht="15.75" customHeight="1"/>
     <row r="76" ht="15.75" customHeight="1"/>
     <row r="77" ht="15.75" customHeight="1"/>
@@ -3005,6 +3059,7 @@
     <row r="1002" ht="15.75" customHeight="1"/>
     <row r="1003" ht="15.75" customHeight="1"/>
     <row r="1004" ht="15.75" customHeight="1"/>
+    <row r="1005" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3082,10 +3137,13 @@
     <hyperlink r:id="rId73" ref="C69"/>
     <hyperlink r:id="rId74" ref="C70"/>
     <hyperlink r:id="rId75" ref="C71"/>
+    <hyperlink r:id="rId76" ref="C72"/>
+    <hyperlink r:id="rId77" ref="C73"/>
+    <hyperlink r:id="rId78" ref="C74"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId76"/>
+  <drawing r:id="rId79"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 03-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="205">
   <si>
     <t>date</t>
   </si>
@@ -519,6 +519,9 @@
     <t>Entrenamiento de resistencia, rueda de pases, juego de posesion</t>
   </si>
   <si>
+    <t>partido</t>
+  </si>
+  <si>
     <t>https://youtu.be/Hod9nJ9w4gM</t>
   </si>
   <si>
@@ -691,6 +694,48 @@
   </si>
   <si>
     <t>Entrenamiento 3pm</t>
+  </si>
+  <si>
+    <t>https://youtu.be/QsdV3CV-klA</t>
+  </si>
+  <si>
+    <t>Entrenamiento 4pm</t>
+  </si>
+  <si>
+    <t>https://youtu.be/e-WhTZ7sMgA</t>
+  </si>
+  <si>
+    <t>Ejercicio de definición</t>
+  </si>
+  <si>
+    <t>Ejercicio de definición con puntaje</t>
+  </si>
+  <si>
+    <t>https://youtu.be/f7cBcoW2CLc</t>
+  </si>
+  <si>
+    <t>Salidas y ABPs a favor</t>
+  </si>
+  <si>
+    <t>Salidas vs presión alta. Salidas vs bloque bajo. Tiros libre laterales a favor. Corners a favor</t>
+  </si>
+  <si>
+    <t>https://youtu.be/j5qjoOjpxuw</t>
+  </si>
+  <si>
+    <t>FECHA 1: vs JM Arguedas</t>
+  </si>
+  <si>
+    <t>Partido oficial en casa</t>
+  </si>
+  <si>
+    <t>https://youtu.be/pzpF7guAzGY</t>
+  </si>
+  <si>
+    <t>Entrenamiento 03-06</t>
+  </si>
+  <si>
+    <t>Turno tarde</t>
   </si>
 </sst>
 </file>
@@ -1109,7 +1154,7 @@
     <col customWidth="1" min="2" max="2" width="14.71"/>
     <col customWidth="1" min="3" max="3" width="45.43"/>
     <col customWidth="1" min="4" max="4" width="36.57"/>
-    <col customWidth="1" min="5" max="5" width="12.0"/>
+    <col customWidth="1" min="5" max="5" width="46.0"/>
     <col customWidth="1" min="6" max="15" width="9.14"/>
   </cols>
   <sheetData>
@@ -1130,7 +1175,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" hidden="1">
       <c r="A2" s="5">
         <v>46087.0</v>
       </c>
@@ -1144,7 +1189,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" hidden="1">
       <c r="A3" s="5">
         <v>46087.0</v>
       </c>
@@ -1158,7 +1203,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" hidden="1">
       <c r="A4" s="5">
         <v>46087.0</v>
       </c>
@@ -1172,7 +1217,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" hidden="1">
       <c r="A5" s="11">
         <v>46092.0</v>
       </c>
@@ -1186,7 +1231,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" hidden="1">
       <c r="A6" s="11">
         <v>46092.0</v>
       </c>
@@ -1200,7 +1245,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" hidden="1">
       <c r="A7" s="11">
         <v>46093.0</v>
       </c>
@@ -1214,7 +1259,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" hidden="1">
       <c r="A8" s="11">
         <v>46093.0</v>
       </c>
@@ -1231,7 +1276,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" hidden="1">
       <c r="A9" s="11">
         <v>46093.0</v>
       </c>
@@ -1248,7 +1293,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" hidden="1">
       <c r="A10" s="11">
         <v>46093.0</v>
       </c>
@@ -1265,7 +1310,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" hidden="1">
       <c r="A11" s="11">
         <v>46094.0</v>
       </c>
@@ -1282,7 +1327,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" hidden="1">
       <c r="A12" s="11">
         <v>46094.0</v>
       </c>
@@ -1299,7 +1344,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" hidden="1">
       <c r="A13" s="11">
         <v>46095.0</v>
       </c>
@@ -1316,7 +1361,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" hidden="1">
       <c r="A14" s="13">
         <v>46097.0</v>
       </c>
@@ -1330,7 +1375,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" hidden="1">
       <c r="A15" s="13">
         <v>46098.0</v>
       </c>
@@ -1344,7 +1389,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" hidden="1">
       <c r="A16" s="13">
         <v>46098.0</v>
       </c>
@@ -1358,7 +1403,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" hidden="1">
       <c r="A17" s="13">
         <v>46098.0</v>
       </c>
@@ -1372,7 +1417,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" hidden="1">
       <c r="A18" s="13">
         <v>46099.0</v>
       </c>
@@ -1387,7 +1432,7 @@
       </c>
       <c r="E18" s="14"/>
     </row>
-    <row r="19">
+    <row r="19" hidden="1">
       <c r="A19" s="13">
         <v>46099.0</v>
       </c>
@@ -1404,7 +1449,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
+    <row r="20" ht="15.75" hidden="1" customHeight="1">
       <c r="A20" s="15">
         <v>46102.0</v>
       </c>
@@ -1419,7 +1464,7 @@
       </c>
       <c r="E20" s="18"/>
     </row>
-    <row r="21" ht="15.75" customHeight="1">
+    <row r="21" ht="15.75" hidden="1" customHeight="1">
       <c r="A21" s="13">
         <v>46103.0</v>
       </c>
@@ -1431,7 +1476,7 @@
       </c>
       <c r="E21" s="14"/>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
+    <row r="22" ht="15.75" hidden="1" customHeight="1">
       <c r="A22" s="13">
         <v>46104.0</v>
       </c>
@@ -1443,7 +1488,7 @@
       </c>
       <c r="E22" s="18"/>
     </row>
-    <row r="23" ht="15.75" customHeight="1">
+    <row r="23" ht="15.75" hidden="1" customHeight="1">
       <c r="A23" s="13">
         <v>46105.0</v>
       </c>
@@ -1455,7 +1500,7 @@
       </c>
       <c r="E23" s="14"/>
     </row>
-    <row r="24" ht="15.75" customHeight="1">
+    <row r="24" ht="15.75" hidden="1" customHeight="1">
       <c r="A24" s="13">
         <v>46106.0</v>
       </c>
@@ -1472,7 +1517,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" ht="15.75" customHeight="1">
+    <row r="25" ht="15.75" hidden="1" customHeight="1">
       <c r="A25" s="13">
         <v>46108.0</v>
       </c>
@@ -1483,7 +1528,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" ht="15.75" customHeight="1">
+    <row r="26" ht="15.75" hidden="1" customHeight="1">
       <c r="A26" s="13">
         <v>46108.0</v>
       </c>
@@ -1497,7 +1542,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1">
+    <row r="27" ht="15.75" hidden="1" customHeight="1">
       <c r="A27" s="13">
         <v>46108.0</v>
       </c>
@@ -1508,7 +1553,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" ht="15.75" customHeight="1">
+    <row r="28" ht="15.75" hidden="1" customHeight="1">
       <c r="A28" s="15">
         <v>46109.0</v>
       </c>
@@ -1520,7 +1565,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" ht="15.75" customHeight="1">
+    <row r="29" ht="15.75" hidden="1" customHeight="1">
       <c r="A29" s="15">
         <v>46113.0</v>
       </c>
@@ -1532,7 +1577,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1">
+    <row r="30" ht="15.75" hidden="1" customHeight="1">
       <c r="A30" s="15">
         <v>46114.0</v>
       </c>
@@ -1544,7 +1589,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1">
+    <row r="31" ht="15.75" hidden="1" customHeight="1">
       <c r="A31" s="13">
         <v>46116.0</v>
       </c>
@@ -1555,7 +1600,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1">
+    <row r="32" ht="15.75" hidden="1" customHeight="1">
       <c r="A32" s="13">
         <v>46119.0</v>
       </c>
@@ -1566,7 +1611,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="33" ht="15.75" customHeight="1">
+    <row r="33" ht="15.75" hidden="1" customHeight="1">
       <c r="A33" s="15">
         <v>46120.0</v>
       </c>
@@ -1578,7 +1623,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="34" ht="15.75" customHeight="1">
+    <row r="34" ht="15.75" hidden="1" customHeight="1">
       <c r="A34" s="13">
         <v>46127.0</v>
       </c>
@@ -1589,7 +1634,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" ht="15.75" customHeight="1">
+    <row r="35" ht="15.75" hidden="1" customHeight="1">
       <c r="A35" s="13">
         <v>46127.0</v>
       </c>
@@ -1603,7 +1648,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="36" ht="15.75" customHeight="1">
+    <row r="36" ht="15.75" hidden="1" customHeight="1">
       <c r="A36" s="13">
         <v>46128.0</v>
       </c>
@@ -1614,7 +1659,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" ht="15.75" customHeight="1">
+    <row r="37" ht="15.75" hidden="1" customHeight="1">
       <c r="A37" s="13">
         <v>46129.0</v>
       </c>
@@ -1628,7 +1673,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" ht="15.75" customHeight="1">
+    <row r="38" ht="15.75" hidden="1" customHeight="1">
       <c r="A38" s="13">
         <v>46130.0</v>
       </c>
@@ -1639,7 +1684,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" ht="15.75" customHeight="1">
+    <row r="39" ht="15.75" hidden="1" customHeight="1">
       <c r="A39" s="13">
         <v>46131.0</v>
       </c>
@@ -1653,7 +1698,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" ht="15.75" customHeight="1">
+    <row r="40" ht="15.75" hidden="1" customHeight="1">
       <c r="A40" s="13">
         <v>46131.0</v>
       </c>
@@ -1664,7 +1709,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="41" ht="15.75" customHeight="1">
+    <row r="41" ht="15.75" hidden="1" customHeight="1">
       <c r="A41" s="13">
         <v>46132.0</v>
       </c>
@@ -1678,7 +1723,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="42" ht="15.75" customHeight="1">
+    <row r="42" ht="15.75" hidden="1" customHeight="1">
       <c r="A42" s="13">
         <v>46133.0</v>
       </c>
@@ -1692,7 +1737,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="43" ht="15.75" customHeight="1">
+    <row r="43" ht="15.75" hidden="1" customHeight="1">
       <c r="A43" s="13">
         <v>46133.0</v>
       </c>
@@ -1703,7 +1748,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="44" ht="15.75" customHeight="1">
+    <row r="44" ht="15.75" hidden="1" customHeight="1">
       <c r="A44" s="13">
         <v>46135.0</v>
       </c>
@@ -1718,7 +1763,7 @@
       </c>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" ht="15.75" customHeight="1">
+    <row r="45" ht="15.75" hidden="1" customHeight="1">
       <c r="A45" s="13">
         <v>46135.0</v>
       </c>
@@ -1732,7 +1777,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" ht="15.75" customHeight="1">
+    <row r="46" ht="15.75" hidden="1" customHeight="1">
       <c r="A46" s="13">
         <v>46136.0</v>
       </c>
@@ -1746,7 +1791,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" ht="15.75" customHeight="1">
+    <row r="47" ht="15.75" hidden="1" customHeight="1">
       <c r="A47" s="13">
         <v>46136.0</v>
       </c>
@@ -1760,7 +1805,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="48" ht="15.75" customHeight="1">
+    <row r="48" ht="15.75" hidden="1" customHeight="1">
       <c r="A48" s="13">
         <v>46136.0</v>
       </c>
@@ -1774,7 +1819,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="49" ht="15.75" customHeight="1">
+    <row r="49" ht="15.75" hidden="1" customHeight="1">
       <c r="A49" s="13">
         <v>46137.0</v>
       </c>
@@ -1788,7 +1833,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="50" ht="15.75" customHeight="1">
+    <row r="50" ht="15.75" hidden="1" customHeight="1">
       <c r="A50" s="13">
         <v>46138.0</v>
       </c>
@@ -1802,7 +1847,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="51" ht="15.75" customHeight="1">
+    <row r="51" ht="15.75" hidden="1" customHeight="1">
       <c r="A51" s="13">
         <v>46138.0</v>
       </c>
@@ -1816,7 +1861,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="52" ht="15.75" customHeight="1">
+    <row r="52" ht="15.75" hidden="1" customHeight="1">
       <c r="A52" s="13">
         <v>46138.0</v>
       </c>
@@ -1828,7 +1873,7 @@
       </c>
       <c r="E52" s="6"/>
     </row>
-    <row r="53" ht="15.75" customHeight="1">
+    <row r="53" ht="15.75" hidden="1" customHeight="1">
       <c r="A53" s="13">
         <v>46140.0</v>
       </c>
@@ -1846,14 +1891,17 @@
       <c r="A54" s="13">
         <v>46143.0</v>
       </c>
+      <c r="B54" s="6" t="s">
+        <v>132</v>
+      </c>
       <c r="C54" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
@@ -1861,13 +1909,13 @@
         <v>46146.0</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E55" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
@@ -1875,13 +1923,13 @@
         <v>46147.0</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
@@ -1889,10 +1937,10 @@
         <v>46148.0</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D57" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
@@ -1900,27 +1948,30 @@
         <v>46148.0</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="13">
         <v>46149.0</v>
       </c>
+      <c r="B59" s="6" t="s">
+        <v>132</v>
+      </c>
       <c r="C59" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
@@ -1928,10 +1979,10 @@
         <v>46150.0</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
@@ -1939,13 +1990,13 @@
         <v>46153.0</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D61" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E61" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
@@ -1953,16 +2004,16 @@
         <v>46153.0</v>
       </c>
       <c r="C62" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
@@ -1970,13 +2021,13 @@
         <v>46153.0</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D63" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
@@ -1984,10 +2035,10 @@
         <v>46154.0</v>
       </c>
       <c r="C64" s="22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
@@ -1995,24 +2046,27 @@
         <v>46156.0</v>
       </c>
       <c r="C65" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="13">
         <v>46157.0</v>
       </c>
+      <c r="B66" s="6" t="s">
+        <v>132</v>
+      </c>
       <c r="C66" s="7" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
@@ -2020,13 +2074,13 @@
         <v>46160.0</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
@@ -2034,13 +2088,13 @@
         <v>46160.0</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
@@ -2048,27 +2102,30 @@
         <v>46161.0</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="13">
         <v>46163.0</v>
       </c>
+      <c r="B70" s="6" t="s">
+        <v>132</v>
+      </c>
       <c r="C70" s="7" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D70" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
@@ -2076,13 +2133,13 @@
         <v>46165.0</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D71" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E71" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
@@ -2090,13 +2147,13 @@
         <v>46165.0</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E72" s="23" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F72" s="24"/>
       <c r="G72" s="24"/>
@@ -2111,11 +2168,14 @@
       <c r="A73" s="13">
         <v>46166.0</v>
       </c>
+      <c r="B73" s="6" t="s">
+        <v>132</v>
+      </c>
       <c r="C73" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D73" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
@@ -2123,17 +2183,82 @@
         <v>46168.0</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D74" s="6" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="75" ht="15.75" customHeight="1"/>
-    <row r="76" ht="15.75" customHeight="1"/>
-    <row r="77" ht="15.75" customHeight="1"/>
-    <row r="78" ht="15.75" customHeight="1"/>
-    <row r="79" ht="15.75" customHeight="1"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="75" ht="15.75" customHeight="1">
+      <c r="A75" s="13">
+        <v>46169.0</v>
+      </c>
+      <c r="C75" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="D75" s="6" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="76" ht="15.75" customHeight="1">
+      <c r="A76" s="13">
+        <v>46170.0</v>
+      </c>
+      <c r="C76" s="22" t="s">
+        <v>193</v>
+      </c>
+      <c r="D76" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="77" ht="15.75" customHeight="1">
+      <c r="A77" s="13">
+        <v>46170.0</v>
+      </c>
+      <c r="C77" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="78" ht="15.75" customHeight="1">
+      <c r="A78" s="13">
+        <v>46172.0</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="C78" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="D78" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="79" ht="15.75" customHeight="1">
+      <c r="A79" s="13">
+        <v>46176.0</v>
+      </c>
+      <c r="C79" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>204</v>
+      </c>
+    </row>
     <row r="80" ht="15.75" customHeight="1"/>
     <row r="81" ht="15.75" customHeight="1"/>
     <row r="82" ht="15.75" customHeight="1"/>
@@ -3140,10 +3265,15 @@
     <hyperlink r:id="rId76" ref="C72"/>
     <hyperlink r:id="rId77" ref="C73"/>
     <hyperlink r:id="rId78" ref="C74"/>
+    <hyperlink r:id="rId79" ref="C75"/>
+    <hyperlink r:id="rId80" ref="C76"/>
+    <hyperlink r:id="rId81" ref="C77"/>
+    <hyperlink r:id="rId82" ref="C78"/>
+    <hyperlink r:id="rId83" ref="C79"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId79"/>
+  <drawing r:id="rId84"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 04-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="212">
   <si>
     <t>date</t>
   </si>
@@ -736,6 +736,27 @@
   </si>
   <si>
     <t>Turno tarde</t>
+  </si>
+  <si>
+    <t>https://youtu.be/0UWSRN_GwCk</t>
+  </si>
+  <si>
+    <t>Juego de posesión</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Vg2m-wXQUvU</t>
+  </si>
+  <si>
+    <t>3 vs 2 + definición</t>
+  </si>
+  <si>
+    <t>https://youtu.be/lYai1tVQEU8</t>
+  </si>
+  <si>
+    <t>Trabajo final</t>
+  </si>
+  <si>
+    <t>Partido 11 vs 11</t>
   </si>
 </sst>
 </file>
@@ -2259,9 +2280,42 @@
         <v>204</v>
       </c>
     </row>
-    <row r="80" ht="15.75" customHeight="1"/>
-    <row r="81" ht="15.75" customHeight="1"/>
-    <row r="82" ht="15.75" customHeight="1"/>
+    <row r="80" ht="15.75" customHeight="1">
+      <c r="A80" s="13">
+        <v>46177.0</v>
+      </c>
+      <c r="C80" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="D80" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="81" ht="15.75" customHeight="1">
+      <c r="A81" s="13">
+        <v>46177.0</v>
+      </c>
+      <c r="C81" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="82" ht="15.75" customHeight="1">
+      <c r="A82" s="13">
+        <v>46177.0</v>
+      </c>
+      <c r="C82" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="D82" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="E82" s="6" t="s">
+        <v>211</v>
+      </c>
+    </row>
     <row r="83" ht="15.75" customHeight="1"/>
     <row r="84" ht="15.75" customHeight="1"/>
     <row r="85" ht="15.75" customHeight="1"/>
@@ -3270,10 +3324,13 @@
     <hyperlink r:id="rId81" ref="C77"/>
     <hyperlink r:id="rId82" ref="C78"/>
     <hyperlink r:id="rId83" ref="C79"/>
+    <hyperlink r:id="rId84" ref="C80"/>
+    <hyperlink r:id="rId85" ref="C81"/>
+    <hyperlink r:id="rId86" ref="C82"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId84"/>
+  <drawing r:id="rId87"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 05-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="214">
   <si>
     <t>date</t>
   </si>
@@ -757,6 +757,12 @@
   </si>
   <si>
     <t>Partido 11 vs 11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/2ipkm5tH_po</t>
+  </si>
+  <si>
+    <t>https://youtu.be/gNEhllrfNks</t>
   </si>
 </sst>
 </file>
@@ -2316,8 +2322,22 @@
         <v>211</v>
       </c>
     </row>
-    <row r="83" ht="15.75" customHeight="1"/>
-    <row r="84" ht="15.75" customHeight="1"/>
+    <row r="83" ht="15.75" customHeight="1">
+      <c r="A83" s="13">
+        <v>46178.0</v>
+      </c>
+      <c r="C83" s="7" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="84" ht="15.75" customHeight="1">
+      <c r="A84" s="13">
+        <v>46178.0</v>
+      </c>
+      <c r="C84" s="7" t="s">
+        <v>213</v>
+      </c>
+    </row>
     <row r="85" ht="15.75" customHeight="1"/>
     <row r="86" ht="15.75" customHeight="1"/>
     <row r="87" ht="15.75" customHeight="1"/>
@@ -3327,10 +3347,12 @@
     <hyperlink r:id="rId84" ref="C80"/>
     <hyperlink r:id="rId85" ref="C81"/>
     <hyperlink r:id="rId86" ref="C82"/>
+    <hyperlink r:id="rId87" ref="C83"/>
+    <hyperlink r:id="rId88" ref="C84"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId87"/>
+  <drawing r:id="rId89"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 13-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="219">
   <si>
     <t>date</t>
   </si>
@@ -763,6 +763,21 @@
   </si>
   <si>
     <t>https://youtu.be/gNEhllrfNks</t>
+  </si>
+  <si>
+    <t>https://youtu.be/QKf25OTTdPY</t>
+  </si>
+  <si>
+    <t>https://youtu.be/aEfYNvPZRx0</t>
+  </si>
+  <si>
+    <t>https://youtu.be/kOhg4rxmGFs</t>
+  </si>
+  <si>
+    <t>https://youtu.be/pBl7S0WDG5Q</t>
+  </si>
+  <si>
+    <t>https://youtu.be/AEYpZrjOiHA</t>
   </si>
 </sst>
 </file>
@@ -2338,11 +2353,52 @@
         <v>213</v>
       </c>
     </row>
-    <row r="85" ht="15.75" customHeight="1"/>
-    <row r="86" ht="15.75" customHeight="1"/>
-    <row r="87" ht="15.75" customHeight="1"/>
-    <row r="88" ht="15.75" customHeight="1"/>
-    <row r="89" ht="15.75" customHeight="1"/>
+    <row r="85" ht="15.75" customHeight="1">
+      <c r="A85" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="C85" s="7" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="86" ht="15.75" customHeight="1">
+      <c r="A86" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="C86" s="22" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="87" ht="15.75" customHeight="1">
+      <c r="A87" s="13">
+        <v>46179.0</v>
+      </c>
+      <c r="C87" s="7" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="88" ht="15.75" customHeight="1">
+      <c r="A88" s="13">
+        <v>46180.0</v>
+      </c>
+      <c r="C88" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="D88" s="6" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="89" ht="15.75" customHeight="1">
+      <c r="A89" s="13">
+        <v>46186.0</v>
+      </c>
+      <c r="C89" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="D89" s="6" t="s">
+        <v>168</v>
+      </c>
+    </row>
     <row r="90" ht="15.75" customHeight="1"/>
     <row r="91" ht="15.75" customHeight="1"/>
     <row r="92" ht="15.75" customHeight="1"/>
@@ -3349,10 +3405,15 @@
     <hyperlink r:id="rId86" ref="C82"/>
     <hyperlink r:id="rId87" ref="C83"/>
     <hyperlink r:id="rId88" ref="C84"/>
+    <hyperlink r:id="rId89" ref="C85"/>
+    <hyperlink r:id="rId90" ref="C86"/>
+    <hyperlink r:id="rId91" ref="C87"/>
+    <hyperlink r:id="rId92" ref="C88"/>
+    <hyperlink r:id="rId93" ref="C89"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId89"/>
+  <drawing r:id="rId94"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 17-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="iYnBsaeGnAZvtGM8/noNG3xrTTjpBKqMc/Ub/MqKvT8="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="8FUU9kY3xgzMeoNWu4VhkOZfQtPixBQseXXFvkmyJj0="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="222">
   <si>
     <t>date</t>
   </si>
@@ -777,7 +777,16 @@
     <t>https://youtu.be/pBl7S0WDG5Q</t>
   </si>
   <si>
+    <t>https://youtu.be/GeU26DDUd4k</t>
+  </si>
+  <si>
     <t>https://youtu.be/AEYpZrjOiHA</t>
+  </si>
+  <si>
+    <t>https://youtu.be/P5AOosd3QP8</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Hvo_Zh-Qq7M</t>
   </si>
 </sst>
 </file>
@@ -2390,18 +2399,42 @@
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="13">
-        <v>46186.0</v>
+        <v>46182.0</v>
       </c>
       <c r="C89" s="7" t="s">
         <v>218</v>
       </c>
       <c r="D89" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="90" ht="15.75" customHeight="1">
+      <c r="A90" s="13">
+        <v>46186.0</v>
+      </c>
+      <c r="C90" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="D90" s="6" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="90" ht="15.75" customHeight="1"/>
-    <row r="91" ht="15.75" customHeight="1"/>
-    <row r="92" ht="15.75" customHeight="1"/>
+    <row r="91" ht="15.75" customHeight="1">
+      <c r="A91" s="13">
+        <v>46189.0</v>
+      </c>
+      <c r="C91" s="7" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="92" ht="15.75" customHeight="1">
+      <c r="A92" s="13">
+        <v>46190.0</v>
+      </c>
+      <c r="C92" s="7" t="s">
+        <v>221</v>
+      </c>
+    </row>
     <row r="93" ht="15.75" customHeight="1"/>
     <row r="94" ht="15.75" customHeight="1"/>
     <row r="95" ht="15.75" customHeight="1"/>
@@ -3315,6 +3348,7 @@
     <row r="1003" ht="15.75" customHeight="1"/>
     <row r="1004" ht="15.75" customHeight="1"/>
     <row r="1005" ht="15.75" customHeight="1"/>
+    <row r="1006" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
@@ -3410,10 +3444,13 @@
     <hyperlink r:id="rId91" ref="C87"/>
     <hyperlink r:id="rId92" ref="C88"/>
     <hyperlink r:id="rId93" ref="C89"/>
+    <hyperlink r:id="rId94" ref="C90"/>
+    <hyperlink r:id="rId95" ref="C91"/>
+    <hyperlink r:id="rId96" ref="C92"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId94"/>
+  <drawing r:id="rId97"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 20-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="226">
   <si>
     <t>date</t>
   </si>
@@ -787,6 +787,18 @@
   </si>
   <si>
     <t>https://youtu.be/Hvo_Zh-Qq7M</t>
+  </si>
+  <si>
+    <t>https://youtu.be/yP61kJ2JqnQ</t>
+  </si>
+  <si>
+    <t>https://youtu.be/c3dNkc-cIrY</t>
+  </si>
+  <si>
+    <t>11 vs 11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ET6NrbvaJ2A</t>
   </si>
 </sst>
 </file>
@@ -2435,9 +2447,39 @@
         <v>221</v>
       </c>
     </row>
-    <row r="93" ht="15.75" customHeight="1"/>
-    <row r="94" ht="15.75" customHeight="1"/>
-    <row r="95" ht="15.75" customHeight="1"/>
+    <row r="93" ht="15.75" customHeight="1">
+      <c r="A93" s="13">
+        <v>46191.0</v>
+      </c>
+      <c r="C93" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="D93" s="6" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="94" ht="15.75" customHeight="1">
+      <c r="A94" s="13">
+        <v>46191.0</v>
+      </c>
+      <c r="C94" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="D94" s="6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="95" ht="15.75" customHeight="1">
+      <c r="A95" s="13">
+        <v>46193.0</v>
+      </c>
+      <c r="C95" s="7" t="s">
+        <v>225</v>
+      </c>
+      <c r="D95" s="6" t="s">
+        <v>188</v>
+      </c>
+    </row>
     <row r="96" ht="15.75" customHeight="1"/>
     <row r="97" ht="15.75" customHeight="1"/>
     <row r="98" ht="15.75" customHeight="1"/>
@@ -3447,10 +3489,13 @@
     <hyperlink r:id="rId94" ref="C90"/>
     <hyperlink r:id="rId95" ref="C91"/>
     <hyperlink r:id="rId96" ref="C92"/>
+    <hyperlink r:id="rId97" ref="C93"/>
+    <hyperlink r:id="rId98" ref="C94"/>
+    <hyperlink r:id="rId99" ref="C95"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId97"/>
+  <drawing r:id="rId100"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 20-06 con analisis d arqueros
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="228">
   <si>
     <t>date</t>
   </si>
@@ -783,10 +783,16 @@
     <t>https://youtu.be/AEYpZrjOiHA</t>
   </si>
   <si>
+    <t>https://youtu.be/91NeyqV7shg</t>
+  </si>
+  <si>
     <t>https://youtu.be/P5AOosd3QP8</t>
   </si>
   <si>
     <t>https://youtu.be/Hvo_Zh-Qq7M</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Hj2mPLMEp-M</t>
   </si>
   <si>
     <t>https://youtu.be/yP61kJ2JqnQ</t>
@@ -1238,7 +1244,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" hidden="1">
+    <row r="2">
       <c r="A2" s="5">
         <v>46087.0</v>
       </c>
@@ -1252,7 +1258,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" hidden="1">
+    <row r="3">
       <c r="A3" s="5">
         <v>46087.0</v>
       </c>
@@ -1266,7 +1272,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" hidden="1">
+    <row r="4">
       <c r="A4" s="5">
         <v>46087.0</v>
       </c>
@@ -1280,7 +1286,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" hidden="1">
+    <row r="5">
       <c r="A5" s="11">
         <v>46092.0</v>
       </c>
@@ -1294,7 +1300,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" hidden="1">
+    <row r="6">
       <c r="A6" s="11">
         <v>46092.0</v>
       </c>
@@ -1308,7 +1314,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" hidden="1">
+    <row r="7">
       <c r="A7" s="11">
         <v>46093.0</v>
       </c>
@@ -1322,7 +1328,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" hidden="1">
+    <row r="8">
       <c r="A8" s="11">
         <v>46093.0</v>
       </c>
@@ -1339,7 +1345,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" hidden="1">
+    <row r="9">
       <c r="A9" s="11">
         <v>46093.0</v>
       </c>
@@ -1356,7 +1362,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" hidden="1">
+    <row r="10">
       <c r="A10" s="11">
         <v>46093.0</v>
       </c>
@@ -1373,7 +1379,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="11" hidden="1">
+    <row r="11">
       <c r="A11" s="11">
         <v>46094.0</v>
       </c>
@@ -1390,7 +1396,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" hidden="1">
+    <row r="12">
       <c r="A12" s="11">
         <v>46094.0</v>
       </c>
@@ -1407,7 +1413,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" hidden="1">
+    <row r="13">
       <c r="A13" s="11">
         <v>46095.0</v>
       </c>
@@ -1424,7 +1430,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" hidden="1">
+    <row r="14">
       <c r="A14" s="13">
         <v>46097.0</v>
       </c>
@@ -1438,7 +1444,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="15" hidden="1">
+    <row r="15">
       <c r="A15" s="13">
         <v>46098.0</v>
       </c>
@@ -1452,7 +1458,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" hidden="1">
+    <row r="16">
       <c r="A16" s="13">
         <v>46098.0</v>
       </c>
@@ -1466,7 +1472,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" hidden="1">
+    <row r="17">
       <c r="A17" s="13">
         <v>46098.0</v>
       </c>
@@ -1480,7 +1486,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" hidden="1">
+    <row r="18">
       <c r="A18" s="13">
         <v>46099.0</v>
       </c>
@@ -1495,7 +1501,7 @@
       </c>
       <c r="E18" s="14"/>
     </row>
-    <row r="19" hidden="1">
+    <row r="19">
       <c r="A19" s="13">
         <v>46099.0</v>
       </c>
@@ -1512,7 +1518,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" ht="15.75" hidden="1" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="15">
         <v>46102.0</v>
       </c>
@@ -1527,7 +1533,7 @@
       </c>
       <c r="E20" s="18"/>
     </row>
-    <row r="21" ht="15.75" hidden="1" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="13">
         <v>46103.0</v>
       </c>
@@ -1539,7 +1545,7 @@
       </c>
       <c r="E21" s="14"/>
     </row>
-    <row r="22" ht="15.75" hidden="1" customHeight="1">
+    <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="13">
         <v>46104.0</v>
       </c>
@@ -1551,7 +1557,7 @@
       </c>
       <c r="E22" s="18"/>
     </row>
-    <row r="23" ht="15.75" hidden="1" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="13">
         <v>46105.0</v>
       </c>
@@ -1563,7 +1569,7 @@
       </c>
       <c r="E23" s="14"/>
     </row>
-    <row r="24" ht="15.75" hidden="1" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="13">
         <v>46106.0</v>
       </c>
@@ -1580,7 +1586,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" ht="15.75" hidden="1" customHeight="1">
+    <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="13">
         <v>46108.0</v>
       </c>
@@ -1591,7 +1597,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="26" ht="15.75" hidden="1" customHeight="1">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="13">
         <v>46108.0</v>
       </c>
@@ -1605,7 +1611,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="27" ht="15.75" hidden="1" customHeight="1">
+    <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="13">
         <v>46108.0</v>
       </c>
@@ -1616,7 +1622,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="28" ht="15.75" hidden="1" customHeight="1">
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="15">
         <v>46109.0</v>
       </c>
@@ -1628,7 +1634,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="29" ht="15.75" hidden="1" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="15">
         <v>46113.0</v>
       </c>
@@ -1640,7 +1646,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="30" ht="15.75" hidden="1" customHeight="1">
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="15">
         <v>46114.0</v>
       </c>
@@ -1652,7 +1658,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="31" ht="15.75" hidden="1" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="13">
         <v>46116.0</v>
       </c>
@@ -1663,7 +1669,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="32" ht="15.75" hidden="1" customHeight="1">
+    <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="13">
         <v>46119.0</v>
       </c>
@@ -1674,7 +1680,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="33" ht="15.75" hidden="1" customHeight="1">
+    <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="15">
         <v>46120.0</v>
       </c>
@@ -1686,7 +1692,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="34" ht="15.75" hidden="1" customHeight="1">
+    <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="13">
         <v>46127.0</v>
       </c>
@@ -1697,7 +1703,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" ht="15.75" hidden="1" customHeight="1">
+    <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="13">
         <v>46127.0</v>
       </c>
@@ -1711,7 +1717,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="36" ht="15.75" hidden="1" customHeight="1">
+    <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="13">
         <v>46128.0</v>
       </c>
@@ -1722,7 +1728,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="37" ht="15.75" hidden="1" customHeight="1">
+    <row r="37" ht="15.75" customHeight="1">
       <c r="A37" s="13">
         <v>46129.0</v>
       </c>
@@ -1736,7 +1742,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" ht="15.75" hidden="1" customHeight="1">
+    <row r="38" ht="15.75" customHeight="1">
       <c r="A38" s="13">
         <v>46130.0</v>
       </c>
@@ -1747,7 +1753,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="39" ht="15.75" hidden="1" customHeight="1">
+    <row r="39" ht="15.75" customHeight="1">
       <c r="A39" s="13">
         <v>46131.0</v>
       </c>
@@ -1761,7 +1767,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="40" ht="15.75" hidden="1" customHeight="1">
+    <row r="40" ht="15.75" customHeight="1">
       <c r="A40" s="13">
         <v>46131.0</v>
       </c>
@@ -1772,7 +1778,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="41" ht="15.75" hidden="1" customHeight="1">
+    <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="13">
         <v>46132.0</v>
       </c>
@@ -1786,7 +1792,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="42" ht="15.75" hidden="1" customHeight="1">
+    <row r="42" ht="15.75" customHeight="1">
       <c r="A42" s="13">
         <v>46133.0</v>
       </c>
@@ -1800,7 +1806,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="43" ht="15.75" hidden="1" customHeight="1">
+    <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="13">
         <v>46133.0</v>
       </c>
@@ -1811,7 +1817,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="44" ht="15.75" hidden="1" customHeight="1">
+    <row r="44" ht="15.75" customHeight="1">
       <c r="A44" s="13">
         <v>46135.0</v>
       </c>
@@ -1826,7 +1832,7 @@
       </c>
       <c r="H44" s="6"/>
     </row>
-    <row r="45" ht="15.75" hidden="1" customHeight="1">
+    <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="13">
         <v>46135.0</v>
       </c>
@@ -1840,7 +1846,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="46" ht="15.75" hidden="1" customHeight="1">
+    <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="13">
         <v>46136.0</v>
       </c>
@@ -1854,7 +1860,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="47" ht="15.75" hidden="1" customHeight="1">
+    <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="13">
         <v>46136.0</v>
       </c>
@@ -1868,7 +1874,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="48" ht="15.75" hidden="1" customHeight="1">
+    <row r="48" ht="15.75" customHeight="1">
       <c r="A48" s="13">
         <v>46136.0</v>
       </c>
@@ -1882,7 +1888,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="49" ht="15.75" hidden="1" customHeight="1">
+    <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="13">
         <v>46137.0</v>
       </c>
@@ -1896,7 +1902,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="50" ht="15.75" hidden="1" customHeight="1">
+    <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13">
         <v>46138.0</v>
       </c>
@@ -1910,7 +1916,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="51" ht="15.75" hidden="1" customHeight="1">
+    <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="13">
         <v>46138.0</v>
       </c>
@@ -1924,7 +1930,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="52" ht="15.75" hidden="1" customHeight="1">
+    <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="13">
         <v>46138.0</v>
       </c>
@@ -1936,7 +1942,7 @@
       </c>
       <c r="E52" s="6"/>
     </row>
-    <row r="53" ht="15.75" hidden="1" customHeight="1">
+    <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="13">
         <v>46140.0</v>
       </c>
@@ -2430,13 +2436,16 @@
       <c r="D90" s="6" t="s">
         <v>168</v>
       </c>
+      <c r="E90" s="7" t="s">
+        <v>220</v>
+      </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="13">
         <v>46189.0</v>
       </c>
       <c r="C91" s="7" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
@@ -2444,7 +2453,10 @@
         <v>46190.0</v>
       </c>
       <c r="C92" s="7" t="s">
-        <v>221</v>
+        <v>222</v>
+      </c>
+      <c r="E92" s="7" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
@@ -2452,7 +2464,7 @@
         <v>46191.0</v>
       </c>
       <c r="C93" s="7" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D93" s="6" t="s">
         <v>206</v>
@@ -2463,10 +2475,10 @@
         <v>46191.0</v>
       </c>
       <c r="C94" s="7" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D94" s="6" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
@@ -2474,7 +2486,7 @@
         <v>46193.0</v>
       </c>
       <c r="C95" s="7" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D95" s="6" t="s">
         <v>188</v>
@@ -3487,15 +3499,17 @@
     <hyperlink r:id="rId92" ref="C88"/>
     <hyperlink r:id="rId93" ref="C89"/>
     <hyperlink r:id="rId94" ref="C90"/>
-    <hyperlink r:id="rId95" ref="C91"/>
-    <hyperlink r:id="rId96" ref="C92"/>
-    <hyperlink r:id="rId97" ref="C93"/>
-    <hyperlink r:id="rId98" ref="C94"/>
-    <hyperlink r:id="rId99" ref="C95"/>
+    <hyperlink r:id="rId95" ref="E90"/>
+    <hyperlink r:id="rId96" ref="C91"/>
+    <hyperlink r:id="rId97" ref="C92"/>
+    <hyperlink r:id="rId98" ref="E92"/>
+    <hyperlink r:id="rId99" ref="C93"/>
+    <hyperlink r:id="rId100" ref="C94"/>
+    <hyperlink r:id="rId101" ref="C95"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId100"/>
+  <drawing r:id="rId102"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 23-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="230">
   <si>
     <t>date</t>
   </si>
@@ -805,6 +805,12 @@
   </si>
   <si>
     <t>https://youtu.be/ET6NrbvaJ2A</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xtyqkXcTy9s</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Qiz2Y1a6hZI</t>
   </si>
 </sst>
 </file>
@@ -2492,8 +2498,28 @@
         <v>188</v>
       </c>
     </row>
-    <row r="96" ht="15.75" customHeight="1"/>
-    <row r="97" ht="15.75" customHeight="1"/>
+    <row r="96" ht="15.75" customHeight="1">
+      <c r="A96" s="13">
+        <v>46195.0</v>
+      </c>
+      <c r="C96" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="D96" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="97" ht="15.75" customHeight="1">
+      <c r="A97" s="13">
+        <v>46196.0</v>
+      </c>
+      <c r="C97" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="D97" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
     <row r="98" ht="15.75" customHeight="1"/>
     <row r="99" ht="15.75" customHeight="1"/>
     <row r="100" ht="15.75" customHeight="1"/>
@@ -3506,10 +3532,12 @@
     <hyperlink r:id="rId99" ref="C93"/>
     <hyperlink r:id="rId100" ref="C94"/>
     <hyperlink r:id="rId101" ref="C95"/>
+    <hyperlink r:id="rId102" ref="C96"/>
+    <hyperlink r:id="rId103" ref="C97"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId102"/>
+  <drawing r:id="rId104"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 23-06 v2
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="226">
   <si>
     <t>date</t>
   </si>
@@ -33,9 +33,6 @@
     <t>comentarios</t>
   </si>
   <si>
-    <t>activación</t>
-  </si>
-  <si>
     <t>https://youtu.be/n5sBx_cosTY</t>
   </si>
   <si>
@@ -48,9 +45,6 @@
     <t>Parte 2 Activación</t>
   </si>
   <si>
-    <t>principal</t>
-  </si>
-  <si>
     <t>https://youtu.be/ivunOFSM1ME</t>
   </si>
   <si>
@@ -129,16 +123,10 @@
     <t>https://youtu.be/Ub1KGSTFWaY</t>
   </si>
   <si>
-    <t>pruebas</t>
-  </si>
-  <si>
     <t>https://youtu.be/GUwuiwzLQOo</t>
   </si>
   <si>
     <t>Yo-yo test</t>
-  </si>
-  <si>
-    <t>Pre activación</t>
   </si>
   <si>
     <t>https://youtu.be/3EX6bh7VSE4</t>
@@ -519,207 +507,207 @@
     <t>Entrenamiento de resistencia, rueda de pases, juego de posesion</t>
   </si>
   <si>
+    <t>https://youtu.be/Hod9nJ9w4gM</t>
+  </si>
+  <si>
+    <t>Amistoso vs Real Católica</t>
+  </si>
+  <si>
+    <t>Partido Amistoso VS Catolica</t>
+  </si>
+  <si>
+    <t>https://youtu.be/O_RFkTcApiY</t>
+  </si>
+  <si>
+    <t>1er Turno  09:00 am</t>
+  </si>
+  <si>
+    <t>Trabajo de Fuerza, Juego de Centros y Transiciones D-A , A-D</t>
+  </si>
+  <si>
+    <t>https://youtu.be/7HBr7Vxj_kA</t>
+  </si>
+  <si>
+    <t>Turno unico 2:30 pm</t>
+  </si>
+  <si>
+    <t>Trabajo de velocidad - Juego 11 vs11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/3Z_xecPmSew</t>
+  </si>
+  <si>
+    <t>Activación 06/05</t>
+  </si>
+  <si>
+    <t>https://youtu.be/hC8wydyucPk</t>
+  </si>
+  <si>
+    <t>ABPs</t>
+  </si>
+  <si>
+    <t>Corner y Tiro libre lateral</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bey02ugnB4U</t>
+  </si>
+  <si>
+    <t>Amistoso vs Liberty schoool</t>
+  </si>
+  <si>
+    <t>Partido amistos vs Liberty (Moquegua)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/VlC2L9ODx1Q</t>
+  </si>
+  <si>
+    <t>Entrenamiento 4:00 p.m</t>
+  </si>
+  <si>
+    <t>https://youtu.be/fh7C4BXJDJg</t>
+  </si>
+  <si>
+    <t>1er Turno 9:00 a.m</t>
+  </si>
+  <si>
+    <t>Entrenamiento de resistencia</t>
+  </si>
+  <si>
+    <t>https://youtu.be/CdhE6Pk3Qvk</t>
+  </si>
+  <si>
+    <t>2do Turno - activación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rondos </t>
+  </si>
+  <si>
+    <t>//</t>
+  </si>
+  <si>
+    <t>https://youtu.be/cPF7Sij2ZBk</t>
+  </si>
+  <si>
+    <t>2do Turno - Salida real</t>
+  </si>
+  <si>
+    <t>Salida de balón: estructura y movimientos</t>
+  </si>
+  <si>
+    <t>https://youtu.be/47_QGKmmLw4</t>
+  </si>
+  <si>
+    <t>Turno único</t>
+  </si>
+  <si>
+    <t>https://youtu.be/OnXQbmlEqUo</t>
+  </si>
+  <si>
+    <t>Definición 14-05</t>
+  </si>
+  <si>
+    <t>Ejercicio de definición 14 de mayo 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://youtu.be/VSLhcOEX8ho </t>
+  </si>
+  <si>
+    <t>Amistoso A vs B</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-zf5eWAEF_w</t>
+  </si>
+  <si>
+    <t>11 vs 11 con condición</t>
+  </si>
+  <si>
+    <t>11 vs 11 con condición || 23-05-26</t>
+  </si>
+  <si>
+    <t>https://youtu.be/sVRy3ma9PpQ</t>
+  </si>
+  <si>
+    <t>11 vs 11 - 18/05/26</t>
+  </si>
+  <si>
+    <t>Libre 11 vs 11</t>
+  </si>
+  <si>
+    <t>https://youtu.be/LGVYMTdnvps</t>
+  </si>
+  <si>
+    <t>11 vs 11 - 19/05/26</t>
+  </si>
+  <si>
+    <t>Equipo A  vs Equipo B. Equipo A vs Equipo "a prueba"</t>
+  </si>
+  <si>
+    <t>https://youtu.be/EK7GF8KsKNo</t>
+  </si>
+  <si>
+    <t>Partido amistoso</t>
+  </si>
+  <si>
+    <t>Amistos vs Sportivo Huracán</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-7p876MvXF8</t>
+  </si>
+  <si>
+    <t>Salida 23-05</t>
+  </si>
+  <si>
+    <t>Salida sin oposición</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Vcp_XV58azM</t>
+  </si>
+  <si>
+    <t>ABPs  23-05</t>
+  </si>
+  <si>
+    <t>Practicando ABP (corners, tiros libres y penales)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/y-_Cd_Pa61k</t>
+  </si>
+  <si>
+    <t>Amistoso vs ANBA</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xy0qpug4-W8</t>
+  </si>
+  <si>
+    <t>Entrenamiento 3pm</t>
+  </si>
+  <si>
+    <t>https://youtu.be/QsdV3CV-klA</t>
+  </si>
+  <si>
+    <t>Entrenamiento 4pm</t>
+  </si>
+  <si>
+    <t>https://youtu.be/e-WhTZ7sMgA</t>
+  </si>
+  <si>
+    <t>Ejercicio de definición</t>
+  </si>
+  <si>
+    <t>Ejercicio de definición con puntaje</t>
+  </si>
+  <si>
+    <t>https://youtu.be/f7cBcoW2CLc</t>
+  </si>
+  <si>
+    <t>Salidas y ABPs a favor</t>
+  </si>
+  <si>
+    <t>Salidas vs presión alta. Salidas vs bloque bajo. Tiros libre laterales a favor. Corners a favor</t>
+  </si>
+  <si>
     <t>partido</t>
   </si>
   <si>
-    <t>https://youtu.be/Hod9nJ9w4gM</t>
-  </si>
-  <si>
-    <t>Amistoso vs Real Católica</t>
-  </si>
-  <si>
-    <t>Partido Amistoso VS Catolica</t>
-  </si>
-  <si>
-    <t>https://youtu.be/O_RFkTcApiY</t>
-  </si>
-  <si>
-    <t>1er Turno  09:00 am</t>
-  </si>
-  <si>
-    <t>Trabajo de Fuerza, Juego de Centros y Transiciones D-A , A-D</t>
-  </si>
-  <si>
-    <t>https://youtu.be/7HBr7Vxj_kA</t>
-  </si>
-  <si>
-    <t>Turno unico 2:30 pm</t>
-  </si>
-  <si>
-    <t>Trabajo de velocidad - Juego 11 vs11</t>
-  </si>
-  <si>
-    <t>https://youtu.be/3Z_xecPmSew</t>
-  </si>
-  <si>
-    <t>Activación 06/05</t>
-  </si>
-  <si>
-    <t>https://youtu.be/hC8wydyucPk</t>
-  </si>
-  <si>
-    <t>ABPs</t>
-  </si>
-  <si>
-    <t>Corner y Tiro libre lateral</t>
-  </si>
-  <si>
-    <t>https://youtu.be/bey02ugnB4U</t>
-  </si>
-  <si>
-    <t>Amistoso vs Liberty schoool</t>
-  </si>
-  <si>
-    <t>Partido amistos vs Liberty (Moquegua)</t>
-  </si>
-  <si>
-    <t>https://youtu.be/VlC2L9ODx1Q</t>
-  </si>
-  <si>
-    <t>Entrenamiento 4:00 p.m</t>
-  </si>
-  <si>
-    <t>https://youtu.be/fh7C4BXJDJg</t>
-  </si>
-  <si>
-    <t>1er Turno 9:00 a.m</t>
-  </si>
-  <si>
-    <t>Entrenamiento de resistencia</t>
-  </si>
-  <si>
-    <t>https://youtu.be/CdhE6Pk3Qvk</t>
-  </si>
-  <si>
-    <t>2do Turno - activación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rondos </t>
-  </si>
-  <si>
-    <t>//</t>
-  </si>
-  <si>
-    <t>https://youtu.be/cPF7Sij2ZBk</t>
-  </si>
-  <si>
-    <t>2do Turno - Salida real</t>
-  </si>
-  <si>
-    <t>Salida de balón: estructura y movimientos</t>
-  </si>
-  <si>
-    <t>https://youtu.be/47_QGKmmLw4</t>
-  </si>
-  <si>
-    <t>Turno único</t>
-  </si>
-  <si>
-    <t>https://youtu.be/OnXQbmlEqUo</t>
-  </si>
-  <si>
-    <t>Definición 14-05</t>
-  </si>
-  <si>
-    <t>Ejercicio de definición 14 de mayo 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://youtu.be/VSLhcOEX8ho </t>
-  </si>
-  <si>
-    <t>Amistoso A vs B</t>
-  </si>
-  <si>
-    <t>https://youtu.be/-zf5eWAEF_w</t>
-  </si>
-  <si>
-    <t>11 vs 11 con condición</t>
-  </si>
-  <si>
-    <t>11 vs 11 con condición || 23-05-26</t>
-  </si>
-  <si>
-    <t>https://youtu.be/sVRy3ma9PpQ</t>
-  </si>
-  <si>
-    <t>11 vs 11 - 18/05/26</t>
-  </si>
-  <si>
-    <t>Libre 11 vs 11</t>
-  </si>
-  <si>
-    <t>https://youtu.be/LGVYMTdnvps</t>
-  </si>
-  <si>
-    <t>11 vs 11 - 19/05/26</t>
-  </si>
-  <si>
-    <t>Equipo A  vs Equipo B. Equipo A vs Equipo "a prueba"</t>
-  </si>
-  <si>
-    <t>https://youtu.be/EK7GF8KsKNo</t>
-  </si>
-  <si>
-    <t>Partido amistoso</t>
-  </si>
-  <si>
-    <t>Amistos vs Sportivo Huracán</t>
-  </si>
-  <si>
-    <t>https://youtu.be/-7p876MvXF8</t>
-  </si>
-  <si>
-    <t>Salida 23-05</t>
-  </si>
-  <si>
-    <t>Salida sin oposición</t>
-  </si>
-  <si>
-    <t>https://youtu.be/Vcp_XV58azM</t>
-  </si>
-  <si>
-    <t>ABPs  23-05</t>
-  </si>
-  <si>
-    <t>Practicando ABP (corners, tiros libres y penales)</t>
-  </si>
-  <si>
-    <t>https://youtu.be/y-_Cd_Pa61k</t>
-  </si>
-  <si>
-    <t>Amistoso vs ANBA</t>
-  </si>
-  <si>
-    <t>https://youtu.be/xy0qpug4-W8</t>
-  </si>
-  <si>
-    <t>Entrenamiento 3pm</t>
-  </si>
-  <si>
-    <t>https://youtu.be/QsdV3CV-klA</t>
-  </si>
-  <si>
-    <t>Entrenamiento 4pm</t>
-  </si>
-  <si>
-    <t>https://youtu.be/e-WhTZ7sMgA</t>
-  </si>
-  <si>
-    <t>Ejercicio de definición</t>
-  </si>
-  <si>
-    <t>Ejercicio de definición con puntaje</t>
-  </si>
-  <si>
-    <t>https://youtu.be/f7cBcoW2CLc</t>
-  </si>
-  <si>
-    <t>Salidas y ABPs a favor</t>
-  </si>
-  <si>
-    <t>Salidas vs presión alta. Salidas vs bloque bajo. Tiros libre laterales a favor. Corners a favor</t>
-  </si>
-  <si>
     <t>https://youtu.be/j5qjoOjpxuw</t>
   </si>
   <si>
@@ -810,7 +798,7 @@
     <t>https://youtu.be/xtyqkXcTy9s</t>
   </si>
   <si>
-    <t>https://youtu.be/Qiz2Y1a6hZI</t>
+    <t>https://youtu.be/MEpLI9f7JJQ</t>
   </si>
 </sst>
 </file>
@@ -853,13 +841,13 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <u/>
+      <color rgb="FF0000FF"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <color rgb="FF0000FF"/>
     </font>
     <font>
       <u/>
@@ -942,7 +930,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -974,22 +962,22 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="2" fontId="6" numFmtId="166" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -999,7 +987,6 @@
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -1254,256 +1241,206 @@
       <c r="A2" s="5">
         <v>46087.0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5">
         <v>46087.0</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="7" t="s">
         <v>8</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5">
         <v>46087.0</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="10" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="11">
         <v>46092.0</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>14</v>
+      <c r="C5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="11">
         <v>46092.0</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>16</v>
+      <c r="C6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>18</v>
+      <c r="C7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="C8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="7" t="s">
+      <c r="C9" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="7" t="s">
         <v>22</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="11">
         <v>46093.0</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="7" t="s">
+      <c r="C10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>25</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="11">
         <v>46094.0</v>
       </c>
-      <c r="B11" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="C11" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="11">
         <v>46094.0</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E12" s="12" t="s">
         <v>31</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="11">
         <v>46095.0</v>
       </c>
-      <c r="B13" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C13" s="7" t="s">
+      <c r="C13" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="12" t="s">
         <v>34</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="13">
         <v>46097.0</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>39</v>
+      <c r="C14" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="13">
         <v>46098.0</v>
       </c>
-      <c r="B15" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>42</v>
+      <c r="C15" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13">
         <v>46098.0</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>44</v>
+      <c r="C16" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="13">
         <v>46098.0</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>46</v>
+      <c r="C17" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="13">
         <v>46099.0</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>48</v>
+      <c r="C18" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="E18" s="14"/>
     </row>
@@ -1511,17 +1448,14 @@
       <c r="A19" s="13">
         <v>46099.0</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="C19" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>12</v>
-      </c>
       <c r="E19" s="14" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
@@ -1529,13 +1463,13 @@
         <v>46102.0</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="D20" s="16" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="E20" s="18"/>
     </row>
@@ -1543,11 +1477,11 @@
       <c r="A21" s="13">
         <v>46103.0</v>
       </c>
-      <c r="C21" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>55</v>
+      <c r="C21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="E21" s="14"/>
     </row>
@@ -1555,11 +1489,11 @@
       <c r="A22" s="13">
         <v>46104.0</v>
       </c>
-      <c r="C22" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>55</v>
+      <c r="C22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="E22" s="18"/>
     </row>
@@ -1567,11 +1501,11 @@
       <c r="A23" s="13">
         <v>46105.0</v>
       </c>
-      <c r="C23" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>55</v>
+      <c r="C23" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="E23" s="14"/>
     </row>
@@ -1579,89 +1513,95 @@
       <c r="A24" s="13">
         <v>46106.0</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>51</v>
+      <c r="B24" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>60</v>
+        <v>54</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="13">
         <v>46108.0</v>
       </c>
-      <c r="C25" s="7" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>62</v>
+      <c r="C25" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="13">
         <v>46108.0</v>
       </c>
-      <c r="C26" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>65</v>
+      <c r="C26" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="E26" s="7" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="13">
         <v>46108.0</v>
       </c>
-      <c r="C27" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>67</v>
+      <c r="C27" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="15">
         <v>46109.0</v>
       </c>
-      <c r="B28" s="20"/>
+      <c r="B28" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C28" s="17" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D28" s="16" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="15">
         <v>46113.0</v>
       </c>
-      <c r="B29" s="20"/>
+      <c r="B29" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C29" s="17" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D29" s="16" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="15">
         <v>46114.0</v>
       </c>
-      <c r="B30" s="20"/>
+      <c r="B30" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C30" s="17" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="D30" s="16" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
@@ -1669,33 +1609,35 @@
         <v>46116.0</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>74</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>75</v>
+        <v>70</v>
+      </c>
+      <c r="D31" s="7" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="A32" s="13">
         <v>46119.0</v>
       </c>
-      <c r="C32" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>77</v>
+      <c r="C32" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="A33" s="15">
         <v>46120.0</v>
       </c>
-      <c r="B33" s="20"/>
+      <c r="B33" s="7" t="s">
+        <v>47</v>
+      </c>
       <c r="C33" s="17" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D33" s="16" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
@@ -1703,10 +1645,10 @@
         <v>46127.0</v>
       </c>
       <c r="C34" s="19" t="s">
-        <v>80</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>81</v>
+        <v>76</v>
+      </c>
+      <c r="D34" s="7" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
@@ -1714,13 +1656,13 @@
         <v>46127.0</v>
       </c>
       <c r="C35" s="19" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>84</v>
+        <v>78</v>
+      </c>
+      <c r="D35" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E35" s="7" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
@@ -1728,10 +1670,10 @@
         <v>46128.0</v>
       </c>
       <c r="C36" s="19" t="s">
-        <v>85</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>86</v>
+        <v>81</v>
+      </c>
+      <c r="D36" s="7" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
@@ -1739,13 +1681,13 @@
         <v>46129.0</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>87</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>89</v>
+        <v>83</v>
+      </c>
+      <c r="D37" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E37" s="7" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
@@ -1753,10 +1695,10 @@
         <v>46130.0</v>
       </c>
       <c r="C38" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="D38" s="6" t="s">
         <v>86</v>
+      </c>
+      <c r="D38" s="7" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
@@ -1764,13 +1706,13 @@
         <v>46131.0</v>
       </c>
       <c r="C39" s="19" t="s">
-        <v>91</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>93</v>
+        <v>87</v>
+      </c>
+      <c r="D39" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E39" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
@@ -1778,24 +1720,24 @@
         <v>46131.0</v>
       </c>
       <c r="C40" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
+      </c>
+      <c r="D40" s="7" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="13">
         <v>46132.0</v>
       </c>
-      <c r="C41" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>98</v>
+      <c r="C41" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D41" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E41" s="7" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
@@ -1803,24 +1745,24 @@
         <v>46133.0</v>
       </c>
       <c r="C42" s="19" t="s">
-        <v>99</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>101</v>
+        <v>95</v>
+      </c>
+      <c r="D42" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E42" s="7" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="A43" s="13">
         <v>46133.0</v>
       </c>
-      <c r="C43" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>103</v>
+      <c r="C43" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D43" s="7" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
@@ -1828,56 +1770,56 @@
         <v>46135.0</v>
       </c>
       <c r="C44" s="19" t="s">
-        <v>104</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="H44" s="6"/>
+        <v>100</v>
+      </c>
+      <c r="D44" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="E44" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="H44" s="7"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="A45" s="13">
         <v>46135.0</v>
       </c>
-      <c r="C45" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="E45" s="7" t="s">
-        <v>109</v>
+      <c r="C45" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="A46" s="13">
         <v>46136.0</v>
       </c>
-      <c r="C46" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>112</v>
+      <c r="C46" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E46" s="7" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="A47" s="13">
         <v>46136.0</v>
       </c>
-      <c r="C47" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>115</v>
+      <c r="C47" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D47" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E47" s="7" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
@@ -1885,639 +1827,648 @@
         <v>46136.0</v>
       </c>
       <c r="C48" s="19" t="s">
-        <v>116</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>118</v>
+        <v>112</v>
+      </c>
+      <c r="D48" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="E48" s="7" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="A49" s="13">
         <v>46137.0</v>
       </c>
-      <c r="C49" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>118</v>
+      <c r="C49" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D49" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="A50" s="13">
         <v>46138.0</v>
       </c>
-      <c r="C50" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="D50" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="E50" s="6" t="s">
-        <v>123</v>
+      <c r="C50" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D50" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="E50" s="7" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="A51" s="13">
         <v>46138.0</v>
       </c>
-      <c r="C51" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="D51" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="E51" s="6" t="s">
-        <v>126</v>
+      <c r="C51" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D51" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="E51" s="7" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="A52" s="13">
         <v>46138.0</v>
       </c>
-      <c r="C52" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="E52" s="6"/>
+      <c r="C52" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E52" s="7"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="13">
         <v>46140.0</v>
       </c>
-      <c r="C53" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>131</v>
+      <c r="C53" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D53" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="13">
         <v>46143.0</v>
       </c>
-      <c r="B54" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C54" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="D54" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="E54" s="6" t="s">
-        <v>135</v>
+      <c r="B54" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D54" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E54" s="7" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="A55" s="13">
         <v>46146.0</v>
       </c>
-      <c r="C55" s="7" t="s">
-        <v>136</v>
-      </c>
-      <c r="D55" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="E55" s="6" t="s">
-        <v>138</v>
+      <c r="C55" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D55" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="A56" s="13">
         <v>46147.0</v>
       </c>
-      <c r="C56" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="D56" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="E56" s="6" t="s">
-        <v>141</v>
+      <c r="C56" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D56" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="A57" s="13">
         <v>46148.0</v>
       </c>
-      <c r="C57" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>143</v>
+      <c r="C57" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="A58" s="13">
         <v>46148.0</v>
       </c>
-      <c r="C58" s="7" t="s">
-        <v>144</v>
-      </c>
-      <c r="D58" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>146</v>
+      <c r="C58" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D58" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="E58" s="7" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="A59" s="13">
         <v>46149.0</v>
       </c>
-      <c r="B59" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C59" s="7" t="s">
-        <v>147</v>
-      </c>
-      <c r="D59" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="E59" s="6" t="s">
-        <v>149</v>
+      <c r="B59" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D59" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="E59" s="7" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="A60" s="13">
         <v>46150.0</v>
       </c>
-      <c r="C60" s="7" t="s">
-        <v>150</v>
-      </c>
-      <c r="D60" s="6" t="s">
-        <v>151</v>
+      <c r="C60" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D60" s="7" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="A61" s="13">
         <v>46153.0</v>
       </c>
-      <c r="C61" s="7" t="s">
-        <v>152</v>
-      </c>
-      <c r="D61" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="E61" s="6" t="s">
-        <v>154</v>
+      <c r="C61" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D61" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E61" s="7" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="A62" s="13">
         <v>46153.0</v>
       </c>
-      <c r="C62" s="7" t="s">
-        <v>155</v>
-      </c>
-      <c r="D62" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="E62" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="O62" s="6" t="s">
-        <v>158</v>
+      <c r="C62" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D62" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="O62" s="7" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="A63" s="13">
         <v>46153.0</v>
       </c>
-      <c r="C63" s="7" t="s">
-        <v>159</v>
-      </c>
-      <c r="D63" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="E63" s="6" t="s">
-        <v>161</v>
+      <c r="C63" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="D63" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="E63" s="7" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="A64" s="13">
         <v>46154.0</v>
       </c>
-      <c r="C64" s="22" t="s">
-        <v>162</v>
-      </c>
-      <c r="D64" s="6" t="s">
-        <v>163</v>
+      <c r="C64" s="21" t="s">
+        <v>157</v>
+      </c>
+      <c r="D64" s="7" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="A65" s="13">
         <v>46156.0</v>
       </c>
-      <c r="C65" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E65" s="6" t="s">
-        <v>166</v>
+      <c r="C65" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="E65" s="7" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="A66" s="13">
         <v>46157.0</v>
       </c>
-      <c r="B66" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C66" s="7" t="s">
-        <v>167</v>
-      </c>
-      <c r="D66" s="6" t="s">
-        <v>168</v>
+      <c r="B66" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D66" s="7" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="A67" s="13">
         <v>46160.0</v>
       </c>
-      <c r="C67" s="7" t="s">
-        <v>169</v>
-      </c>
-      <c r="D67" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="E67" s="6" t="s">
-        <v>171</v>
+      <c r="C67" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="A68" s="13">
         <v>46160.0</v>
       </c>
-      <c r="C68" s="7" t="s">
-        <v>172</v>
-      </c>
-      <c r="D68" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="E68" s="6" t="s">
-        <v>174</v>
+      <c r="C68" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="A69" s="13">
         <v>46161.0</v>
       </c>
-      <c r="C69" s="7" t="s">
-        <v>175</v>
-      </c>
-      <c r="D69" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E69" s="6" t="s">
-        <v>177</v>
+      <c r="C69" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D69" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="E69" s="7" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="A70" s="13">
         <v>46163.0</v>
       </c>
-      <c r="B70" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C70" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="D70" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E70" s="6" t="s">
-        <v>180</v>
+      <c r="B70" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="E70" s="7" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="A71" s="13">
         <v>46165.0</v>
       </c>
-      <c r="C71" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D71" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="E71" s="6" t="s">
-        <v>183</v>
+      <c r="C71" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="E71" s="7" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="A72" s="13">
         <v>46165.0</v>
       </c>
-      <c r="C72" s="7" t="s">
-        <v>184</v>
-      </c>
-      <c r="D72" s="23" t="s">
-        <v>185</v>
-      </c>
-      <c r="E72" s="23" t="s">
-        <v>186</v>
-      </c>
-      <c r="F72" s="24"/>
-      <c r="G72" s="24"/>
-      <c r="H72" s="24"/>
-      <c r="I72" s="24"/>
-      <c r="J72" s="24"/>
-      <c r="K72" s="24"/>
-      <c r="L72" s="24"/>
-      <c r="M72" s="24"/>
+      <c r="C72" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D72" s="22" t="s">
+        <v>180</v>
+      </c>
+      <c r="E72" s="22" t="s">
+        <v>181</v>
+      </c>
+      <c r="F72" s="23"/>
+      <c r="G72" s="23"/>
+      <c r="H72" s="23"/>
+      <c r="I72" s="23"/>
+      <c r="J72" s="23"/>
+      <c r="K72" s="23"/>
+      <c r="L72" s="23"/>
+      <c r="M72" s="23"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="A73" s="13">
         <v>46166.0</v>
       </c>
-      <c r="B73" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C73" s="7" t="s">
-        <v>187</v>
-      </c>
-      <c r="D73" s="6" t="s">
-        <v>188</v>
+      <c r="B73" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="A74" s="13">
         <v>46168.0</v>
       </c>
-      <c r="C74" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="D74" s="6" t="s">
-        <v>190</v>
+      <c r="C74" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="A75" s="13">
         <v>46169.0</v>
       </c>
-      <c r="C75" s="7" t="s">
-        <v>191</v>
-      </c>
-      <c r="D75" s="6" t="s">
-        <v>192</v>
+      <c r="C75" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D75" s="7" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="A76" s="13">
         <v>46170.0</v>
       </c>
-      <c r="C76" s="22" t="s">
-        <v>193</v>
-      </c>
-      <c r="D76" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="E76" s="6" t="s">
-        <v>195</v>
+      <c r="C76" s="21" t="s">
+        <v>188</v>
+      </c>
+      <c r="D76" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="E76" s="7" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="A77" s="13">
         <v>46170.0</v>
       </c>
-      <c r="C77" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D77" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="E77" s="6" t="s">
-        <v>198</v>
+      <c r="C77" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D77" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="E77" s="7" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="A78" s="13">
         <v>46172.0</v>
       </c>
-      <c r="B78" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="C78" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="D78" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="E78" s="6" t="s">
-        <v>201</v>
+      <c r="B78" s="7" t="s">
+        <v>194</v>
+      </c>
+      <c r="C78" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D78" s="7" t="s">
+        <v>196</v>
+      </c>
+      <c r="E78" s="7" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="A79" s="13">
         <v>46176.0</v>
       </c>
-      <c r="C79" s="7" t="s">
-        <v>202</v>
-      </c>
-      <c r="D79" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="E79" s="6" t="s">
-        <v>204</v>
+      <c r="C79" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D79" s="7" t="s">
+        <v>199</v>
+      </c>
+      <c r="E79" s="7" t="s">
+        <v>200</v>
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="13">
         <v>46177.0</v>
       </c>
-      <c r="C80" s="7" t="s">
-        <v>205</v>
-      </c>
-      <c r="D80" s="6" t="s">
-        <v>206</v>
+      <c r="C80" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="13">
         <v>46177.0</v>
       </c>
-      <c r="C81" s="7" t="s">
-        <v>207</v>
-      </c>
-      <c r="D81" s="6" t="s">
-        <v>208</v>
+      <c r="C81" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D81" s="7" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="A82" s="13">
         <v>46177.0</v>
       </c>
-      <c r="C82" s="7" t="s">
-        <v>209</v>
-      </c>
-      <c r="D82" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E82" s="6" t="s">
-        <v>211</v>
+      <c r="C82" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D82" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="E82" s="7" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="A83" s="13">
         <v>46178.0</v>
       </c>
-      <c r="C83" s="7" t="s">
-        <v>212</v>
+      <c r="C83" s="6" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="A84" s="13">
         <v>46178.0</v>
       </c>
-      <c r="C84" s="7" t="s">
-        <v>213</v>
+      <c r="C84" s="6" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="A85" s="13">
         <v>46179.0</v>
       </c>
-      <c r="C85" s="7" t="s">
-        <v>214</v>
+      <c r="C85" s="6" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="A86" s="13">
         <v>46179.0</v>
       </c>
-      <c r="C86" s="22" t="s">
-        <v>215</v>
+      <c r="C86" s="21" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="A87" s="13">
         <v>46179.0</v>
       </c>
-      <c r="C87" s="7" t="s">
-        <v>216</v>
+      <c r="C87" s="6" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="A88" s="13">
         <v>46180.0</v>
       </c>
-      <c r="C88" s="7" t="s">
-        <v>217</v>
-      </c>
-      <c r="D88" s="6" t="s">
-        <v>168</v>
+      <c r="B88" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="D88" s="7" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="A89" s="13">
         <v>46182.0</v>
       </c>
-      <c r="C89" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="D89" s="6" t="s">
-        <v>55</v>
+      <c r="C89" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="D89" s="7" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="A90" s="13">
         <v>46186.0</v>
       </c>
-      <c r="C90" s="7" t="s">
-        <v>219</v>
-      </c>
-      <c r="D90" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="E90" s="7" t="s">
-        <v>220</v>
+      <c r="B90" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C90" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="D90" s="7" t="s">
+        <v>163</v>
+      </c>
+      <c r="E90" s="6" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="A91" s="13">
         <v>46189.0</v>
       </c>
-      <c r="C91" s="7" t="s">
-        <v>221</v>
+      <c r="C91" s="6" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="A92" s="13">
         <v>46190.0</v>
       </c>
-      <c r="C92" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="E92" s="7" t="s">
-        <v>223</v>
+      <c r="C92" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="E92" s="6" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="A93" s="13">
         <v>46191.0</v>
       </c>
-      <c r="C93" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="D93" s="6" t="s">
-        <v>206</v>
+      <c r="C93" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="D93" s="7" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="A94" s="13">
         <v>46191.0</v>
       </c>
-      <c r="C94" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="D94" s="6" t="s">
-        <v>226</v>
+      <c r="C94" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="D94" s="7" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="A95" s="13">
         <v>46193.0</v>
       </c>
-      <c r="C95" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="D95" s="6" t="s">
-        <v>188</v>
+      <c r="B95" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C95" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="D95" s="7" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="13">
         <v>46195.0</v>
       </c>
-      <c r="C96" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="D96" s="6" t="s">
-        <v>55</v>
+      <c r="C96" s="6" t="s">
+        <v>224</v>
+      </c>
+      <c r="D96" s="7" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="A97" s="13">
         <v>46196.0</v>
       </c>
-      <c r="C97" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="D97" s="6" t="s">
-        <v>55</v>
+      <c r="C97" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D97" s="7" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
update entrenamientos hasta 24-06
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="226">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="230">
   <si>
     <t>date</t>
   </si>
@@ -795,10 +795,22 @@
     <t>https://youtu.be/ET6NrbvaJ2A</t>
   </si>
   <si>
+    <t>https://youtu.be/pr01ompIZzg</t>
+  </si>
+  <si>
     <t>https://youtu.be/xtyqkXcTy9s</t>
   </si>
   <si>
     <t>https://youtu.be/MEpLI9f7JJQ</t>
+  </si>
+  <si>
+    <t>https://youtu.be/wVx7ihMAHEQ</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-7i4ngwX5mU</t>
+  </si>
+  <si>
+    <t>Salidas (equipos naranja)</t>
   </si>
 </sst>
 </file>
@@ -2448,13 +2460,16 @@
       <c r="D95" s="7" t="s">
         <v>183</v>
       </c>
+      <c r="E95" s="6" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="A96" s="13">
         <v>46195.0</v>
       </c>
       <c r="C96" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D96" s="7" t="s">
         <v>51</v>
@@ -2465,14 +2480,34 @@
         <v>46196.0</v>
       </c>
       <c r="C97" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D97" s="7" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="98" ht="15.75" customHeight="1"/>
-    <row r="99" ht="15.75" customHeight="1"/>
+    <row r="98" ht="15.75" customHeight="1">
+      <c r="A98" s="13">
+        <v>46197.0</v>
+      </c>
+      <c r="C98" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="D98" s="7" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="99" ht="15.75" customHeight="1">
+      <c r="A99" s="13">
+        <v>46197.0</v>
+      </c>
+      <c r="C99" s="6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D99" s="7" t="s">
+        <v>229</v>
+      </c>
+    </row>
     <row r="100" ht="15.75" customHeight="1"/>
     <row r="101" ht="15.75" customHeight="1"/>
     <row r="102" ht="15.75" customHeight="1"/>
@@ -3483,12 +3518,15 @@
     <hyperlink r:id="rId99" ref="C93"/>
     <hyperlink r:id="rId100" ref="C94"/>
     <hyperlink r:id="rId101" ref="C95"/>
-    <hyperlink r:id="rId102" ref="C96"/>
-    <hyperlink r:id="rId103" ref="C97"/>
+    <hyperlink r:id="rId102" ref="E95"/>
+    <hyperlink r:id="rId103" ref="C96"/>
+    <hyperlink r:id="rId104" ref="C97"/>
+    <hyperlink r:id="rId105" ref="C98"/>
+    <hyperlink r:id="rId106" ref="C99"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId104"/>
+  <drawing r:id="rId107"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 2706
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="235">
   <si>
     <t>date</t>
   </si>
@@ -811,6 +811,21 @@
   </si>
   <si>
     <t>Salidas (equipos naranja)</t>
+  </si>
+  <si>
+    <t>https://youtu.be/uvTEFA2dgB0</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ryhZ_ktddfU</t>
+  </si>
+  <si>
+    <t>https://youtu.be/RMRVl8DJv8w</t>
+  </si>
+  <si>
+    <t>Salidas: en vacío y con oposición</t>
+  </si>
+  <si>
+    <t>https://youtu.be/5oNuwiJkerU</t>
   </si>
 </sst>
 </file>
@@ -2508,10 +2523,47 @@
         <v>229</v>
       </c>
     </row>
-    <row r="100" ht="15.75" customHeight="1"/>
-    <row r="101" ht="15.75" customHeight="1"/>
-    <row r="102" ht="15.75" customHeight="1"/>
-    <row r="103" ht="15.75" customHeight="1"/>
+    <row r="100" ht="15.75" customHeight="1">
+      <c r="A100" s="13">
+        <v>46199.0</v>
+      </c>
+      <c r="C100" s="6" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="101" ht="15.75" customHeight="1">
+      <c r="A101" s="13">
+        <v>46199.0</v>
+      </c>
+      <c r="C101" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="D101" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="102" ht="15.75" customHeight="1">
+      <c r="A102" s="13">
+        <v>46200.0</v>
+      </c>
+      <c r="C102" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="D102" s="7" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="103" ht="15.75" customHeight="1">
+      <c r="A103" s="13">
+        <v>46200.0</v>
+      </c>
+      <c r="C103" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="D103" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
     <row r="104" ht="15.75" customHeight="1"/>
     <row r="105" ht="15.75" customHeight="1"/>
     <row r="106" ht="15.75" customHeight="1"/>
@@ -3523,10 +3575,14 @@
     <hyperlink r:id="rId104" ref="C97"/>
     <hyperlink r:id="rId105" ref="C98"/>
     <hyperlink r:id="rId106" ref="C99"/>
+    <hyperlink r:id="rId107" ref="C100"/>
+    <hyperlink r:id="rId108" ref="C101"/>
+    <hyperlink r:id="rId109" ref="C102"/>
+    <hyperlink r:id="rId110" ref="C103"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId107"/>
+  <drawing r:id="rId111"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 3006
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="237">
   <si>
     <t>date</t>
   </si>
@@ -826,6 +826,12 @@
   </si>
   <si>
     <t>https://youtu.be/5oNuwiJkerU</t>
+  </si>
+  <si>
+    <t>https://youtu.be/3slreko_RwE</t>
+  </si>
+  <si>
+    <t>https://youtu.be/G7ILRQ29sAA</t>
   </si>
 </sst>
 </file>
@@ -2564,8 +2570,28 @@
         <v>222</v>
       </c>
     </row>
-    <row r="104" ht="15.75" customHeight="1"/>
-    <row r="105" ht="15.75" customHeight="1"/>
+    <row r="104" ht="15.75" customHeight="1">
+      <c r="A104" s="13">
+        <v>46202.0</v>
+      </c>
+      <c r="C104" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="105" ht="15.75" customHeight="1">
+      <c r="A105" s="13">
+        <v>46203.0</v>
+      </c>
+      <c r="C105" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="D105" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
     <row r="106" ht="15.75" customHeight="1"/>
     <row r="107" ht="15.75" customHeight="1"/>
     <row r="108" ht="15.75" customHeight="1"/>
@@ -3579,10 +3605,12 @@
     <hyperlink r:id="rId108" ref="C101"/>
     <hyperlink r:id="rId109" ref="C102"/>
     <hyperlink r:id="rId110" ref="C103"/>
+    <hyperlink r:id="rId111" ref="C104"/>
+    <hyperlink r:id="rId112" ref="C105"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId111"/>
+  <drawing r:id="rId113"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 020726
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="240">
   <si>
     <t>date</t>
   </si>
@@ -832,6 +832,15 @@
   </si>
   <si>
     <t>https://youtu.be/G7ILRQ29sAA</t>
+  </si>
+  <si>
+    <t>https://youtu.be/dKTc3r2fY8A</t>
+  </si>
+  <si>
+    <t>https://youtu.be/WTb_OvISiRU</t>
+  </si>
+  <si>
+    <t>Amistoso vs Amigos de la PNP</t>
   </si>
 </sst>
 </file>
@@ -2592,8 +2601,31 @@
         <v>51</v>
       </c>
     </row>
-    <row r="106" ht="15.75" customHeight="1"/>
-    <row r="107" ht="15.75" customHeight="1"/>
+    <row r="106" ht="15.75" customHeight="1">
+      <c r="A106" s="13">
+        <v>46204.0</v>
+      </c>
+      <c r="C106" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="D106" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="107" ht="15.75" customHeight="1">
+      <c r="A107" s="13">
+        <v>46205.0</v>
+      </c>
+      <c r="B107" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="D107" s="7" t="s">
+        <v>239</v>
+      </c>
+    </row>
     <row r="108" ht="15.75" customHeight="1"/>
     <row r="109" ht="15.75" customHeight="1"/>
     <row r="110" ht="15.75" customHeight="1"/>
@@ -3607,10 +3639,12 @@
     <hyperlink r:id="rId110" ref="C103"/>
     <hyperlink r:id="rId111" ref="C104"/>
     <hyperlink r:id="rId112" ref="C105"/>
+    <hyperlink r:id="rId113" ref="C106"/>
+    <hyperlink r:id="rId114" ref="C107"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId113"/>
+  <drawing r:id="rId115"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
update entrenamientos hasta 100726 .2
</commit_message>
<xml_diff>
--- a/entrenamientos.xlsx
+++ b/entrenamientos.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="256">
   <si>
     <t>date</t>
   </si>
@@ -841,6 +841,54 @@
   </si>
   <si>
     <t>Amistoso vs Amigos de la PNP</t>
+  </si>
+  <si>
+    <t>https://youtu.be/c4JgpWgxgs0</t>
+  </si>
+  <si>
+    <t>Salidas</t>
+  </si>
+  <si>
+    <t>https://youtu.be/u9WfF7l2dq0</t>
+  </si>
+  <si>
+    <t>https://youtu.be/rN0zMezQxf8</t>
+  </si>
+  <si>
+    <t>Primerz parte</t>
+  </si>
+  <si>
+    <t>https://youtu.be/O0CEEEccC80</t>
+  </si>
+  <si>
+    <t>Defensa alta, 3/4 y bloque bajo</t>
+  </si>
+  <si>
+    <t>https://youtu.be/7Gimgf3MqYE</t>
+  </si>
+  <si>
+    <t>Centros y duelos</t>
+  </si>
+  <si>
+    <t>https://youtu.be/MtpDzA0Z7bU</t>
+  </si>
+  <si>
+    <t>Salidas 08-07</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Lo3XIfbHLkU</t>
+  </si>
+  <si>
+    <t>Duelos 3 vs 2</t>
+  </si>
+  <si>
+    <t>https://youtu.be/-h2rmy01K_U</t>
+  </si>
+  <si>
+    <t>https://youtu.be/cTH6XILoMXY</t>
+  </si>
+  <si>
+    <t>Amistoso interno</t>
   </si>
 </sst>
 </file>
@@ -2626,15 +2674,105 @@
         <v>239</v>
       </c>
     </row>
-    <row r="108" ht="15.75" customHeight="1"/>
-    <row r="109" ht="15.75" customHeight="1"/>
-    <row r="110" ht="15.75" customHeight="1"/>
-    <row r="111" ht="15.75" customHeight="1"/>
-    <row r="112" ht="15.75" customHeight="1"/>
-    <row r="113" ht="15.75" customHeight="1"/>
-    <row r="114" ht="15.75" customHeight="1"/>
-    <row r="115" ht="15.75" customHeight="1"/>
-    <row r="116" ht="15.75" customHeight="1"/>
+    <row r="108" ht="15.75" customHeight="1">
+      <c r="A108" s="13">
+        <v>46206.0</v>
+      </c>
+      <c r="C108" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="D108" s="7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="109" ht="15.75" customHeight="1">
+      <c r="A109" s="13">
+        <v>46209.0</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="110" ht="15.75" customHeight="1">
+      <c r="A110" s="13">
+        <v>46210.0</v>
+      </c>
+      <c r="C110" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="D110" s="7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="111" ht="15.75" customHeight="1">
+      <c r="A111" s="13">
+        <v>46210.0</v>
+      </c>
+      <c r="C111" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="D111" s="7" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="112" ht="15.75" customHeight="1">
+      <c r="A112" s="13">
+        <v>46211.0</v>
+      </c>
+      <c r="C112" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="D112" s="7" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="113" ht="15.75" customHeight="1">
+      <c r="A113" s="13">
+        <v>46211.0</v>
+      </c>
+      <c r="C113" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="D113" s="7" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="114" ht="15.75" customHeight="1">
+      <c r="A114" s="13">
+        <v>46212.0</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="D114" s="7" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="115" ht="15.75" customHeight="1">
+      <c r="A115" s="13">
+        <v>46212.0</v>
+      </c>
+      <c r="C115" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="D115" s="7" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="116" ht="15.75" customHeight="1">
+      <c r="A116" s="13">
+        <v>46213.0</v>
+      </c>
+      <c r="C116" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="D116" s="7" t="s">
+        <v>255</v>
+      </c>
+    </row>
     <row r="117" ht="15.75" customHeight="1"/>
     <row r="118" ht="15.75" customHeight="1"/>
     <row r="119" ht="15.75" customHeight="1"/>
@@ -3641,10 +3779,19 @@
     <hyperlink r:id="rId112" ref="C105"/>
     <hyperlink r:id="rId113" ref="C106"/>
     <hyperlink r:id="rId114" ref="C107"/>
+    <hyperlink r:id="rId115" ref="C108"/>
+    <hyperlink r:id="rId116" ref="C109"/>
+    <hyperlink r:id="rId117" ref="C110"/>
+    <hyperlink r:id="rId118" ref="C111"/>
+    <hyperlink r:id="rId119" ref="C112"/>
+    <hyperlink r:id="rId120" ref="C113"/>
+    <hyperlink r:id="rId121" ref="C114"/>
+    <hyperlink r:id="rId122" ref="C115"/>
+    <hyperlink r:id="rId123" ref="C116"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId115"/>
+  <drawing r:id="rId124"/>
 </worksheet>
 </file>
</xml_diff>